<commit_message>
DC investor deck: workbook regenerated for racks-soon and server enclosures; slide 4 beam and slide 5 notes
The campus model (analyses/build_model.py, gen_md.py) now carries the
2026-09-04 horizons: racking stays in Soon with a development note, and a
new input puts 40% of IT mass (server and equipment enclosures) in the Long
term, electronics excluded. Workbook, narrative and chart regenerated; the
scripts read their row metadata from a local model_rows.json. Slide 6 rounds
to the workbook (58-362 kt, 1.8-12 years). Slide 4's SUPERWOOD-only beam
is now an image-to-image edit of the hybrid render, same camera and color,
boards stacked flat. Slide 5 notes enlarged on both the web and the PPTX.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1439,14 +1439,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
+          <t>Share of IT mass that is server and equipment enclosures (boxes), replaceable long term</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1455,26 +1455,26 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>estimated [L]; Alex 2026-09-04</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Remainder is slab on grade, paving and yard</t>
+          <t>Server boxes eventually; the electronics never</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
+          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1483,26 +1483,26 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan; no design or code pathway yet</t>
+          <t>Remainder is slab on grade, paving and yard</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
+          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1516,53 +1516,53 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan</t>
+          <t>Technical potential, not a plan; no design or code pathway yet</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>kg SUPERWOOD per kg of concrete replaced</t>
+          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>0.05</v>
+        <v>0.9</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.15</v>
+        <v>0.9</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
+          <t>Technical potential, not a plan</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ducting, plenums and air-distribution sheet metal</t>
+          <t>kg SUPERWOOD per kg of concrete replaced</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>3</v>
+        <v>0.05</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>8</v>
+        <v>0.15</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>t/MW</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1572,82 +1572,86 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Separate from the mechanical-equipment row</t>
+          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Concrete emissions</t>
+          <t>Ducting, plenums and air-distribution sheet metal</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>0.12</v>
+        <v>3</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.12</v>
+        <v>8</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>t/MW</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
+          <t>Separate from the mechanical-equipment row</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SUPERWOOD average board thickness</t>
+          <t>Concrete emissions</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>7.2</v>
+        <v>0.12</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>7.2</v>
+        <v>0.12</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>internal TEM basis [H]</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SUPERWOOD density</t>
+          <t>SUPERWOOD average board thickness</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>1300</v>
+        <v>7.2</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1300</v>
+        <v>7.2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>kg/m³</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>internal TEM [H]</t>
+          <t>internal TEM basis [H]</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -1655,23 +1659,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SuperMill One output</t>
+          <t>SUPERWOOD density</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>1000000</v>
+        <v>1300</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1000000</v>
+        <v>1300</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>sf/yr</t>
+          <t>kg/m³</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>internal [H]</t>
+          <t>internal TEM [H]</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -1679,14 +1683,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SuperMill Two output</t>
+          <t>SuperMill One output</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>36000000</v>
+        <v>1000000</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>36000000</v>
+        <v>1000000</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1703,46 +1707,42 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
+          <t>SuperMill Two output</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>0.3</v>
+        <v>36000000</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.6</v>
+        <v>36000000</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>sf/yr</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
-        </is>
-      </c>
+          <t>internal [H]</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
+          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>20</v>
+        <v>0.3</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>40</v>
+        <v>0.6</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>kg/m²</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1752,25 +1752,25 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Panel design unsettled</t>
+          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Addressable share of other tray / containment / doors (medium term)</t>
+          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>0.5</v>
+        <v>20</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0.5</v>
+        <v>40</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>kg/m²</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1778,71 +1778,75 @@
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Panel design unsettled</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Count rebar as addressable in the long term? (0/1)</t>
+          <t>Addressable share of other tray / containment / doors (medium term)</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Rebar is a frontier market with no pathway; off by default</t>
-        </is>
-      </c>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Steel emissions, global average (BF-BOF)</t>
+          <t>Count rebar as addressable in the long term? (0/1)</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>published-class [M]</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Rebar is a frontier market with no pathway; off by default</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Steel emissions, recycled (EAF)</t>
+          <t>Steel emissions, global average (BF-BOF)</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0.7</v>
+        <v>1.8</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1851,7 +1855,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
+          <t>published-class [M]</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -1859,14 +1863,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SUPERWOOD manufacturing emissions</t>
+          <t>Steel emissions, recycled (EAF)</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1875,38 +1879,62 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
-        </is>
-      </c>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>SUPERWOOD manufacturing emissions</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>internal, pre-LCA [L]</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>SUPERWOOD biogenic carbon stored</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n">
+      <c r="B47" s="2" t="n">
         <v>1.3</v>
       </c>
-      <c r="C46" s="2" t="n">
+      <c r="C47" s="2" t="n">
         <v>1.3</v>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>kg CO₂e/kg</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>internal, pre-LCA [L]</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Report separately; module C release under EN 15804</t>
         </is>
@@ -2099,20 +2127,20 @@
         </is>
       </c>
       <c r="B3" s="5">
-        <f>Inputs!$B$11*(1-Inputs!$B$29)*Inputs!$B$12*Inputs!$B$2-B5</f>
-        <v>720000.0</v>
+        <f>Inputs!$B$11*(1-Inputs!$B$30)*Inputs!$B$12*Inputs!$B$2-B5</f>
+        <v/>
       </c>
       <c r="C3" s="5">
-        <f>Inputs!$C$11*(1-Inputs!$C$29)*Inputs!$C$12*Inputs!$C$2-C5</f>
-        <v>1200000.0</v>
+        <f>Inputs!$C$11*(1-Inputs!$C$30)*Inputs!$C$12*Inputs!$C$2-C5</f>
+        <v/>
       </c>
       <c r="D3" s="5">
         <f>B3</f>
-        <v>720000.0</v>
+        <v/>
       </c>
       <c r="E3" s="5">
         <f>C3</f>
-        <v>1200000.0</v>
+        <v/>
       </c>
       <c r="F3" s="6" t="n">
         <v>0</v>
@@ -2124,24 +2152,24 @@
         <v>0</v>
       </c>
       <c r="I3" s="6">
-        <f>Inputs!$B$30</f>
-        <v>0.75</v>
+        <f>Inputs!$B$31</f>
+        <v/>
       </c>
       <c r="J3" s="5">
         <f>B3*SUM($F3:$I3)</f>
-        <v>540000.0</v>
+        <v/>
       </c>
       <c r="K3" s="5">
         <f>C3*SUM($F3:$I3)</f>
-        <v>900000.0</v>
+        <v/>
       </c>
       <c r="L3" s="5">
-        <f>J3*Inputs!$B$32</f>
-        <v>27000.0</v>
+        <f>J3*Inputs!$B$33</f>
+        <v/>
       </c>
       <c r="M3" s="5">
-        <f>K3*Inputs!$C$32</f>
-        <v>135000.0</v>
+        <f>K3*Inputs!$C$33</f>
+        <v/>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -2150,39 +2178,39 @@
       </c>
       <c r="O3" s="5">
         <f>C3-K3</f>
-        <v>300000.0</v>
+        <v/>
       </c>
       <c r="P3" s="5">
         <f>IF(SUM($F3:$I3)=0,0,L3*F3/SUM($F3:$I3))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q3" s="5">
         <f>IF(SUM($F3:$I3)=0,0,L3*G3/SUM($F3:$I3))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R3" s="5">
         <f>IF(SUM($F3:$I3)=0,0,L3*H3/SUM($F3:$I3))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S3" s="5">
         <f>IF(SUM($F3:$I3)=0,0,L3*I3/SUM($F3:$I3))</f>
-        <v>27000.0</v>
+        <v/>
       </c>
       <c r="T3" s="5">
         <f>IF(SUM($F3:$I3)=0,0,M3*F3/SUM($F3:$I3))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U3" s="5">
         <f>IF(SUM($F3:$I3)=0,0,M3*G3/SUM($F3:$I3))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V3" s="5">
         <f>IF(SUM($F3:$I3)=0,0,M3*H3/SUM($F3:$I3))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W3" s="5">
         <f>IF(SUM($F3:$I3)=0,0,M3*I3/SUM($F3:$I3))</f>
-        <v>135000.0</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -2192,20 +2220,20 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>Inputs!$B$11*Inputs!$B$29*Inputs!$B$12*Inputs!$B$2</f>
-        <v>480000.0</v>
+        <f>Inputs!$B$11*Inputs!$B$30*Inputs!$B$12*Inputs!$B$2</f>
+        <v/>
       </c>
       <c r="C4" s="5">
-        <f>Inputs!$C$11*Inputs!$C$29*Inputs!$C$12*Inputs!$C$2</f>
-        <v>1200000.0</v>
+        <f>Inputs!$C$11*Inputs!$C$30*Inputs!$C$12*Inputs!$C$2</f>
+        <v/>
       </c>
       <c r="D4" s="5">
         <f>D3+B4</f>
-        <v>1200000.0</v>
+        <v/>
       </c>
       <c r="E4" s="5">
         <f>E3+C4</f>
-        <v>2400000.0</v>
+        <v/>
       </c>
       <c r="F4" s="6" t="n">
         <v>0</v>
@@ -2217,24 +2245,24 @@
         <v>0</v>
       </c>
       <c r="I4" s="6">
-        <f>Inputs!$B$31</f>
-        <v>0.9</v>
+        <f>Inputs!$B$32</f>
+        <v/>
       </c>
       <c r="J4" s="5">
         <f>B4*SUM($F4:$I4)</f>
-        <v>432000.0</v>
+        <v/>
       </c>
       <c r="K4" s="5">
         <f>C4*SUM($F4:$I4)</f>
-        <v>1080000.0</v>
+        <v/>
       </c>
       <c r="L4" s="5">
-        <f>J4*Inputs!$B$32</f>
-        <v>21600.0</v>
+        <f>J4*Inputs!$B$33</f>
+        <v/>
       </c>
       <c r="M4" s="5">
-        <f>K4*Inputs!$C$32</f>
-        <v>162000.0</v>
+        <f>K4*Inputs!$C$33</f>
+        <v/>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -2243,39 +2271,39 @@
       </c>
       <c r="O4" s="5">
         <f>C4-K4</f>
-        <v>120000.0</v>
+        <v/>
       </c>
       <c r="P4" s="5">
         <f>IF(SUM($F4:$I4)=0,0,L4*F4/SUM($F4:$I4))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q4" s="5">
         <f>IF(SUM($F4:$I4)=0,0,L4*G4/SUM($F4:$I4))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R4" s="5">
         <f>IF(SUM($F4:$I4)=0,0,L4*H4/SUM($F4:$I4))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S4" s="5">
         <f>IF(SUM($F4:$I4)=0,0,L4*I4/SUM($F4:$I4))</f>
-        <v>21600.0</v>
+        <v/>
       </c>
       <c r="T4" s="5">
         <f>IF(SUM($F4:$I4)=0,0,M4*F4/SUM($F4:$I4))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U4" s="5">
         <f>IF(SUM($F4:$I4)=0,0,M4*G4/SUM($F4:$I4))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V4" s="5">
         <f>IF(SUM($F4:$I4)=0,0,M4*H4/SUM($F4:$I4))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W4" s="5">
         <f>IF(SUM($F4:$I4)=0,0,M4*I4/SUM($F4:$I4))</f>
-        <v>162000.0</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -2286,19 +2314,19 @@
       </c>
       <c r="B5" s="5">
         <f>Inputs!$B$13*Derived!B4*Inputs!$B$14*Inputs!$B$12</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="C5" s="5">
         <f>Inputs!$C$13*Derived!C4*Inputs!$C$14*Inputs!$C$12</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="D5" s="5">
         <f>D4+B5</f>
-        <v>1200000.0</v>
+        <v/>
       </c>
       <c r="E5" s="5">
         <f>E4+C5</f>
-        <v>2400000.0</v>
+        <v/>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -2314,19 +2342,19 @@
       </c>
       <c r="J5" s="5">
         <f>B5*SUM($F5:$I5)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="K5" s="5">
         <f>C5*SUM($F5:$I5)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="L5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$40/1000</f>
-        <v>0.0</v>
+        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$41/1000</f>
+        <v/>
       </c>
       <c r="M5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$40/1000</f>
-        <v>0.0</v>
+        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$41/1000</f>
+        <v/>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -2335,39 +2363,39 @@
       </c>
       <c r="O5" s="5">
         <f>C5-K5</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P5" s="5">
         <f>IF(SUM($F5:$I5)=0,0,L5*F5/SUM($F5:$I5))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q5" s="5">
         <f>IF(SUM($F5:$I5)=0,0,L5*G5/SUM($F5:$I5))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R5" s="5">
         <f>IF(SUM($F5:$I5)=0,0,L5*H5/SUM($F5:$I5))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S5" s="5">
         <f>IF(SUM($F5:$I5)=0,0,L5*I5/SUM($F5:$I5))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T5" s="5">
         <f>IF(SUM($F5:$I5)=0,0,M5*F5/SUM($F5:$I5))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U5" s="5">
         <f>IF(SUM($F5:$I5)=0,0,M5*G5/SUM($F5:$I5))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V5" s="5">
         <f>IF(SUM($F5:$I5)=0,0,M5*H5/SUM($F5:$I5))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W5" s="5">
         <f>IF(SUM($F5:$I5)=0,0,M5*I5/SUM($F5:$I5))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -2378,19 +2406,19 @@
       </c>
       <c r="B6" s="5">
         <f>Inputs!$B$11*Inputs!$B$17/1000*Inputs!$B$2</f>
-        <v>30000.0</v>
+        <v/>
       </c>
       <c r="C6" s="5">
         <f>Inputs!$C$11*Inputs!$C$17/1000*Inputs!$C$2</f>
-        <v>100000.0</v>
+        <v/>
       </c>
       <c r="D6" s="5">
         <f>D5+B6</f>
-        <v>1230000.0</v>
+        <v/>
       </c>
       <c r="E6" s="5">
         <f>E5+C6</f>
-        <v>2500000.0</v>
+        <v/>
       </c>
       <c r="F6" s="6" t="n">
         <v>0</v>
@@ -2402,24 +2430,24 @@
         <v>0</v>
       </c>
       <c r="I6" s="6">
-        <f>Inputs!$B$29*Inputs!$B$31+(1-Inputs!$B$29)*Inputs!$B$30</f>
-        <v>0.81</v>
+        <f>Inputs!$B$30*Inputs!$B$32+(1-Inputs!$B$30)*Inputs!$B$31</f>
+        <v/>
       </c>
       <c r="J6" s="5">
         <f>B6*SUM($F6:$I6)</f>
-        <v>24300.0</v>
+        <v/>
       </c>
       <c r="K6" s="5">
         <f>C6*SUM($F6:$I6)</f>
-        <v>81000.0</v>
+        <v/>
       </c>
       <c r="L6" s="5">
-        <f>J6*Inputs!$B$39</f>
-        <v>7290.0</v>
+        <f>J6*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M6" s="5">
-        <f>K6*Inputs!$C$39</f>
-        <v>48600.0</v>
+        <f>K6*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -2428,39 +2456,39 @@
       </c>
       <c r="O6" s="5">
         <f>C6-K6</f>
-        <v>19000.0</v>
+        <v/>
       </c>
       <c r="P6" s="5">
         <f>IF(SUM($F6:$I6)=0,0,L6*F6/SUM($F6:$I6))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q6" s="5">
         <f>IF(SUM($F6:$I6)=0,0,L6*G6/SUM($F6:$I6))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R6" s="5">
         <f>IF(SUM($F6:$I6)=0,0,L6*H6/SUM($F6:$I6))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S6" s="5">
         <f>IF(SUM($F6:$I6)=0,0,L6*I6/SUM($F6:$I6))</f>
-        <v>7290.0</v>
+        <v/>
       </c>
       <c r="T6" s="5">
         <f>IF(SUM($F6:$I6)=0,0,M6*F6/SUM($F6:$I6))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U6" s="5">
         <f>IF(SUM($F6:$I6)=0,0,M6*G6/SUM($F6:$I6))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V6" s="5">
         <f>IF(SUM($F6:$I6)=0,0,M6*H6/SUM($F6:$I6))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W6" s="5">
         <f>IF(SUM($F6:$I6)=0,0,M6*I6/SUM($F6:$I6))</f>
-        <v>48600.0</v>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -2471,19 +2499,19 @@
       </c>
       <c r="B7" s="5">
         <f>Inputs!$B$15*(1-Inputs!$B$16)*Inputs!$B$2</f>
-        <v>30000.0</v>
+        <v/>
       </c>
       <c r="C7" s="5">
         <f>Inputs!$C$15*(1-Inputs!$C$16)*Inputs!$C$2</f>
-        <v>40000.0</v>
+        <v/>
       </c>
       <c r="D7" s="5">
         <f>D6+B7</f>
-        <v>1260000.0</v>
+        <v/>
       </c>
       <c r="E7" s="5">
         <f>E6+C7</f>
-        <v>2540000.0</v>
+        <v/>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -2499,19 +2527,19 @@
       </c>
       <c r="J7" s="5">
         <f>B7*SUM($F7:$I7)</f>
-        <v>30000.0</v>
+        <v/>
       </c>
       <c r="K7" s="5">
         <f>C7*SUM($F7:$I7)</f>
-        <v>40000.0</v>
+        <v/>
       </c>
       <c r="L7" s="5">
-        <f>J7*Inputs!$B$39</f>
-        <v>9000.0</v>
+        <f>J7*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M7" s="5">
-        <f>K7*Inputs!$C$39</f>
-        <v>24000.0</v>
+        <f>K7*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -2520,39 +2548,39 @@
       </c>
       <c r="O7" s="5">
         <f>C7-K7</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P7" s="5">
         <f>IF(SUM($F7:$I7)=0,0,L7*F7/SUM($F7:$I7))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q7" s="5">
         <f>IF(SUM($F7:$I7)=0,0,L7*G7/SUM($F7:$I7))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R7" s="5">
         <f>IF(SUM($F7:$I7)=0,0,L7*H7/SUM($F7:$I7))</f>
-        <v>9000.0</v>
+        <v/>
       </c>
       <c r="S7" s="5">
         <f>IF(SUM($F7:$I7)=0,0,L7*I7/SUM($F7:$I7))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T7" s="5">
         <f>IF(SUM($F7:$I7)=0,0,M7*F7/SUM($F7:$I7))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U7" s="5">
         <f>IF(SUM($F7:$I7)=0,0,M7*G7/SUM($F7:$I7))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V7" s="5">
         <f>IF(SUM($F7:$I7)=0,0,M7*H7/SUM($F7:$I7))</f>
-        <v>24000.0</v>
+        <v/>
       </c>
       <c r="W7" s="5">
         <f>IF(SUM($F7:$I7)=0,0,M7*I7/SUM($F7:$I7))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -2563,19 +2591,19 @@
       </c>
       <c r="B8" s="5">
         <f>Inputs!$B$15*Inputs!$B$16*Inputs!$B$2</f>
-        <v>20000.0</v>
+        <v/>
       </c>
       <c r="C8" s="5">
         <f>Inputs!$C$15*Inputs!$C$16*Inputs!$C$2</f>
-        <v>60000.0</v>
+        <v/>
       </c>
       <c r="D8" s="5">
         <f>D7+B8</f>
-        <v>1280000.0</v>
+        <v/>
       </c>
       <c r="E8" s="5">
         <f>E7+C8</f>
-        <v>2600000.0</v>
+        <v/>
       </c>
       <c r="F8" s="6" t="n">
         <v>0</v>
@@ -2591,19 +2619,19 @@
       </c>
       <c r="J8" s="5">
         <f>B8*SUM($F8:$I8)</f>
-        <v>20000.0</v>
+        <v/>
       </c>
       <c r="K8" s="5">
         <f>C8*SUM($F8:$I8)</f>
-        <v>60000.0</v>
+        <v/>
       </c>
       <c r="L8" s="5">
-        <f>J8*Inputs!$B$39</f>
-        <v>6000.0</v>
+        <f>J8*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M8" s="5">
-        <f>K8*Inputs!$C$39</f>
-        <v>36000.0</v>
+        <f>K8*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -2612,39 +2640,39 @@
       </c>
       <c r="O8" s="5">
         <f>C8-K8</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P8" s="5">
         <f>IF(SUM($F8:$I8)=0,0,L8*F8/SUM($F8:$I8))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q8" s="5">
         <f>IF(SUM($F8:$I8)=0,0,L8*G8/SUM($F8:$I8))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R8" s="5">
         <f>IF(SUM($F8:$I8)=0,0,L8*H8/SUM($F8:$I8))</f>
-        <v>6000.0</v>
+        <v/>
       </c>
       <c r="S8" s="5">
         <f>IF(SUM($F8:$I8)=0,0,L8*I8/SUM($F8:$I8))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T8" s="5">
         <f>IF(SUM($F8:$I8)=0,0,M8*F8/SUM($F8:$I8))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U8" s="5">
         <f>IF(SUM($F8:$I8)=0,0,M8*G8/SUM($F8:$I8))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V8" s="5">
         <f>IF(SUM($F8:$I8)=0,0,M8*H8/SUM($F8:$I8))</f>
-        <v>36000.0</v>
+        <v/>
       </c>
       <c r="W8" s="5">
         <f>IF(SUM($F8:$I8)=0,0,M8*I8/SUM($F8:$I8))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -2655,19 +2683,19 @@
       </c>
       <c r="B9" s="5">
         <f>(1-Inputs!$B$13)*Derived!B4*Inputs!$B$19/1000</f>
-        <v>1858.0599999999997</v>
+        <v/>
       </c>
       <c r="C9" s="5">
         <f>(1-Inputs!$C$13)*Derived!C4*Inputs!$C$19/1000</f>
-        <v>7432.239999999999</v>
+        <v/>
       </c>
       <c r="D9" s="5">
         <f>D8+B9</f>
-        <v>1281858.06</v>
+        <v/>
       </c>
       <c r="E9" s="5">
         <f>E8+C9</f>
-        <v>2607432.24</v>
+        <v/>
       </c>
       <c r="F9" s="6" t="n">
         <v>1</v>
@@ -2683,19 +2711,19 @@
       </c>
       <c r="J9" s="5">
         <f>B9*SUM($F9:$I9)</f>
-        <v>1858.0599999999997</v>
+        <v/>
       </c>
       <c r="K9" s="5">
         <f>C9*SUM($F9:$I9)</f>
-        <v>7432.239999999999</v>
+        <v/>
       </c>
       <c r="L9" s="5">
         <f>SUM($F9:$I9)*(1-Inputs!$B$13)*Derived!B3*Derived!B6/1000</f>
-        <v>695.657664</v>
+        <v/>
       </c>
       <c r="M9" s="5">
         <f>SUM($F9:$I9)*(1-Inputs!$C$13)*Derived!C3*Derived!C6/1000</f>
-        <v>1391.315328</v>
+        <v/>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -2704,39 +2732,39 @@
       </c>
       <c r="O9" s="5">
         <f>C9-K9</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P9" s="5">
         <f>IF(SUM($F9:$I9)=0,0,L9*F9/SUM($F9:$I9))</f>
-        <v>695.657664</v>
+        <v/>
       </c>
       <c r="Q9" s="5">
         <f>IF(SUM($F9:$I9)=0,0,L9*G9/SUM($F9:$I9))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R9" s="5">
         <f>IF(SUM($F9:$I9)=0,0,L9*H9/SUM($F9:$I9))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S9" s="5">
         <f>IF(SUM($F9:$I9)=0,0,L9*I9/SUM($F9:$I9))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T9" s="5">
         <f>IF(SUM($F9:$I9)=0,0,M9*F9/SUM($F9:$I9))</f>
-        <v>1391.315328</v>
+        <v/>
       </c>
       <c r="U9" s="5">
         <f>IF(SUM($F9:$I9)=0,0,M9*G9/SUM($F9:$I9))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V9" s="5">
         <f>IF(SUM($F9:$I9)=0,0,M9*H9/SUM($F9:$I9))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W9" s="5">
         <f>IF(SUM($F9:$I9)=0,0,M9*I9/SUM($F9:$I9))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -2747,19 +2775,19 @@
       </c>
       <c r="B10" s="5">
         <f>Inputs!$B$6*0.092903*Inputs!$B$20/1000</f>
-        <v>185.806</v>
+        <v/>
       </c>
       <c r="C10" s="5">
         <f>Inputs!$C$6*0.092903*Inputs!$C$20/1000</f>
-        <v>929.03</v>
+        <v/>
       </c>
       <c r="D10" s="5">
         <f>D9+B10</f>
-        <v>1282043.8660000002</v>
+        <v/>
       </c>
       <c r="E10" s="5">
         <f>E9+C10</f>
-        <v>2608361.27</v>
+        <v/>
       </c>
       <c r="F10" s="6" t="n">
         <v>1</v>
@@ -2775,19 +2803,19 @@
       </c>
       <c r="J10" s="5">
         <f>B10*SUM($F10:$I10)</f>
-        <v>185.806</v>
+        <v/>
       </c>
       <c r="K10" s="5">
         <f>C10*SUM($F10:$I10)</f>
-        <v>929.03</v>
+        <v/>
       </c>
       <c r="L10" s="5">
         <f>SUM($F10:$I10)*Inputs!$B$6*Derived!B6/1000</f>
-        <v>173.914416</v>
+        <v/>
       </c>
       <c r="M10" s="5">
         <f>SUM($F10:$I10)*Inputs!$C$6*Derived!C6/1000</f>
-        <v>434.78603999999996</v>
+        <v/>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -2796,39 +2824,39 @@
       </c>
       <c r="O10" s="5">
         <f>C10-K10</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P10" s="5">
         <f>IF(SUM($F10:$I10)=0,0,L10*F10/SUM($F10:$I10))</f>
-        <v>173.914416</v>
+        <v/>
       </c>
       <c r="Q10" s="5">
         <f>IF(SUM($F10:$I10)=0,0,L10*G10/SUM($F10:$I10))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R10" s="5">
         <f>IF(SUM($F10:$I10)=0,0,L10*H10/SUM($F10:$I10))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S10" s="5">
         <f>IF(SUM($F10:$I10)=0,0,L10*I10/SUM($F10:$I10))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T10" s="5">
         <f>IF(SUM($F10:$I10)=0,0,M10*F10/SUM($F10:$I10))</f>
-        <v>434.78603999999996</v>
+        <v/>
       </c>
       <c r="U10" s="5">
         <f>IF(SUM($F10:$I10)=0,0,M10*G10/SUM($F10:$I10))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V10" s="5">
         <f>IF(SUM($F10:$I10)=0,0,M10*H10/SUM($F10:$I10))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W10" s="5">
         <f>IF(SUM($F10:$I10)=0,0,M10*I10/SUM($F10:$I10))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -2839,19 +2867,19 @@
       </c>
       <c r="B11" s="5">
         <f>Inputs!$B$7*1000*Inputs!$B$21/1000</f>
-        <v>300.0</v>
+        <v/>
       </c>
       <c r="C11" s="5">
         <f>Inputs!$C$7*1000*Inputs!$C$21/1000</f>
-        <v>1000.0</v>
+        <v/>
       </c>
       <c r="D11" s="5">
         <f>D10+B11</f>
-        <v>1282343.8660000002</v>
+        <v/>
       </c>
       <c r="E11" s="5">
         <f>E10+C11</f>
-        <v>2609361.27</v>
+        <v/>
       </c>
       <c r="F11" s="6" t="n">
         <v>1</v>
@@ -2867,19 +2895,19 @@
       </c>
       <c r="J11" s="5">
         <f>B11*SUM($F11:$I11)</f>
-        <v>300.0</v>
+        <v/>
       </c>
       <c r="K11" s="5">
         <f>C11*SUM($F11:$I11)</f>
-        <v>1000.0</v>
+        <v/>
       </c>
       <c r="L11" s="5">
         <f>SUM($F11:$I11)*Derived!B5*Derived!B6/1000</f>
-        <v>233.99999999999997</v>
+        <v/>
       </c>
       <c r="M11" s="5">
         <f>SUM($F11:$I11)*Derived!C5*Derived!C6/1000</f>
-        <v>467.99999999999994</v>
+        <v/>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -2888,39 +2916,39 @@
       </c>
       <c r="O11" s="5">
         <f>C11-K11</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,L11*F11/SUM($F11:$I11))</f>
-        <v>233.99999999999997</v>
+        <v/>
       </c>
       <c r="Q11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,L11*G11/SUM($F11:$I11))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,L11*H11/SUM($F11:$I11))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,L11*I11/SUM($F11:$I11))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,M11*F11/SUM($F11:$I11))</f>
-        <v>467.99999999999994</v>
+        <v/>
       </c>
       <c r="U11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,M11*G11/SUM($F11:$I11))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,M11*H11/SUM($F11:$I11))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,M11*I11/SUM($F11:$I11))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -2955,19 +2983,19 @@
       </c>
       <c r="B13" s="5">
         <f>Inputs!$B$18*Inputs!$B$2</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="C13" s="5">
         <f>Inputs!$C$18*Inputs!$C$2</f>
-        <v>15000.0</v>
+        <v/>
       </c>
       <c r="D13" s="5">
         <f>D11+B13</f>
-        <v>1287343.8660000002</v>
+        <v/>
       </c>
       <c r="E13" s="5">
         <f>E11+C13</f>
-        <v>2624361.27</v>
+        <v/>
       </c>
       <c r="F13" s="6" t="n">
         <v>0</v>
@@ -2983,19 +3011,19 @@
       </c>
       <c r="J13" s="5">
         <f>B13*SUM($F13:$I13)</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="K13" s="5">
         <f>C13*SUM($F13:$I13)</f>
-        <v>15000.0</v>
+        <v/>
       </c>
       <c r="L13" s="5">
-        <f>J13*Inputs!$B$39</f>
-        <v>1500.0</v>
+        <f>J13*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M13" s="5">
-        <f>K13*Inputs!$C$39</f>
-        <v>9000.0</v>
+        <f>K13*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -3004,39 +3032,39 @@
       </c>
       <c r="O13" s="5">
         <f>C13-K13</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P13" s="5">
         <f>IF(SUM($F13:$I13)=0,0,L13*F13/SUM($F13:$I13))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q13" s="5">
         <f>IF(SUM($F13:$I13)=0,0,L13*G13/SUM($F13:$I13))</f>
-        <v>1500.0</v>
+        <v/>
       </c>
       <c r="R13" s="5">
         <f>IF(SUM($F13:$I13)=0,0,L13*H13/SUM($F13:$I13))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S13" s="5">
         <f>IF(SUM($F13:$I13)=0,0,L13*I13/SUM($F13:$I13))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T13" s="5">
         <f>IF(SUM($F13:$I13)=0,0,M13*F13/SUM($F13:$I13))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U13" s="5">
         <f>IF(SUM($F13:$I13)=0,0,M13*G13/SUM($F13:$I13))</f>
-        <v>9000.0</v>
+        <v/>
       </c>
       <c r="V13" s="5">
         <f>IF(SUM($F13:$I13)=0,0,M13*H13/SUM($F13:$I13))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W13" s="5">
         <f>IF(SUM($F13:$I13)=0,0,M13*I13/SUM($F13:$I13))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -3047,19 +3075,19 @@
       </c>
       <c r="B14" s="5">
         <f>Inputs!$B$22*Inputs!$B$2</f>
-        <v>2000.0</v>
+        <v/>
       </c>
       <c r="C14" s="5">
         <f>Inputs!$C$22*Inputs!$C$2</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="D14" s="5">
         <f>D13+B14</f>
-        <v>1289343.8660000002</v>
+        <v/>
       </c>
       <c r="E14" s="5">
         <f>E13+C14</f>
-        <v>2629361.27</v>
+        <v/>
       </c>
       <c r="F14" s="6" t="n">
         <v>0</v>
@@ -3075,19 +3103,19 @@
       </c>
       <c r="J14" s="5">
         <f>B14*SUM($F14:$I14)</f>
-        <v>2000.0</v>
+        <v/>
       </c>
       <c r="K14" s="5">
         <f>C14*SUM($F14:$I14)</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="L14" s="5">
-        <f>J14*Inputs!$B$39</f>
-        <v>600.0</v>
+        <f>J14*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M14" s="5">
-        <f>K14*Inputs!$C$39</f>
-        <v>3000.0</v>
+        <f>K14*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -3096,39 +3124,39 @@
       </c>
       <c r="O14" s="5">
         <f>C14-K14</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P14" s="5">
         <f>IF(SUM($F14:$I14)=0,0,L14*F14/SUM($F14:$I14))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q14" s="5">
         <f>IF(SUM($F14:$I14)=0,0,L14*G14/SUM($F14:$I14))</f>
-        <v>600.0</v>
+        <v/>
       </c>
       <c r="R14" s="5">
         <f>IF(SUM($F14:$I14)=0,0,L14*H14/SUM($F14:$I14))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S14" s="5">
         <f>IF(SUM($F14:$I14)=0,0,L14*I14/SUM($F14:$I14))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T14" s="5">
         <f>IF(SUM($F14:$I14)=0,0,M14*F14/SUM($F14:$I14))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U14" s="5">
         <f>IF(SUM($F14:$I14)=0,0,M14*G14/SUM($F14:$I14))</f>
-        <v>3000.0</v>
+        <v/>
       </c>
       <c r="V14" s="5">
         <f>IF(SUM($F14:$I14)=0,0,M14*H14/SUM($F14:$I14))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W14" s="5">
         <f>IF(SUM($F14:$I14)=0,0,M14*I14/SUM($F14:$I14))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -3139,19 +3167,19 @@
       </c>
       <c r="B15" s="5">
         <f>Inputs!$B$23*Inputs!$B$2</f>
-        <v>2000.0</v>
+        <v/>
       </c>
       <c r="C15" s="5">
         <f>Inputs!$C$23*Inputs!$C$2</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="D15" s="5">
         <f>D14+B15</f>
-        <v>1291343.8660000002</v>
+        <v/>
       </c>
       <c r="E15" s="5">
         <f>E14+C15</f>
-        <v>2634361.27</v>
+        <v/>
       </c>
       <c r="F15" s="6" t="n">
         <v>0</v>
@@ -3167,60 +3195,60 @@
       </c>
       <c r="J15" s="5">
         <f>B15*SUM($F15:$I15)</f>
-        <v>2000.0</v>
+        <v/>
       </c>
       <c r="K15" s="5">
         <f>C15*SUM($F15:$I15)</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="L15" s="5">
-        <f>J15*Inputs!$B$39</f>
-        <v>600.0</v>
+        <f>J15*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M15" s="5">
-        <f>K15*Inputs!$C$39</f>
-        <v>3000.0</v>
+        <f>K15*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Design values, seismic qualification</t>
+          <t>A few months of design and load-data development (Alex 2026-09-04)</t>
         </is>
       </c>
       <c r="O15" s="5">
         <f>C15-K15</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P15" s="5">
         <f>IF(SUM($F15:$I15)=0,0,L15*F15/SUM($F15:$I15))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q15" s="5">
         <f>IF(SUM($F15:$I15)=0,0,L15*G15/SUM($F15:$I15))</f>
-        <v>600.0</v>
+        <v/>
       </c>
       <c r="R15" s="5">
         <f>IF(SUM($F15:$I15)=0,0,L15*H15/SUM($F15:$I15))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S15" s="5">
         <f>IF(SUM($F15:$I15)=0,0,L15*I15/SUM($F15:$I15))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T15" s="5">
         <f>IF(SUM($F15:$I15)=0,0,M15*F15/SUM($F15:$I15))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U15" s="5">
         <f>IF(SUM($F15:$I15)=0,0,M15*G15/SUM($F15:$I15))</f>
-        <v>3000.0</v>
+        <v/>
       </c>
       <c r="V15" s="5">
         <f>IF(SUM($F15:$I15)=0,0,M15*H15/SUM($F15:$I15))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W15" s="5">
         <f>IF(SUM($F15:$I15)=0,0,M15*I15/SUM($F15:$I15))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -3231,26 +3259,26 @@
       </c>
       <c r="B16" s="5">
         <f>Inputs!$B$24*Inputs!$B$2</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="C16" s="5">
         <f>Inputs!$C$24*Inputs!$C$2</f>
-        <v>10000.0</v>
+        <v/>
       </c>
       <c r="D16" s="5">
         <f>D15+B16</f>
-        <v>1296343.8660000002</v>
+        <v/>
       </c>
       <c r="E16" s="5">
         <f>E15+C16</f>
-        <v>2644361.27</v>
+        <v/>
       </c>
       <c r="F16" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="6">
-        <f>Inputs!$B$41</f>
-        <v>0.5</v>
+        <f>Inputs!$B$42</f>
+        <v/>
       </c>
       <c r="H16" s="6" t="n">
         <v>0</v>
@@ -3260,19 +3288,19 @@
       </c>
       <c r="J16" s="5">
         <f>B16*SUM($F16:$I16)</f>
-        <v>2500.0</v>
+        <v/>
       </c>
       <c r="K16" s="5">
         <f>C16*SUM($F16:$I16)</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="L16" s="5">
-        <f>J16*Inputs!$B$39</f>
-        <v>750.0</v>
+        <f>J16*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M16" s="5">
-        <f>K16*Inputs!$C$39</f>
-        <v>3000.0</v>
+        <f>K16*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -3281,39 +3309,39 @@
       </c>
       <c r="O16" s="5">
         <f>C16-K16</f>
-        <v>5000.0</v>
+        <v/>
       </c>
       <c r="P16" s="5">
         <f>IF(SUM($F16:$I16)=0,0,L16*F16/SUM($F16:$I16))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q16" s="5">
         <f>IF(SUM($F16:$I16)=0,0,L16*G16/SUM($F16:$I16))</f>
-        <v>750.0</v>
+        <v/>
       </c>
       <c r="R16" s="5">
         <f>IF(SUM($F16:$I16)=0,0,L16*H16/SUM($F16:$I16))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S16" s="5">
         <f>IF(SUM($F16:$I16)=0,0,L16*I16/SUM($F16:$I16))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T16" s="5">
         <f>IF(SUM($F16:$I16)=0,0,M16*F16/SUM($F16:$I16))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U16" s="5">
         <f>IF(SUM($F16:$I16)=0,0,M16*G16/SUM($F16:$I16))</f>
-        <v>3000.0</v>
+        <v/>
       </c>
       <c r="V16" s="5">
         <f>IF(SUM($F16:$I16)=0,0,M16*H16/SUM($F16:$I16))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W16" s="5">
         <f>IF(SUM($F16:$I16)=0,0,M16*I16/SUM($F16:$I16))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -3323,20 +3351,20 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>Inputs!$B$33*Inputs!$B$2</f>
-        <v>3000.0</v>
+        <f>Inputs!$B$34*Inputs!$B$2</f>
+        <v/>
       </c>
       <c r="C17" s="5">
-        <f>Inputs!$C$33*Inputs!$C$2</f>
-        <v>8000.0</v>
+        <f>Inputs!$C$34*Inputs!$C$2</f>
+        <v/>
       </c>
       <c r="D17" s="5">
         <f>D16+B17</f>
-        <v>1299343.8660000002</v>
+        <v/>
       </c>
       <c r="E17" s="5">
         <f>E16+C17</f>
-        <v>2652361.27</v>
+        <v/>
       </c>
       <c r="F17" s="6" t="n">
         <v>0</v>
@@ -3352,19 +3380,19 @@
       </c>
       <c r="J17" s="5">
         <f>B17*SUM($F17:$I17)</f>
-        <v>3000.0</v>
+        <v/>
       </c>
       <c r="K17" s="5">
         <f>C17*SUM($F17:$I17)</f>
-        <v>8000.0</v>
+        <v/>
       </c>
       <c r="L17" s="5">
-        <f>J17*Inputs!$B$39</f>
-        <v>900.0</v>
+        <f>J17*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M17" s="5">
-        <f>K17*Inputs!$C$39</f>
-        <v>4800.0</v>
+        <f>K17*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -3373,39 +3401,39 @@
       </c>
       <c r="O17" s="5">
         <f>C17-K17</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P17" s="5">
         <f>IF(SUM($F17:$I17)=0,0,L17*F17/SUM($F17:$I17))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q17" s="5">
         <f>IF(SUM($F17:$I17)=0,0,L17*G17/SUM($F17:$I17))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R17" s="5">
         <f>IF(SUM($F17:$I17)=0,0,L17*H17/SUM($F17:$I17))</f>
-        <v>900.0</v>
+        <v/>
       </c>
       <c r="S17" s="5">
         <f>IF(SUM($F17:$I17)=0,0,L17*I17/SUM($F17:$I17))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T17" s="5">
         <f>IF(SUM($F17:$I17)=0,0,M17*F17/SUM($F17:$I17))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U17" s="5">
         <f>IF(SUM($F17:$I17)=0,0,M17*G17/SUM($F17:$I17))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V17" s="5">
         <f>IF(SUM($F17:$I17)=0,0,M17*H17/SUM($F17:$I17))</f>
-        <v>4800.0</v>
+        <v/>
       </c>
       <c r="W17" s="5">
         <f>IF(SUM($F17:$I17)=0,0,M17*I17/SUM($F17:$I17))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -3416,19 +3444,19 @@
       </c>
       <c r="B18" s="5">
         <f>Inputs!$B$25*Inputs!$B$2</f>
-        <v>1000.0</v>
+        <v/>
       </c>
       <c r="C18" s="5">
         <f>Inputs!$C$25*Inputs!$C$2</f>
-        <v>3000.0</v>
+        <v/>
       </c>
       <c r="D18" s="5">
         <f>D17+B18</f>
-        <v>1300343.8660000002</v>
+        <v/>
       </c>
       <c r="E18" s="5">
         <f>E17+C18</f>
-        <v>2655361.27</v>
+        <v/>
       </c>
       <c r="F18" s="6" t="n">
         <v>1</v>
@@ -3444,19 +3472,19 @@
       </c>
       <c r="J18" s="5">
         <f>B18*SUM($F18:$I18)</f>
-        <v>1000.0</v>
+        <v/>
       </c>
       <c r="K18" s="5">
         <f>C18*SUM($F18:$I18)</f>
-        <v>3000.0</v>
+        <v/>
       </c>
       <c r="L18" s="5">
         <f>SUM($F18:$I18)*(Inputs!$B$9+Inputs!$B$10)*Derived!B6/1000</f>
-        <v>130.435812</v>
+        <v/>
       </c>
       <c r="M18" s="5">
         <f>SUM($F18:$I18)*(Inputs!$C$9+Inputs!$C$10)*Derived!C6/1000</f>
-        <v>391.307436</v>
+        <v/>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -3465,39 +3493,39 @@
       </c>
       <c r="O18" s="5">
         <f>C18-K18</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="P18" s="5">
         <f>IF(SUM($F18:$I18)=0,0,L18*F18/SUM($F18:$I18))</f>
-        <v>130.435812</v>
+        <v/>
       </c>
       <c r="Q18" s="5">
         <f>IF(SUM($F18:$I18)=0,0,L18*G18/SUM($F18:$I18))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R18" s="5">
         <f>IF(SUM($F18:$I18)=0,0,L18*H18/SUM($F18:$I18))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S18" s="5">
         <f>IF(SUM($F18:$I18)=0,0,L18*I18/SUM($F18:$I18))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T18" s="5">
         <f>IF(SUM($F18:$I18)=0,0,M18*F18/SUM($F18:$I18))</f>
-        <v>391.307436</v>
+        <v/>
       </c>
       <c r="U18" s="5">
         <f>IF(SUM($F18:$I18)=0,0,M18*G18/SUM($F18:$I18))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V18" s="5">
         <f>IF(SUM($F18:$I18)=0,0,M18*H18/SUM($F18:$I18))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W18" s="5">
         <f>IF(SUM($F18:$I18)=0,0,M18*I18/SUM($F18:$I18))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -3508,19 +3536,19 @@
       </c>
       <c r="B19" s="5">
         <f>Inputs!$B$26*Inputs!$B$2</f>
-        <v>50000.0</v>
+        <v/>
       </c>
       <c r="C19" s="5">
         <f>Inputs!$C$26*Inputs!$C$2</f>
-        <v>100000.0</v>
+        <v/>
       </c>
       <c r="D19" s="5">
         <f>D18+B19</f>
-        <v>1350343.8660000002</v>
+        <v/>
       </c>
       <c r="E19" s="5">
         <f>E18+C19</f>
-        <v>2755361.27</v>
+        <v/>
       </c>
       <c r="F19" s="6" t="n">
         <v>0</v>
@@ -3536,19 +3564,19 @@
       </c>
       <c r="J19" s="5">
         <f>B19*SUM($F19:$I19)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="K19" s="5">
         <f>C19*SUM($F19:$I19)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="L19" s="5">
         <f>0</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="M19" s="5">
         <f>0</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -3557,39 +3585,39 @@
       </c>
       <c r="O19" s="5">
         <f>C19-K19</f>
-        <v>100000.0</v>
+        <v/>
       </c>
       <c r="P19" s="5">
         <f>IF(SUM($F19:$I19)=0,0,L19*F19/SUM($F19:$I19))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q19" s="5">
         <f>IF(SUM($F19:$I19)=0,0,L19*G19/SUM($F19:$I19))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R19" s="5">
         <f>IF(SUM($F19:$I19)=0,0,L19*H19/SUM($F19:$I19))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S19" s="5">
         <f>IF(SUM($F19:$I19)=0,0,L19*I19/SUM($F19:$I19))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T19" s="5">
         <f>IF(SUM($F19:$I19)=0,0,M19*F19/SUM($F19:$I19))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U19" s="5">
         <f>IF(SUM($F19:$I19)=0,0,M19*G19/SUM($F19:$I19))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V19" s="5">
         <f>IF(SUM($F19:$I19)=0,0,M19*H19/SUM($F19:$I19))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W19" s="5">
         <f>IF(SUM($F19:$I19)=0,0,M19*I19/SUM($F19:$I19))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -3600,19 +3628,19 @@
       </c>
       <c r="B20" s="5">
         <f>Inputs!$B$27*Inputs!$B$2</f>
-        <v>20000.0</v>
+        <v/>
       </c>
       <c r="C20" s="5">
         <f>Inputs!$C$27*Inputs!$C$2</f>
-        <v>50000.0</v>
+        <v/>
       </c>
       <c r="D20" s="5">
         <f>D19+B20</f>
-        <v>1370343.8660000002</v>
+        <v/>
       </c>
       <c r="E20" s="5">
         <f>E19+C20</f>
-        <v>2805361.27</v>
+        <v/>
       </c>
       <c r="F20" s="6" t="n">
         <v>0</v>
@@ -3628,19 +3656,19 @@
       </c>
       <c r="J20" s="5">
         <f>B20*SUM($F20:$I20)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="K20" s="5">
         <f>C20*SUM($F20:$I20)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="L20" s="5">
         <f>0</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="M20" s="5">
         <f>0</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -3649,39 +3677,39 @@
       </c>
       <c r="O20" s="5">
         <f>C20-K20</f>
-        <v>50000.0</v>
+        <v/>
       </c>
       <c r="P20" s="5">
         <f>IF(SUM($F20:$I20)=0,0,L20*F20/SUM($F20:$I20))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q20" s="5">
         <f>IF(SUM($F20:$I20)=0,0,L20*G20/SUM($F20:$I20))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R20" s="5">
         <f>IF(SUM($F20:$I20)=0,0,L20*H20/SUM($F20:$I20))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S20" s="5">
         <f>IF(SUM($F20:$I20)=0,0,L20*I20/SUM($F20:$I20))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T20" s="5">
         <f>IF(SUM($F20:$I20)=0,0,M20*F20/SUM($F20:$I20))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U20" s="5">
         <f>IF(SUM($F20:$I20)=0,0,M20*G20/SUM($F20:$I20))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V20" s="5">
         <f>IF(SUM($F20:$I20)=0,0,M20*H20/SUM($F20:$I20))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W20" s="5">
         <f>IF(SUM($F20:$I20)=0,0,M20*I20/SUM($F20:$I20))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -3692,19 +3720,19 @@
       </c>
       <c r="B21" s="5">
         <f>Inputs!$B$28*Inputs!$B$2</f>
-        <v>15000.0</v>
+        <v/>
       </c>
       <c r="C21" s="5">
         <f>Inputs!$C$28*Inputs!$C$2</f>
-        <v>70000.0</v>
+        <v/>
       </c>
       <c r="D21" s="5">
         <f>D20+B21</f>
-        <v>1385343.8660000002</v>
+        <v/>
       </c>
       <c r="E21" s="5">
         <f>E20+C21</f>
-        <v>2875361.27</v>
+        <v/>
       </c>
       <c r="F21" s="6" t="n">
         <v>0</v>
@@ -3715,65 +3743,66 @@
       <c r="H21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="6" t="n">
-        <v>0</v>
+      <c r="I21" s="6">
+        <f>Inputs!$B$29</f>
+        <v/>
       </c>
       <c r="J21" s="5">
         <f>B21*SUM($F21:$I21)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="K21" s="5">
         <f>C21*SUM($F21:$I21)</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="L21" s="5">
-        <f>0</f>
-        <v>0.0</v>
+        <f>J21*Inputs!$B$40</f>
+        <v/>
       </c>
       <c r="M21" s="5">
-        <f>0</f>
-        <v>0.0</v>
+        <f>K21*Inputs!$C$40</f>
+        <v/>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Rack masses [H]; aggregate [L]</t>
+          <t>Server and equipment enclosures only (40% of IT mass, estimate); electronics never. Rack masses [H]; aggregate [L]</t>
         </is>
       </c>
       <c r="O21" s="5">
         <f>C21-K21</f>
-        <v>70000.0</v>
+        <v/>
       </c>
       <c r="P21" s="5">
         <f>IF(SUM($F21:$I21)=0,0,L21*F21/SUM($F21:$I21))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="Q21" s="5">
         <f>IF(SUM($F21:$I21)=0,0,L21*G21/SUM($F21:$I21))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="R21" s="5">
         <f>IF(SUM($F21:$I21)=0,0,L21*H21/SUM($F21:$I21))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="S21" s="5">
         <f>IF(SUM($F21:$I21)=0,0,L21*I21/SUM($F21:$I21))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="T21" s="5">
         <f>IF(SUM($F21:$I21)=0,0,M21*F21/SUM($F21:$I21))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="U21" s="5">
         <f>IF(SUM($F21:$I21)=0,0,M21*G21/SUM($F21:$I21))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="V21" s="5">
         <f>IF(SUM($F21:$I21)=0,0,M21*H21/SUM($F21:$I21))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="W21" s="5">
         <f>IF(SUM($F21:$I21)=0,0,M21*I21/SUM($F21:$I21))</f>
-        <v>0.0</v>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -3791,11 +3820,11 @@
       </c>
       <c r="B24" s="8">
         <f>SUM(B3:B21)</f>
-        <v>1385343.866</v>
+        <v/>
       </c>
       <c r="C24" s="8">
         <f>SUM(C3:C21)</f>
-        <v>2875361.27</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -3806,11 +3835,11 @@
       </c>
       <c r="B25" s="8">
         <f>B24-B3-B4-B5</f>
-        <v>185343.86599999992</v>
+        <v/>
       </c>
       <c r="C25" s="8">
         <f>C24-C3-C4-C5</f>
-        <v>475361.27</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -3828,11 +3857,11 @@
       </c>
       <c r="B28" s="10">
         <f>SUMPRODUCT(B3:B21,F3:F21)</f>
-        <v>3343.866</v>
+        <v/>
       </c>
       <c r="C28" s="10">
         <f>SUMPRODUCT(C3:C21,F3:F21)</f>
-        <v>12361.269999999999</v>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -3843,11 +3872,11 @@
       </c>
       <c r="B29" s="10">
         <f>SUM(P3:P21)</f>
-        <v>1234.0078919999999</v>
+        <v/>
       </c>
       <c r="C29" s="10">
         <f>SUM(T3:T21)</f>
-        <v>2685.4088039999997</v>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -3858,11 +3887,11 @@
       </c>
       <c r="B30" s="10">
         <f>B29*1000/Derived!B6</f>
-        <v>1419097.8762795602</v>
+        <v/>
       </c>
       <c r="C30" s="10">
         <f>C29*1000/Derived!C6</f>
-        <v>3088195.7525591203</v>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -3873,11 +3902,11 @@
       </c>
       <c r="B31" s="11">
         <f>B29/Derived!B7</f>
-        <v>1.4190978762795603</v>
+        <v/>
       </c>
       <c r="C31" s="11">
         <f>C29/Derived!C7</f>
-        <v>3.0881957525591206</v>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -3888,11 +3917,11 @@
       </c>
       <c r="B33" s="10">
         <f>SUMPRODUCT(B3:B21,G3:G21)</f>
-        <v>11500.0</v>
+        <v/>
       </c>
       <c r="C33" s="10">
         <f>SUMPRODUCT(C3:C21,G3:G21)</f>
-        <v>30000.0</v>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -3903,11 +3932,11 @@
       </c>
       <c r="B34" s="10">
         <f>SUM(Q3:Q21)</f>
-        <v>3450.0</v>
+        <v/>
       </c>
       <c r="C34" s="10">
         <f>SUM(U3:U21)</f>
-        <v>18000.0</v>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -3918,11 +3947,11 @@
       </c>
       <c r="B35" s="11">
         <f>B34/Derived!B8</f>
-        <v>0.11020746357603078</v>
+        <v/>
       </c>
       <c r="C35" s="11">
         <f>C34/Derived!C8</f>
-        <v>0.5749954621358128</v>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -3933,11 +3962,11 @@
       </c>
       <c r="B37" s="10">
         <f>SUMPRODUCT(B3:B21,H3:H21)</f>
-        <v>53000.0</v>
+        <v/>
       </c>
       <c r="C37" s="10">
         <f>SUMPRODUCT(C3:C21,H3:H21)</f>
-        <v>108000.0</v>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -3948,11 +3977,11 @@
       </c>
       <c r="B38" s="10">
         <f>SUM(R3:R21)</f>
-        <v>15900.0</v>
+        <v/>
       </c>
       <c r="C38" s="10">
         <f>SUM(V3:V21)</f>
-        <v>64800.0</v>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -3963,11 +3992,11 @@
       </c>
       <c r="B39" s="11">
         <f>B38/Derived!B8</f>
-        <v>0.507912658219968</v>
+        <v/>
       </c>
       <c r="C39" s="11">
         <f>C38/Derived!C8</f>
-        <v>2.069983663688926</v>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -3978,11 +4007,11 @@
       </c>
       <c r="B41" s="10">
         <f>SUMPRODUCT(B3:B21,I3:I21)</f>
-        <v>996300.0</v>
+        <v/>
       </c>
       <c r="C41" s="10">
         <f>SUMPRODUCT(C3:C21,I3:I21)</f>
-        <v>2061000.0</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -3993,11 +4022,11 @@
       </c>
       <c r="B42" s="10">
         <f>SUM(S3:S21)</f>
-        <v>55890.0</v>
+        <v/>
       </c>
       <c r="C42" s="10">
         <f>SUM(W3:W21)</f>
-        <v>345600.0</v>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -4008,11 +4037,11 @@
       </c>
       <c r="B43" s="11">
         <f>B42/Derived!B8</f>
-        <v>1.7853609099316987</v>
+        <v/>
       </c>
       <c r="C43" s="11">
         <f>C42/Derived!C8</f>
-        <v>11.039912873007607</v>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -4023,11 +4052,11 @@
       </c>
       <c r="B45" s="8">
         <f>SUM(J3:J21)</f>
-        <v>1064143.866</v>
+        <v/>
       </c>
       <c r="C45" s="8">
         <f>SUM(K3:K21)</f>
-        <v>2211361.27</v>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -4038,11 +4067,11 @@
       </c>
       <c r="B46" s="8">
         <f>SUM(L3:L21)</f>
-        <v>76474.007892</v>
+        <v/>
       </c>
       <c r="C46" s="8">
         <f>SUM(M3:M21)</f>
-        <v>431085.408804</v>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -4053,11 +4082,11 @@
       </c>
       <c r="B47" s="11">
         <f>B46/Derived!B8</f>
-        <v>2.4429004171799074</v>
+        <v/>
       </c>
       <c r="C47" s="11">
         <f>C46/Derived!C8</f>
-        <v>13.77067521418121</v>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -4068,11 +4097,11 @@
       </c>
       <c r="B48" s="12">
         <f>B45/B24</f>
-        <v>0.7681442074541224</v>
+        <v/>
       </c>
       <c r="C48" s="12">
         <f>C45/C24</f>
-        <v>0.7690724964101642</v>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -4083,11 +4112,11 @@
       </c>
       <c r="B49" s="12">
         <f>(B45-B41)/B25</f>
-        <v>0.36604322260117284</v>
+        <v/>
       </c>
       <c r="C49" s="12">
         <f>(C45-C41)/C25</f>
-        <v>0.3163094671132968</v>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -4098,11 +4127,11 @@
       </c>
       <c r="B50" s="8">
         <f>B24-B45</f>
-        <v>321200.0</v>
+        <v/>
       </c>
       <c r="C50" s="8">
         <f>C24-C45</f>
-        <v>664000.0</v>
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -4113,11 +4142,11 @@
       </c>
       <c r="B51" s="12">
         <f>B50/B24</f>
-        <v>0.23185579254587757</v>
+        <v/>
       </c>
       <c r="C51" s="12">
         <f>C50/C24</f>
-        <v>0.23092750358983585</v>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4171,11 +4200,11 @@
       </c>
       <c r="B2" s="13">
         <f>Inputs!$B$3*Inputs!$B$2/Inputs!$B$4</f>
-        <v>5.0</v>
+        <v/>
       </c>
       <c r="C2" s="13">
         <f>Inputs!$C$3*Inputs!$C$2/Inputs!$C$4</f>
-        <v>10.0</v>
+        <v/>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -4191,11 +4220,11 @@
       </c>
       <c r="B3" s="13">
         <f>B2*Inputs!$B$5</f>
-        <v>800000.0</v>
+        <v/>
       </c>
       <c r="C3" s="13">
         <f>C2*Inputs!$C$5</f>
-        <v>1600000.0</v>
+        <v/>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -4211,11 +4240,11 @@
       </c>
       <c r="B4" s="13">
         <f>B3*0.092903</f>
-        <v>74322.4</v>
+        <v/>
       </c>
       <c r="C4" s="13">
         <f>C3*0.092903</f>
-        <v>148644.8</v>
+        <v/>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -4231,11 +4260,11 @@
       </c>
       <c r="B5" s="13">
         <f>Inputs!$B$7*1000*Inputs!$B$8/0.092903</f>
-        <v>269097.8762795604</v>
+        <v/>
       </c>
       <c r="C5" s="13">
         <f>Inputs!$C$7*1000*Inputs!$C$8/0.092903</f>
-        <v>538195.7525591208</v>
+        <v/>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -4250,12 +4279,12 @@
         </is>
       </c>
       <c r="B6" s="13">
-        <f>Inputs!$B$35/1000*Inputs!$B$36*0.092903</f>
-        <v>0.86957208</v>
+        <f>Inputs!$B$36/1000*Inputs!$B$37*0.092903</f>
+        <v/>
       </c>
       <c r="C6" s="13">
-        <f>Inputs!$C$35/1000*Inputs!$C$36*0.092903</f>
-        <v>0.86957208</v>
+        <f>Inputs!$C$36/1000*Inputs!$C$37*0.092903</f>
+        <v/>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -4270,12 +4299,12 @@
         </is>
       </c>
       <c r="B7" s="13">
-        <f>Inputs!$B$37*B6/1000</f>
-        <v>869.5720799999999</v>
+        <f>Inputs!$B$38*B6/1000</f>
+        <v/>
       </c>
       <c r="C7" s="13">
-        <f>Inputs!$C$37*C6/1000</f>
-        <v>869.5720799999999</v>
+        <f>Inputs!$C$38*C6/1000</f>
+        <v/>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -4290,12 +4319,12 @@
         </is>
       </c>
       <c r="B8" s="13">
-        <f>Inputs!$B$38*B6/1000</f>
-        <v>31304.59488</v>
+        <f>Inputs!$B$39*B6/1000</f>
+        <v/>
       </c>
       <c r="C8" s="13">
-        <f>Inputs!$C$38*C6/1000</f>
-        <v>31304.59488</v>
+        <f>Inputs!$C$39*C6/1000</f>
+        <v/>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -4394,44 +4423,44 @@
         </is>
       </c>
       <c r="B2" s="4">
-        <f>'1 GW data center'!B28*Inputs!$B$43</f>
-        <v>6018.9588</v>
+        <f>'1 GW data center'!B28*Inputs!$B$44</f>
+        <v/>
       </c>
       <c r="C2" s="4">
-        <f>'1 GW data center'!C28*Inputs!$C$43</f>
-        <v>22250.285999999996</v>
+        <f>'1 GW data center'!C28*Inputs!$C$44</f>
+        <v/>
       </c>
       <c r="D2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$45</f>
-        <v>617.0039459999999</v>
+        <f>'1 GW data center'!B29*Inputs!$B$46</f>
+        <v/>
       </c>
       <c r="E2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$45</f>
-        <v>1342.7044019999998</v>
+        <f>'1 GW data center'!C29*Inputs!$C$46</f>
+        <v/>
       </c>
       <c r="F2" s="4">
         <f>B2-D2</f>
-        <v>5401.9548540000005</v>
+        <v/>
       </c>
       <c r="G2" s="4">
         <f>C2-E2</f>
-        <v>20907.581597999997</v>
+        <v/>
       </c>
       <c r="H2" s="4">
-        <f>'1 GW data center'!B28*Inputs!$B$44-D2</f>
-        <v>720.5424540000002</v>
+        <f>'1 GW data center'!B28*Inputs!$B$45-D2</f>
+        <v/>
       </c>
       <c r="I2" s="4">
-        <f>'1 GW data center'!C28*Inputs!$C$44-E2</f>
-        <v>7310.184598</v>
+        <f>'1 GW data center'!C28*Inputs!$C$45-E2</f>
+        <v/>
       </c>
       <c r="J2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$46</f>
-        <v>1604.2102596</v>
+        <f>'1 GW data center'!B29*Inputs!$B$47</f>
+        <v/>
       </c>
       <c r="K2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$46</f>
-        <v>3491.0314452</v>
+        <f>'1 GW data center'!C29*Inputs!$C$47</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -4441,44 +4470,44 @@
         </is>
       </c>
       <c r="B3" s="4">
-        <f>'1 GW data center'!B33*Inputs!$B$43</f>
-        <v>20700.0</v>
+        <f>'1 GW data center'!B33*Inputs!$B$44</f>
+        <v/>
       </c>
       <c r="C3" s="4">
-        <f>'1 GW data center'!C33*Inputs!$C$43</f>
-        <v>54000.0</v>
+        <f>'1 GW data center'!C33*Inputs!$C$44</f>
+        <v/>
       </c>
       <c r="D3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$45</f>
-        <v>1725.0</v>
+        <f>'1 GW data center'!B34*Inputs!$B$46</f>
+        <v/>
       </c>
       <c r="E3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$45</f>
-        <v>9000.0</v>
+        <f>'1 GW data center'!C34*Inputs!$C$46</f>
+        <v/>
       </c>
       <c r="F3" s="4">
         <f>B3-D3</f>
-        <v>18975.0</v>
+        <v/>
       </c>
       <c r="G3" s="4">
         <f>C3-E3</f>
-        <v>45000.0</v>
+        <v/>
       </c>
       <c r="H3" s="4">
-        <f>'1 GW data center'!B33*Inputs!$B$44-D3</f>
-        <v>2875.0</v>
+        <f>'1 GW data center'!B33*Inputs!$B$45-D3</f>
+        <v/>
       </c>
       <c r="I3" s="4">
-        <f>'1 GW data center'!C33*Inputs!$C$44-E3</f>
-        <v>12000.0</v>
+        <f>'1 GW data center'!C33*Inputs!$C$45-E3</f>
+        <v/>
       </c>
       <c r="J3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$46</f>
-        <v>4485.0</v>
+        <f>'1 GW data center'!B34*Inputs!$B$47</f>
+        <v/>
       </c>
       <c r="K3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$46</f>
-        <v>23400.0</v>
+        <f>'1 GW data center'!C34*Inputs!$C$47</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -4488,44 +4517,44 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>'1 GW data center'!B37*Inputs!$B$43</f>
-        <v>95400.0</v>
+        <f>'1 GW data center'!B37*Inputs!$B$44</f>
+        <v/>
       </c>
       <c r="C4" s="4">
-        <f>'1 GW data center'!C37*Inputs!$C$43</f>
-        <v>194400.0</v>
+        <f>'1 GW data center'!C37*Inputs!$C$44</f>
+        <v/>
       </c>
       <c r="D4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$45</f>
-        <v>7950.0</v>
+        <f>'1 GW data center'!B38*Inputs!$B$46</f>
+        <v/>
       </c>
       <c r="E4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$45</f>
-        <v>32400.0</v>
+        <f>'1 GW data center'!C38*Inputs!$C$46</f>
+        <v/>
       </c>
       <c r="F4" s="4">
         <f>B4-D4</f>
-        <v>87450.0</v>
+        <v/>
       </c>
       <c r="G4" s="4">
         <f>C4-E4</f>
-        <v>162000.0</v>
+        <v/>
       </c>
       <c r="H4" s="4">
-        <f>'1 GW data center'!B37*Inputs!$B$44-D4</f>
-        <v>13250.0</v>
+        <f>'1 GW data center'!B37*Inputs!$B$45-D4</f>
+        <v/>
       </c>
       <c r="I4" s="4">
-        <f>'1 GW data center'!C37*Inputs!$C$44-E4</f>
-        <v>43200.0</v>
+        <f>'1 GW data center'!C37*Inputs!$C$45-E4</f>
+        <v/>
       </c>
       <c r="J4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$46</f>
-        <v>20670.0</v>
+        <f>'1 GW data center'!B38*Inputs!$B$47</f>
+        <v/>
       </c>
       <c r="K4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$46</f>
-        <v>84240.0</v>
+        <f>'1 GW data center'!C38*Inputs!$C$47</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -4535,44 +4564,44 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>'1 GW data center'!B41*Inputs!$B$34</f>
-        <v>119556.0</v>
+        <f>'1 GW data center'!B41*Inputs!$B$35</f>
+        <v/>
       </c>
       <c r="C5" s="4">
-        <f>'1 GW data center'!C41*Inputs!$C$34</f>
-        <v>247320.0</v>
+        <f>'1 GW data center'!C41*Inputs!$C$35</f>
+        <v/>
       </c>
       <c r="D5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$45</f>
-        <v>27945.0</v>
+        <f>'1 GW data center'!B42*Inputs!$B$46</f>
+        <v/>
       </c>
       <c r="E5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$45</f>
-        <v>172800.0</v>
+        <f>'1 GW data center'!C42*Inputs!$C$46</f>
+        <v/>
       </c>
       <c r="F5" s="4">
         <f>B5-D5</f>
-        <v>91611.0</v>
+        <v/>
       </c>
       <c r="G5" s="4">
         <f>C5-E5</f>
-        <v>74520.0</v>
-      </c>
-      <c r="H5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H5" s="4">
         <f>"n/a"</f>
-        <v>n/a</v>
-      </c>
-      <c r="I5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I5" s="4">
         <f>"n/a"</f>
-        <v>n/a</v>
+        <v/>
       </c>
       <c r="J5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$46</f>
-        <v>72657.0</v>
+        <f>'1 GW data center'!B42*Inputs!$B$47</f>
+        <v/>
       </c>
       <c r="K5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$46</f>
-        <v>449280.0</v>
+        <f>'1 GW data center'!C42*Inputs!$C$47</f>
+        <v/>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
DC investor deck: tons instead of kt, "data center" instead of "campus", stable chart rows
Every quantity now prints in tons with thousands separators ('000s of tons on
chart axes) and every "campus" in slide text reads "data center"; ids, asset
names and file paths are unchanged. The slide 5 HTML chart uses fixed column
widths and a constant row height so rows do not shift between the mass and
carbon views. The analyses model scripts, workbook, narrative and chart are
regenerated with the same units and wording; matplotlib PNGs for the PPTX
regenerated too.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -186,7 +186,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>High case, tonnes per campus — replaced by SUPERWOOD vs not (slab concrete row excluded)</a:t>
+              <a:t>High case, tons per data center — replaced by SUPERWOOD vs not (slab concrete row excluded)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -278,7 +278,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>t per campus</a:t>
+                  <a:t>tons per data center</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -633,7 +633,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Reference unit: 1 GW IT-load campus. Change any yellow cell on Inputs (and the four addressable-share columns on 1 GW data center — immediate, soon, medium term, long term; a row may split across them); everything recalculates.</t>
+          <t>Reference unit: 1 GW IT-load data center. Change any yellow cell on Inputs (and the four addressable-share columns on 1 GW data center — immediate, soon, medium term, long term; a row may split across them); everything recalculates.</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IT load of reference campus</t>
+          <t>IT load of reference data center</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -847,7 +847,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Yard / mechanical screens and louvers (per campus)</t>
+          <t>Yard / mechanical screens and louvers (per data center)</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -892,7 +892,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Campus perimeter plus transformer / generator yards</t>
+          <t>Data center perimeter plus transformer / generator yards</t>
         </is>
       </c>
     </row>
@@ -1987,12 +1987,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Low  t per campus</t>
+          <t>Low  tons per data center</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>High  t per campus</t>
+          <t>High  tons per data center</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -3808,14 +3808,14 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>SUMMARY — per campus</t>
+          <t>SUMMARY — per data center</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Total mass, building and contents (t)</t>
+          <t>Total mass, building and contents (tons)</t>
         </is>
       </c>
       <c r="B24" s="8">
@@ -3830,7 +3830,7 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Total excluding concrete (t)</t>
+          <t>Total excluding concrete (tons)</t>
         </is>
       </c>
       <c r="B25" s="8">
@@ -3852,7 +3852,7 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Immediate — incumbent mass replaced (t)</t>
+          <t>Immediate — incumbent mass replaced (tons)</t>
         </is>
       </c>
       <c r="B28" s="10">
@@ -3867,7 +3867,7 @@
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Immediate — SUPERWOOD required (t)</t>
+          <t>Immediate — SUPERWOOD required (tons)</t>
         </is>
       </c>
       <c r="B29" s="10">
@@ -3912,7 +3912,7 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Soon — incumbent mass replaced (t)</t>
+          <t>Soon — incumbent mass replaced (tons)</t>
         </is>
       </c>
       <c r="B33" s="10">
@@ -3927,7 +3927,7 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>Soon — SUPERWOOD required (t)</t>
+          <t>Soon — SUPERWOOD required (tons)</t>
         </is>
       </c>
       <c r="B34" s="10">
@@ -3957,7 +3957,7 @@
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>Medium term — incumbent mass replaced (t)</t>
+          <t>Medium term — incumbent mass replaced (tons)</t>
         </is>
       </c>
       <c r="B37" s="10">
@@ -3972,7 +3972,7 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Medium term — SUPERWOOD required (t)</t>
+          <t>Medium term — SUPERWOOD required (tons)</t>
         </is>
       </c>
       <c r="B38" s="10">
@@ -4002,7 +4002,7 @@
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>Long term — incumbent mass replaced (t)</t>
+          <t>Long term — incumbent mass replaced (tons)</t>
         </is>
       </c>
       <c r="B41" s="10">
@@ -4017,7 +4017,7 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>Long term — SUPERWOOD required (t)</t>
+          <t>Long term — SUPERWOOD required (tons)</t>
         </is>
       </c>
       <c r="B42" s="10">
@@ -4047,7 +4047,7 @@
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Cumulative incumbent mass replaced (t)</t>
+          <t>Cumulative incumbent mass replaced (tons)</t>
         </is>
       </c>
       <c r="B45" s="8">
@@ -4062,7 +4062,7 @@
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Cumulative SUPERWOOD required (t)</t>
+          <t>Cumulative SUPERWOOD required (tons)</t>
         </is>
       </c>
       <c r="B46" s="8">
@@ -4122,7 +4122,7 @@
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>Not replaced by SUPERWOOD (t)</t>
+          <t>Not replaced by SUPERWOOD (tons)</t>
         </is>
       </c>
       <c r="B50" s="8">

</xml_diff>

<commit_message>
DC analyses: workbook carries per-component embodied carbon and the steel-share estimate
The 1 GW data center sheet gains a carbon factor per row (concrete, steel,
mixed; equipment not estimated), low/high embodied carbon per component, and
summary rows for building-materials carbon, steel and concrete shares, the
steel-above-slab share and the recycled-steel sensitivity - the basis of the
slide 5 carbon view. A new Steel share sheet holds the per-component steel
fractions behind the 50-80% above-ground headline. The Carbon sheet now rolls
each horizon up at per-row factors. Narrative regenerated with sections 5b and
5c; README and the steel-share note point at the sheets.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 GW data center" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carbon" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steel share" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -81,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -91,6 +92,8 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,6 +101,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -304,7 +308,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>53</row>
+      <row>62</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9360000" cy="4320000"/>
@@ -614,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -623,7 +627,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>SUPERWOOD × Data Centers — material mass build-up and replacement model (2026-09-01, v2)</t>
+          <t>SUPERWOOD × Data Centers — material mass, embodied carbon and replacement model (2026-09-04, v3)</t>
         </is>
       </c>
     </row>
@@ -673,6 +677,13 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>Embodied carbon: columns X–AB on the main sheet value each row at its own factor (concrete, steel, mixed; equipment not estimated), with totals and steel/concrete shares in the summary; the Carbon sheet rolls avoided emissions up by horizon at those factors and at the recycled-steel (EAF) factor. Steel share: the Steel share sheet estimates what fraction of above-ground mass, contents included, is steel (per-component steel fractions are yellow inputs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Companion narrative: materials-mass-and-replacement.md in the same folder.</t>
         </is>
@@ -689,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1940,6 +1951,34 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Used only for the interior finishes row</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1951,7 +1990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W51"/>
+  <dimension ref="A1:AB60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -1977,6 +2016,11 @@
     <col hidden="1" outlineLevel="1" width="11" customWidth="1" min="21" max="21"/>
     <col hidden="1" outlineLevel="1" width="11" customWidth="1" min="22" max="22"/>
     <col hidden="1" outlineLevel="1" width="11" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2093,6 +2137,31 @@
       <c r="W1" s="1" t="inlineStr">
         <is>
           <t>High SW long</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Carbon factor (kg CO₂e/kg)</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Low embodied carbon (t CO₂e)</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>High embodied carbon (t CO₂e)</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>EAF-basis factor (kg CO₂e/kg)</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Material class</t>
         </is>
       </c>
     </row>
@@ -2212,6 +2281,27 @@
         <f>IF(SUM($F3:$I3)=0,0,M3*I3/SUM($F3:$I3))</f>
         <v/>
       </c>
+      <c r="X3" s="7">
+        <f>Inputs!$B$35</f>
+        <v/>
+      </c>
+      <c r="Y3" s="5">
+        <f>B3*X3</f>
+        <v/>
+      </c>
+      <c r="Z3" s="5">
+        <f>C3*X3</f>
+        <v/>
+      </c>
+      <c r="AA3" s="7">
+        <f>Inputs!$B$35</f>
+        <v/>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>concrete</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2305,6 +2395,27 @@
         <f>IF(SUM($F4:$I4)=0,0,M4*I4/SUM($F4:$I4))</f>
         <v/>
       </c>
+      <c r="X4" s="7">
+        <f>Inputs!$B$35</f>
+        <v/>
+      </c>
+      <c r="Y4" s="5">
+        <f>B4*X4</f>
+        <v/>
+      </c>
+      <c r="Z4" s="5">
+        <f>C4*X4</f>
+        <v/>
+      </c>
+      <c r="AA4" s="7">
+        <f>Inputs!$B$35</f>
+        <v/>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>concrete</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2397,6 +2508,27 @@
         <f>IF(SUM($F5:$I5)=0,0,M5*I5/SUM($F5:$I5))</f>
         <v/>
       </c>
+      <c r="X5" s="7">
+        <f>Inputs!$B$35</f>
+        <v/>
+      </c>
+      <c r="Y5" s="5">
+        <f>B5*X5</f>
+        <v/>
+      </c>
+      <c r="Z5" s="5">
+        <f>C5*X5</f>
+        <v/>
+      </c>
+      <c r="AA5" s="7">
+        <f>Inputs!$B$35</f>
+        <v/>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>concrete</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2490,6 +2622,27 @@
         <f>IF(SUM($F6:$I6)=0,0,M6*I6/SUM($F6:$I6))</f>
         <v/>
       </c>
+      <c r="X6" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y6" s="5">
+        <f>B6*X6</f>
+        <v/>
+      </c>
+      <c r="Z6" s="5">
+        <f>C6*X6</f>
+        <v/>
+      </c>
+      <c r="AA6" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2582,6 +2735,27 @@
         <f>IF(SUM($F7:$I7)=0,0,M7*I7/SUM($F7:$I7))</f>
         <v/>
       </c>
+      <c r="X7" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y7" s="5">
+        <f>B7*X7</f>
+        <v/>
+      </c>
+      <c r="Z7" s="5">
+        <f>C7*X7</f>
+        <v/>
+      </c>
+      <c r="AA7" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2674,6 +2848,27 @@
         <f>IF(SUM($F8:$I8)=0,0,M8*I8/SUM($F8:$I8))</f>
         <v/>
       </c>
+      <c r="X8" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y8" s="5">
+        <f>B8*X8</f>
+        <v/>
+      </c>
+      <c r="Z8" s="5">
+        <f>C8*X8</f>
+        <v/>
+      </c>
+      <c r="AA8" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2766,6 +2961,27 @@
         <f>IF(SUM($F9:$I9)=0,0,M9*I9/SUM($F9:$I9))</f>
         <v/>
       </c>
+      <c r="X9" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y9" s="5">
+        <f>B9*X9</f>
+        <v/>
+      </c>
+      <c r="Z9" s="5">
+        <f>C9*X9</f>
+        <v/>
+      </c>
+      <c r="AA9" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2858,6 +3074,27 @@
         <f>IF(SUM($F10:$I10)=0,0,M10*I10/SUM($F10:$I10))</f>
         <v/>
       </c>
+      <c r="X10" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y10" s="5">
+        <f>B10*X10</f>
+        <v/>
+      </c>
+      <c r="Z10" s="5">
+        <f>C10*X10</f>
+        <v/>
+      </c>
+      <c r="AA10" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2949,6 +3186,27 @@
       <c r="W11" s="5">
         <f>IF(SUM($F11:$I11)=0,0,M11*I11/SUM($F11:$I11))</f>
         <v/>
+      </c>
+      <c r="X11" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y11" s="5">
+        <f>B11*X11</f>
+        <v/>
+      </c>
+      <c r="Z11" s="5">
+        <f>C11*X11</f>
+        <v/>
+      </c>
+      <c r="AA11" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -2974,6 +3232,10 @@
       <c r="U12" s="4" t="n"/>
       <c r="V12" s="4" t="n"/>
       <c r="W12" s="4" t="n"/>
+      <c r="X12" s="8" t="n"/>
+      <c r="Y12" s="4" t="n"/>
+      <c r="Z12" s="4" t="n"/>
+      <c r="AA12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3066,6 +3328,27 @@
         <f>IF(SUM($F13:$I13)=0,0,M13*I13/SUM($F13:$I13))</f>
         <v/>
       </c>
+      <c r="X13" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y13" s="5">
+        <f>B13*X13</f>
+        <v/>
+      </c>
+      <c r="Z13" s="5">
+        <f>C13*X13</f>
+        <v/>
+      </c>
+      <c r="AA13" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3158,6 +3441,27 @@
         <f>IF(SUM($F14:$I14)=0,0,M14*I14/SUM($F14:$I14))</f>
         <v/>
       </c>
+      <c r="X14" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y14" s="5">
+        <f>B14*X14</f>
+        <v/>
+      </c>
+      <c r="Z14" s="5">
+        <f>C14*X14</f>
+        <v/>
+      </c>
+      <c r="AA14" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3250,6 +3554,27 @@
         <f>IF(SUM($F15:$I15)=0,0,M15*I15/SUM($F15:$I15))</f>
         <v/>
       </c>
+      <c r="X15" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y15" s="5">
+        <f>B15*X15</f>
+        <v/>
+      </c>
+      <c r="Z15" s="5">
+        <f>C15*X15</f>
+        <v/>
+      </c>
+      <c r="AA15" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3343,6 +3668,27 @@
         <f>IF(SUM($F16:$I16)=0,0,M16*I16/SUM($F16:$I16))</f>
         <v/>
       </c>
+      <c r="X16" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y16" s="5">
+        <f>B16*X16</f>
+        <v/>
+      </c>
+      <c r="Z16" s="5">
+        <f>C16*X16</f>
+        <v/>
+      </c>
+      <c r="AA16" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3435,6 +3781,27 @@
         <f>IF(SUM($F17:$I17)=0,0,M17*I17/SUM($F17:$I17))</f>
         <v/>
       </c>
+      <c r="X17" s="7">
+        <f>Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y17" s="5">
+        <f>B17*X17</f>
+        <v/>
+      </c>
+      <c r="Z17" s="5">
+        <f>C17*X17</f>
+        <v/>
+      </c>
+      <c r="AA17" s="7">
+        <f>Inputs!$C$45</f>
+        <v/>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3527,6 +3894,27 @@
         <f>IF(SUM($F18:$I18)=0,0,M18*I18/SUM($F18:$I18))</f>
         <v/>
       </c>
+      <c r="X18" s="7">
+        <f>Inputs!$B$48</f>
+        <v/>
+      </c>
+      <c r="Y18" s="5">
+        <f>B18*X18</f>
+        <v/>
+      </c>
+      <c r="Z18" s="5">
+        <f>C18*X18</f>
+        <v/>
+      </c>
+      <c r="AA18" s="7">
+        <f>Inputs!$B$48</f>
+        <v/>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3619,6 +4007,25 @@
         <f>IF(SUM($F19:$I19)=0,0,M19*I19/SUM($F19:$I19))</f>
         <v/>
       </c>
+      <c r="X19" s="8" t="inlineStr">
+        <is>
+          <t>not estimated</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3711,6 +4118,25 @@
         <f>IF(SUM($F20:$I20)=0,0,M20*I20/SUM($F20:$I20))</f>
         <v/>
       </c>
+      <c r="X20" s="8" t="inlineStr">
+        <is>
+          <t>not estimated</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3804,6 +4230,25 @@
         <f>IF(SUM($F21:$I21)=0,0,M21*I21/SUM($F21:$I21))</f>
         <v/>
       </c>
+      <c r="X21" s="8" t="inlineStr">
+        <is>
+          <t>not estimated</t>
+        </is>
+      </c>
+      <c r="Y21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -3813,339 +4258,451 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Total mass, building and contents (tons)</t>
         </is>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="10">
         <f>SUM(B3:B21)</f>
         <v/>
       </c>
-      <c r="C24" s="8">
+      <c r="C24" s="10">
         <f>SUM(C3:C21)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Total excluding concrete (tons)</t>
         </is>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="10">
         <f>B24-B3-B4-B5</f>
         <v/>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="10">
         <f>C24-C3-C4-C5</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Replaced by SUPERWOOD, by horizon</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>Immediate — incumbent mass replaced (tons)</t>
         </is>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="12">
         <f>SUMPRODUCT(B3:B21,F3:F21)</f>
         <v/>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="12">
         <f>SUMPRODUCT(C3:C21,F3:F21)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Immediate — SUPERWOOD required (tons)</t>
         </is>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="12">
         <f>SUM(P3:P21)</f>
         <v/>
       </c>
-      <c r="C29" s="10">
+      <c r="C29" s="12">
         <f>SUM(T3:T21)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>Immediate — SUPERWOOD required (sf)</t>
         </is>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="12">
         <f>B29*1000/Derived!B6</f>
         <v/>
       </c>
-      <c r="C30" s="10">
+      <c r="C30" s="12">
         <f>C29*1000/Derived!C6</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Immediate — years of SuperMill One output</t>
         </is>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="13">
         <f>B29/Derived!B7</f>
         <v/>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="13">
         <f>C29/Derived!C7</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>Soon — incumbent mass replaced (tons)</t>
         </is>
       </c>
-      <c r="B33" s="10">
+      <c r="B33" s="12">
         <f>SUMPRODUCT(B3:B21,G3:G21)</f>
         <v/>
       </c>
-      <c r="C33" s="10">
+      <c r="C33" s="12">
         <f>SUMPRODUCT(C3:C21,G3:G21)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>Soon — SUPERWOOD required (tons)</t>
         </is>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="12">
         <f>SUM(Q3:Q21)</f>
         <v/>
       </c>
-      <c r="C34" s="10">
+      <c r="C34" s="12">
         <f>SUM(U3:U21)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>Soon — years of SuperMill Two output</t>
         </is>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="13">
         <f>B34/Derived!B8</f>
         <v/>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="13">
         <f>C34/Derived!C8</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>Medium term — incumbent mass replaced (tons)</t>
         </is>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="12">
         <f>SUMPRODUCT(B3:B21,H3:H21)</f>
         <v/>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="12">
         <f>SUMPRODUCT(C3:C21,H3:H21)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="inlineStr">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>Medium term — SUPERWOOD required (tons)</t>
         </is>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="12">
         <f>SUM(R3:R21)</f>
         <v/>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="12">
         <f>SUM(V3:V21)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Medium term — years of SuperMill Two output</t>
         </is>
       </c>
-      <c r="B39" s="11">
+      <c r="B39" s="13">
         <f>B38/Derived!B8</f>
         <v/>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="13">
         <f>C38/Derived!C8</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="9" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>Long term — incumbent mass replaced (tons)</t>
         </is>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="12">
         <f>SUMPRODUCT(B3:B21,I3:I21)</f>
         <v/>
       </c>
-      <c r="C41" s="10">
+      <c r="C41" s="12">
         <f>SUMPRODUCT(C3:C21,I3:I21)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>Long term — SUPERWOOD required (tons)</t>
         </is>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="12">
         <f>SUM(S3:S21)</f>
         <v/>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="12">
         <f>SUM(W3:W21)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="9" t="inlineStr">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>Long term — years of SuperMill Two output</t>
         </is>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="13">
         <f>B42/Derived!B8</f>
         <v/>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="13">
         <f>C42/Derived!C8</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>Cumulative incumbent mass replaced (tons)</t>
         </is>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="10">
         <f>SUM(J3:J21)</f>
         <v/>
       </c>
-      <c r="C45" s="8">
+      <c r="C45" s="10">
         <f>SUM(K3:K21)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>Cumulative SUPERWOOD required (tons)</t>
         </is>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="10">
         <f>SUM(L3:L21)</f>
         <v/>
       </c>
-      <c r="C46" s="8">
+      <c r="C46" s="10">
         <f>SUM(M3:M21)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="inlineStr">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>Cumulative years of SuperMill Two output</t>
         </is>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="13">
         <f>B46/Derived!B8</f>
         <v/>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="13">
         <f>C46/Derived!C8</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="inlineStr">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>Share of total mass replaced</t>
         </is>
       </c>
-      <c r="B48" s="12">
+      <c r="B48" s="14">
         <f>B45/B24</f>
         <v/>
       </c>
-      <c r="C48" s="12">
+      <c r="C48" s="14">
         <f>C45/C24</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="9" t="inlineStr">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Share of ex-concrete mass replaced through the medium term (excludes foundations)</t>
         </is>
       </c>
-      <c r="B49" s="12">
+      <c r="B49" s="14">
         <f>(B45-B41)/B25</f>
         <v/>
       </c>
-      <c r="C49" s="12">
+      <c r="C49" s="14">
         <f>(C45-C41)/C25</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
+      <c r="A50" s="9" t="inlineStr">
         <is>
           <t>Not replaced by SUPERWOOD (tons)</t>
         </is>
       </c>
-      <c r="B50" s="8">
+      <c r="B50" s="10">
         <f>B24-B45</f>
         <v/>
       </c>
-      <c r="C50" s="8">
+      <c r="C50" s="10">
         <f>C24-C45</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Not replaced, share of total</t>
         </is>
       </c>
-      <c r="B51" s="12">
+      <c r="B51" s="14">
         <f>B50/B24</f>
         <v/>
       </c>
-      <c r="C51" s="12">
+      <c r="C51" s="14">
         <f>C50/C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>EMBODIED CARBON — building materials (equipment not estimated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>Embodied carbon, building materials (t CO₂e)</t>
+        </is>
+      </c>
+      <c r="B54" s="10">
+        <f>SUM(Y3:Y21)</f>
+        <v/>
+      </c>
+      <c r="C54" s="10">
+        <f>SUM(Z3:Z21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which steel (t CO₂e)</t>
+        </is>
+      </c>
+      <c r="B55" s="12">
+        <f>SUMIF(AB3:AB21,"steel",Y3:Y21)</f>
+        <v/>
+      </c>
+      <c r="C55" s="12">
+        <f>SUMIF(AB3:AB21,"steel",Z3:Z21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which concrete (t CO₂e)</t>
+        </is>
+      </c>
+      <c r="B56" s="12">
+        <f>SUMIF(AB3:AB21,"concrete",Y3:Y21)</f>
+        <v/>
+      </c>
+      <c r="C56" s="12">
+        <f>SUMIF(AB3:AB21,"concrete",Z3:Z21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>Steel share of building-materials carbon</t>
+        </is>
+      </c>
+      <c r="B57" s="14">
+        <f>B55/B54</f>
+        <v/>
+      </c>
+      <c r="C57" s="14">
+        <f>C55/C54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>Concrete share of building-materials carbon</t>
+        </is>
+      </c>
+      <c r="B58" s="14">
+        <f>B56/B54</f>
+        <v/>
+      </c>
+      <c r="C58" s="14">
+        <f>C56/C54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>Steel above the slab (steel excl. rebar), share of building-materials carbon</t>
+        </is>
+      </c>
+      <c r="B59" s="14">
+        <f>(B55-Y6)/B54</f>
+        <v/>
+      </c>
+      <c r="C59" s="14">
+        <f>(C55-Z6)/C54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>Steel share if steel is recycled (EAF factor, high end)</t>
+        </is>
+      </c>
+      <c r="B60" s="14">
+        <f>SUMPRODUCT(B3:B21,AA3:AA21,--(AB3:AB21="steel"))/SUMPRODUCT(B3:B21,AA3:AA21)</f>
+        <v/>
+      </c>
+      <c r="C60" s="14">
+        <f>SUMPRODUCT(C3:C21,AA3:AA21,--(AB3:AB21="steel"))/SUMPRODUCT(C3:C21,AA3:AA21)</f>
         <v/>
       </c>
     </row>
@@ -4198,11 +4755,11 @@
           <t>Number of buildings</t>
         </is>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <f>Inputs!$B$3*Inputs!$B$2/Inputs!$B$4</f>
         <v/>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="15">
         <f>Inputs!$C$3*Inputs!$C$2/Inputs!$C$4</f>
         <v/>
       </c>
@@ -4218,11 +4775,11 @@
           <t>Exterior wall area, sf</t>
         </is>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <f>B2*Inputs!$B$5</f>
         <v/>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="15">
         <f>C2*Inputs!$C$5</f>
         <v/>
       </c>
@@ -4238,11 +4795,11 @@
           <t>Exterior wall area, m²</t>
         </is>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <f>B3*0.092903</f>
         <v/>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="15">
         <f>C3*0.092903</f>
         <v/>
       </c>
@@ -4258,11 +4815,11 @@
           <t>Fence face area, sf</t>
         </is>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="15">
         <f>Inputs!$B$7*1000*Inputs!$B$8/0.092903</f>
         <v/>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="15">
         <f>Inputs!$C$7*1000*Inputs!$C$8/0.092903</f>
         <v/>
       </c>
@@ -4278,11 +4835,11 @@
           <t>SUPERWOOD board mass per sf</t>
         </is>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="15">
         <f>Inputs!$B$36/1000*Inputs!$B$37*0.092903</f>
         <v/>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="15">
         <f>Inputs!$C$36/1000*Inputs!$C$37*0.092903</f>
         <v/>
       </c>
@@ -4298,11 +4855,11 @@
           <t>SuperMill One output in tonnes</t>
         </is>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="15">
         <f>Inputs!$B$38*B6/1000</f>
         <v/>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="15">
         <f>Inputs!$C$38*C6/1000</f>
         <v/>
       </c>
@@ -4318,11 +4875,11 @@
           <t>SuperMill Two output in tonnes</t>
         </is>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="15">
         <f>Inputs!$B$39*B6/1000</f>
         <v/>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="15">
         <f>Inputs!$C$39*C6/1000</f>
         <v/>
       </c>
@@ -4423,11 +4980,11 @@
         </is>
       </c>
       <c r="B2" s="4">
-        <f>'1 GW data center'!B28*Inputs!$B$44</f>
+        <f>SUMPRODUCT('1 GW data center'!B3:B21,'1 GW data center'!F3:F21,'1 GW data center'!X3:X21)</f>
         <v/>
       </c>
       <c r="C2" s="4">
-        <f>'1 GW data center'!C28*Inputs!$C$44</f>
+        <f>SUMPRODUCT('1 GW data center'!C3:C21,'1 GW data center'!F3:F21,'1 GW data center'!X3:X21)</f>
         <v/>
       </c>
       <c r="D2" s="4">
@@ -4447,11 +5004,11 @@
         <v/>
       </c>
       <c r="H2" s="4">
-        <f>'1 GW data center'!B28*Inputs!$B$45-D2</f>
+        <f>SUMPRODUCT('1 GW data center'!B3:B21,'1 GW data center'!F3:F21,'1 GW data center'!AA3:AA21)-D2</f>
         <v/>
       </c>
       <c r="I2" s="4">
-        <f>'1 GW data center'!C28*Inputs!$C$45-E2</f>
+        <f>SUMPRODUCT('1 GW data center'!C3:C21,'1 GW data center'!F3:F21,'1 GW data center'!AA3:AA21)-E2</f>
         <v/>
       </c>
       <c r="J2" s="4">
@@ -4470,11 +5027,11 @@
         </is>
       </c>
       <c r="B3" s="4">
-        <f>'1 GW data center'!B33*Inputs!$B$44</f>
+        <f>SUMPRODUCT('1 GW data center'!B3:B21,'1 GW data center'!G3:G21,'1 GW data center'!X3:X21)</f>
         <v/>
       </c>
       <c r="C3" s="4">
-        <f>'1 GW data center'!C33*Inputs!$C$44</f>
+        <f>SUMPRODUCT('1 GW data center'!C3:C21,'1 GW data center'!G3:G21,'1 GW data center'!X3:X21)</f>
         <v/>
       </c>
       <c r="D3" s="4">
@@ -4494,11 +5051,11 @@
         <v/>
       </c>
       <c r="H3" s="4">
-        <f>'1 GW data center'!B33*Inputs!$B$45-D3</f>
+        <f>SUMPRODUCT('1 GW data center'!B3:B21,'1 GW data center'!G3:G21,'1 GW data center'!AA3:AA21)-D3</f>
         <v/>
       </c>
       <c r="I3" s="4">
-        <f>'1 GW data center'!C33*Inputs!$C$45-E3</f>
+        <f>SUMPRODUCT('1 GW data center'!C3:C21,'1 GW data center'!G3:G21,'1 GW data center'!AA3:AA21)-E3</f>
         <v/>
       </c>
       <c r="J3" s="4">
@@ -4517,11 +5074,11 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>'1 GW data center'!B37*Inputs!$B$44</f>
+        <f>SUMPRODUCT('1 GW data center'!B3:B21,'1 GW data center'!H3:H21,'1 GW data center'!X3:X21)</f>
         <v/>
       </c>
       <c r="C4" s="4">
-        <f>'1 GW data center'!C37*Inputs!$C$44</f>
+        <f>SUMPRODUCT('1 GW data center'!C3:C21,'1 GW data center'!H3:H21,'1 GW data center'!X3:X21)</f>
         <v/>
       </c>
       <c r="D4" s="4">
@@ -4541,11 +5098,11 @@
         <v/>
       </c>
       <c r="H4" s="4">
-        <f>'1 GW data center'!B37*Inputs!$B$45-D4</f>
+        <f>SUMPRODUCT('1 GW data center'!B3:B21,'1 GW data center'!H3:H21,'1 GW data center'!AA3:AA21)-D4</f>
         <v/>
       </c>
       <c r="I4" s="4">
-        <f>'1 GW data center'!C37*Inputs!$C$45-E4</f>
+        <f>SUMPRODUCT('1 GW data center'!C3:C21,'1 GW data center'!H3:H21,'1 GW data center'!AA3:AA21)-E4</f>
         <v/>
       </c>
       <c r="J4" s="4">
@@ -4560,15 +5117,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Long term (foundation concrete)</t>
+          <t>Long term (concrete, rebar, server enclosures)</t>
         </is>
       </c>
       <c r="B5" s="4">
-        <f>'1 GW data center'!B41*Inputs!$B$35</f>
+        <f>SUMPRODUCT('1 GW data center'!B3:B21,'1 GW data center'!I3:I21,'1 GW data center'!X3:X21)</f>
         <v/>
       </c>
       <c r="C5" s="4">
-        <f>'1 GW data center'!C41*Inputs!$C$35</f>
+        <f>SUMPRODUCT('1 GW data center'!C3:C21,'1 GW data center'!I3:I21,'1 GW data center'!X3:X21)</f>
         <v/>
       </c>
       <c r="D5" s="4">
@@ -4588,11 +5145,11 @@
         <v/>
       </c>
       <c r="H5" s="4">
-        <f>"n/a"</f>
+        <f>SUMPRODUCT('1 GW data center'!B3:B21,'1 GW data center'!I3:I21,'1 GW data center'!AA3:AA21)-D5</f>
         <v/>
       </c>
       <c r="I5" s="4">
-        <f>"n/a"</f>
+        <f>SUMPRODUCT('1 GW data center'!C3:C21,'1 GW data center'!I3:I21,'1 GW data center'!AA3:AA21)-E5</f>
         <v/>
       </c>
       <c r="J5" s="4">
@@ -4607,7 +5164,635 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pre-LCA projections (LCA under way with Prof. Ming Hu, University of Notre Dame). Long-term row uses a concrete factor (Inputs co2_conc) and treats the rebar in foundations at the concrete factor — conservative. Biogenic storage reported separately (EN 15804 module C).</t>
+          <t>Pre-LCA projections (LCA under way with Prof. Ming Hu, University of Notre Dame). Each row is valued at its own factor (column X on the main sheet): concrete rows at co2_conc, steel rows including rebar at co2_steel, interior finishes at co2_mixed; equipment rows (including the long-term server enclosures) carry no factor, so the long-term row counts concrete and rebar only. The EAF column revalues steel rows at the recycled-steel factor (high end). Equipment rows carry no factor. Biogenic storage reported separately (EN 15804 module C).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="64" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Above-ground component (contents included)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Low tons</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>High tons</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steel fraction — low</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Steel fraction — high</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Low steel tons</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>High steel tons</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Basis for the fraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Structural steel — primary frame (columns, girders)</t>
+        </is>
+      </c>
+      <c r="B2" s="5">
+        <f>'1 GW data center'!B7</f>
+        <v/>
+      </c>
+      <c r="C2" s="5">
+        <f>'1 GW data center'!C7</f>
+        <v/>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="5">
+        <f>B2*D2</f>
+        <v/>
+      </c>
+      <c r="G2" s="5">
+        <f>C2*E2</f>
+        <v/>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>steel by definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Structural steel — roof trusses, joists, roof deck, girts</t>
+        </is>
+      </c>
+      <c r="B3" s="5">
+        <f>'1 GW data center'!B8</f>
+        <v/>
+      </c>
+      <c r="C3" s="5">
+        <f>'1 GW data center'!C8</f>
+        <v/>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="5">
+        <f>B3*D3</f>
+        <v/>
+      </c>
+      <c r="G3" s="5">
+        <f>C3*E3</f>
+        <v/>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>steel by definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Exterior skins — metal panel / IMP (metal-panel case)</t>
+        </is>
+      </c>
+      <c r="B4" s="5">
+        <f>'1 GW data center'!B9</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>'1 GW data center'!C9</f>
+        <v/>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F4" s="5">
+        <f>B4*D4</f>
+        <v/>
+      </c>
+      <c r="G4" s="5">
+        <f>C4*E4</f>
+        <v/>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>steel-faced IMP; some aluminum</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Louvers and yard / mechanical screens</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>'1 GW data center'!B10</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>'1 GW data center'!C10</f>
+        <v/>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F5" s="5">
+        <f>B5*D5</f>
+        <v/>
+      </c>
+      <c r="G5" s="5">
+        <f>C5*E5</f>
+        <v/>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>aluminum common</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Security and staff-area fencing</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>'1 GW data center'!B11</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>'1 GW data center'!C11</f>
+        <v/>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5">
+        <f>B6*D6</f>
+        <v/>
+      </c>
+      <c r="G6" s="5">
+        <f>C6*E6</f>
+        <v/>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>chain-link, palisade, posts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Platforms, walkways, mezzanines, railings, tray supports</t>
+        </is>
+      </c>
+      <c r="B7" s="5">
+        <f>'1 GW data center'!B13</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>'1 GW data center'!C13</f>
+        <v/>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5">
+        <f>B7*D7</f>
+        <v/>
+      </c>
+      <c r="G7" s="5">
+        <f>C7*E7</f>
+        <v/>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>structural and misc. steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Acoustic barriers, enclosures, HVAC separations</t>
+        </is>
+      </c>
+      <c r="B8" s="5">
+        <f>'1 GW data center'!B14</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>'1 GW data center'!C14</f>
+        <v/>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F8" s="5">
+        <f>B8*D8</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>C8*E8</f>
+        <v/>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>steel panels with absorptive fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Racking and equipment supports</t>
+        </is>
+      </c>
+      <c r="B9" s="5">
+        <f>'1 GW data center'!B15</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>'1 GW data center'!C15</f>
+        <v/>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5">
+        <f>B9*D9</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>C9*E9</f>
+        <v/>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Other tray, containment, doors, misc. metals</t>
+        </is>
+      </c>
+      <c r="B10" s="5">
+        <f>'1 GW data center'!B16</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>'1 GW data center'!C16</f>
+        <v/>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F10" s="5">
+        <f>B10*D10</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>C10*E10</f>
+        <v/>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>mostly steel, some aluminum</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ducting, plenums and air-distribution sheet metal</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>'1 GW data center'!B17</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>'1 GW data center'!C17</f>
+        <v/>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="5">
+        <f>B11*D11</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>C11*E11</f>
+        <v/>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>galvanized steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Interior finishes, backplanes, trim (admin / office)</t>
+        </is>
+      </c>
+      <c r="B12" s="5">
+        <f>'1 GW data center'!B18</f>
+        <v/>
+      </c>
+      <c r="C12" s="5">
+        <f>'1 GW data center'!C18</f>
+        <v/>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F12" s="5">
+        <f>B12*D12</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>C12*E12</f>
+        <v/>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>gypsum, wood, steel studs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Electrical equipment and conductors</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>'1 GW data center'!B19</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>'1 GW data center'!C19</f>
+        <v/>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F13" s="5">
+        <f>B13*D13</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>C13*E13</f>
+        <v/>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>enclosures, cores, gensets, switchgear; rest copper, oil, batteries</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Mechanical equipment, piping, loop water</t>
+        </is>
+      </c>
+      <c r="B14" s="5">
+        <f>'1 GW data center'!B20</f>
+        <v/>
+      </c>
+      <c r="C14" s="5">
+        <f>'1 GW data center'!C20</f>
+        <v/>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F14" s="5">
+        <f>B14*D14</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>C14*E14</f>
+        <v/>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>chillers, piping steel; water, copper, refrigerant not</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>IT — servers and racks</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>'1 GW data center'!B21</f>
+        <v/>
+      </c>
+      <c r="C15" s="5">
+        <f>'1 GW data center'!C21</f>
+        <v/>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F15" s="5">
+        <f>B15*D15</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>C15*E15</f>
+        <v/>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>steel chassis and racks; aluminum, PCBs, copper</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Above-ground mass, contents included (tons)</t>
+        </is>
+      </c>
+      <c r="B17" s="4">
+        <f>SUM(B2:B15)</f>
+        <v/>
+      </c>
+      <c r="C17" s="4">
+        <f>SUM(C2:C15)</f>
+        <v/>
+      </c>
+      <c r="F17" s="4" t="n"/>
+      <c r="G17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Steel in it (tons)</t>
+        </is>
+      </c>
+      <c r="B18" s="4">
+        <f>SUM(F2:F15)</f>
+        <v/>
+      </c>
+      <c r="C18" s="4">
+        <f>SUM(G2:G15)</f>
+        <v/>
+      </c>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Steel share of above-ground mass</t>
+        </is>
+      </c>
+      <c r="B19" s="16">
+        <f>B18/B17</f>
+        <v/>
+      </c>
+      <c r="C19" s="16">
+        <f>C18/C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Steel share including slab rebar (at-grade steel)</t>
+        </is>
+      </c>
+      <c r="B20" s="16">
+        <f>(B18+'1 GW data center'!B6)/(B17+'1 GW data center'!B6)</f>
+        <v/>
+      </c>
+      <c r="C20" s="16">
+        <f>(C18+'1 GW data center'!C6)/(C17+'1 GW data center'!C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Structure and envelope only (first five rows)</t>
+        </is>
+      </c>
+      <c r="B21" s="16">
+        <f>SUM(F2:F6)/SUM(B2:B6)</f>
+        <v/>
+      </c>
+      <c r="C21" s="16">
+        <f>SUM(G2:G6)/SUM(C2:C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Excludes slab on grade, paving, foundations and all concrete. Steel fractions per component are estimates [conf: L] (yellow cells). Printed band on the deck: 50–80% (Alex, 2026-09-04). Precast/tilt-up walls would add above-ground concrete and lower the share sharply.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DC analyses: wall system as a factor in the steel share; slide 5 note says the band covers both
The Steel share sheet now includes the precast/tilt-up wall row (rebar
fraction 3-5%), follows the Inputs walls_precast toggle, and adds two forced
cases: metal-panel walls (69-79% steel above ground) and tilt-up/precast walls
(56-66%). Narrative, steel-share note and register updated; slide 5 footnote
states that the printed 50-80% band covers both wall systems.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -82,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -102,6 +102,7 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5179,7 +5180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -5237,22 +5238,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Structural steel — primary frame (columns, girders)</t>
+          <t>Precast / tilt-up perimeter walls (precast case)</t>
         </is>
       </c>
       <c r="B2" s="5">
-        <f>'1 GW data center'!B7</f>
+        <f>'1 GW data center'!B5</f>
         <v/>
       </c>
       <c r="C2" s="5">
-        <f>'1 GW data center'!C7</f>
+        <f>'1 GW data center'!C5</f>
         <v/>
       </c>
       <c r="D2" s="6" t="n">
-        <v>1</v>
+        <v>0.03</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="F2" s="5">
         <f>B2*D2</f>
@@ -5264,22 +5265,22 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>steel by definition</t>
+          <t>rebar in precast/tilt-up panels; row is zero unless Inputs walls_precast = 1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Structural steel — roof trusses, joists, roof deck, girts</t>
+          <t>Structural steel — primary frame (columns, girders)</t>
         </is>
       </c>
       <c r="B3" s="5">
-        <f>'1 GW data center'!B8</f>
+        <f>'1 GW data center'!B7</f>
         <v/>
       </c>
       <c r="C3" s="5">
-        <f>'1 GW data center'!C8</f>
+        <f>'1 GW data center'!C7</f>
         <v/>
       </c>
       <c r="D3" s="6" t="n">
@@ -5305,22 +5306,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Exterior skins — metal panel / IMP (metal-panel case)</t>
+          <t>Structural steel — roof trusses, joists, roof deck, girts</t>
         </is>
       </c>
       <c r="B4" s="5">
-        <f>'1 GW data center'!B9</f>
+        <f>'1 GW data center'!B8</f>
         <v/>
       </c>
       <c r="C4" s="5">
-        <f>'1 GW data center'!C9</f>
+        <f>'1 GW data center'!C8</f>
         <v/>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F4" s="5">
         <f>B4*D4</f>
@@ -5332,29 +5333,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>steel-faced IMP; some aluminum</t>
+          <t>steel by definition</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Louvers and yard / mechanical screens</t>
+          <t>Exterior skins — metal panel / IMP (metal-panel case)</t>
         </is>
       </c>
       <c r="B5" s="5">
-        <f>'1 GW data center'!B10</f>
+        <f>'1 GW data center'!B9</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>'1 GW data center'!C10</f>
+        <f>'1 GW data center'!C9</f>
         <v/>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.4</v>
+        <v>0.85</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="F5" s="5">
         <f>B5*D5</f>
@@ -5366,29 +5367,29 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>aluminum common</t>
+          <t>steel-faced IMP; some aluminum</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Security and staff-area fencing</t>
+          <t>Louvers and yard / mechanical screens</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>'1 GW data center'!B11</f>
+        <f>'1 GW data center'!B10</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>'1 GW data center'!C11</f>
+        <f>'1 GW data center'!C10</f>
         <v/>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="F6" s="5">
         <f>B6*D6</f>
@@ -5400,26 +5401,26 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>chain-link, palisade, posts</t>
+          <t>aluminum common</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Platforms, walkways, mezzanines, railings, tray supports</t>
+          <t>Security and staff-area fencing</t>
         </is>
       </c>
       <c r="B7" s="5">
-        <f>'1 GW data center'!B13</f>
+        <f>'1 GW data center'!B11</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>'1 GW data center'!C13</f>
+        <f>'1 GW data center'!C11</f>
         <v/>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>1</v>
@@ -5434,29 +5435,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>structural and misc. steel</t>
+          <t>chain-link, palisade, posts</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Acoustic barriers, enclosures, HVAC separations</t>
+          <t>Platforms, walkways, mezzanines, railings, tray supports</t>
         </is>
       </c>
       <c r="B8" s="5">
-        <f>'1 GW data center'!B14</f>
+        <f>'1 GW data center'!B13</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>'1 GW data center'!C14</f>
+        <f>'1 GW data center'!C13</f>
         <v/>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.7</v>
+        <v>0.95</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F8" s="5">
         <f>B8*D8</f>
@@ -5468,29 +5469,29 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>steel panels with absorptive fill</t>
+          <t>structural and misc. steel</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Racking and equipment supports</t>
+          <t>Acoustic barriers, enclosures, HVAC separations</t>
         </is>
       </c>
       <c r="B9" s="5">
-        <f>'1 GW data center'!B15</f>
+        <f>'1 GW data center'!B14</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>'1 GW data center'!C15</f>
+        <f>'1 GW data center'!C14</f>
         <v/>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.95</v>
+        <v>0.7</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F9" s="5">
         <f>B9*D9</f>
@@ -5502,29 +5503,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>steel panels with absorptive fill</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Other tray, containment, doors, misc. metals</t>
+          <t>Racking and equipment supports</t>
         </is>
       </c>
       <c r="B10" s="5">
-        <f>'1 GW data center'!B16</f>
+        <f>'1 GW data center'!B15</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>'1 GW data center'!C16</f>
+        <f>'1 GW data center'!C15</f>
         <v/>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F10" s="5">
         <f>B10*D10</f>
@@ -5536,29 +5537,29 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>mostly steel, some aluminum</t>
+          <t>steel</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ducting, plenums and air-distribution sheet metal</t>
+          <t>Other tray, containment, doors, misc. metals</t>
         </is>
       </c>
       <c r="B11" s="5">
-        <f>'1 GW data center'!B17</f>
+        <f>'1 GW data center'!B16</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>'1 GW data center'!C17</f>
+        <f>'1 GW data center'!C16</f>
         <v/>
       </c>
       <c r="D11" s="6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E11" s="6" t="n">
         <v>0.95</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>1</v>
       </c>
       <c r="F11" s="5">
         <f>B11*D11</f>
@@ -5570,29 +5571,29 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>galvanized steel</t>
+          <t>mostly steel, some aluminum</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Interior finishes, backplanes, trim (admin / office)</t>
+          <t>Ducting, plenums and air-distribution sheet metal</t>
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'1 GW data center'!B18</f>
+        <f>'1 GW data center'!B17</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>'1 GW data center'!C18</f>
+        <f>'1 GW data center'!C17</f>
         <v/>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0.2</v>
+        <v>0.95</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="F12" s="5">
         <f>B12*D12</f>
@@ -5604,29 +5605,29 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>gypsum, wood, steel studs</t>
+          <t>galvanized steel</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Electrical equipment and conductors</t>
+          <t>Interior finishes, backplanes, trim (admin / office)</t>
         </is>
       </c>
       <c r="B13" s="5">
-        <f>'1 GW data center'!B19</f>
+        <f>'1 GW data center'!B18</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>'1 GW data center'!C19</f>
+        <f>'1 GW data center'!C18</f>
         <v/>
       </c>
       <c r="D13" s="6" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.65</v>
+        <v>0.4</v>
       </c>
       <c r="F13" s="5">
         <f>B13*D13</f>
@@ -5638,26 +5639,26 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>enclosures, cores, gensets, switchgear; rest copper, oil, batteries</t>
+          <t>gypsum, wood, steel studs</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mechanical equipment, piping, loop water</t>
+          <t>Electrical equipment and conductors</t>
         </is>
       </c>
       <c r="B14" s="5">
-        <f>'1 GW data center'!B20</f>
+        <f>'1 GW data center'!B19</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>'1 GW data center'!C20</f>
+        <f>'1 GW data center'!C19</f>
         <v/>
       </c>
       <c r="D14" s="6" t="n">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>0.65</v>
@@ -5672,29 +5673,29 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>chillers, piping steel; water, copper, refrigerant not</t>
+          <t>enclosures, cores, gensets, switchgear; rest copper, oil, batteries</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT — servers and racks</t>
+          <t>Mechanical equipment, piping, loop water</t>
         </is>
       </c>
       <c r="B15" s="5">
-        <f>'1 GW data center'!B21</f>
+        <f>'1 GW data center'!B20</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>'1 GW data center'!C21</f>
+        <f>'1 GW data center'!C20</f>
         <v/>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="F15" s="5">
         <f>B15*D15</f>
@@ -5706,39 +5707,56 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
+          <t>chillers, piping steel; water, copper, refrigerant not</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>IT — servers and racks</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>'1 GW data center'!B21</f>
+        <v/>
+      </c>
+      <c r="C16" s="5">
+        <f>'1 GW data center'!C21</f>
+        <v/>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F16" s="5">
+        <f>B16*D16</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>C16*E16</f>
+        <v/>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>steel chassis and racks; aluminum, PCBs, copper</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Above-ground mass, contents included (tons)</t>
-        </is>
-      </c>
-      <c r="B17" s="4">
-        <f>SUM(B2:B15)</f>
-        <v/>
-      </c>
-      <c r="C17" s="4">
-        <f>SUM(C2:C15)</f>
-        <v/>
-      </c>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Steel in it (tons)</t>
+          <t>Above-ground mass, contents included (tons)</t>
         </is>
       </c>
       <c r="B18" s="4">
-        <f>SUM(F2:F15)</f>
+        <f>SUM(B2:B16)</f>
         <v/>
       </c>
       <c r="C18" s="4">
-        <f>SUM(G2:G15)</f>
+        <f>SUM(C2:C16)</f>
         <v/>
       </c>
       <c r="F18" s="4" t="n"/>
@@ -5747,52 +5765,136 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Steel share of above-ground mass</t>
-        </is>
-      </c>
-      <c r="B19" s="16">
-        <f>B18/B17</f>
-        <v/>
-      </c>
-      <c r="C19" s="16">
-        <f>C18/C17</f>
-        <v/>
-      </c>
+          <t>Steel in it (tons)</t>
+        </is>
+      </c>
+      <c r="B19" s="4">
+        <f>SUM(F2:F16)</f>
+        <v/>
+      </c>
+      <c r="C19" s="4">
+        <f>SUM(G2:G16)</f>
+        <v/>
+      </c>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Steel share including slab rebar (at-grade steel)</t>
+          <t>Steel share of above-ground mass</t>
         </is>
       </c>
       <c r="B20" s="16">
-        <f>(B18+'1 GW data center'!B6)/(B17+'1 GW data center'!B6)</f>
+        <f>B19/B18</f>
         <v/>
       </c>
       <c r="C20" s="16">
-        <f>(C18+'1 GW data center'!C6)/(C17+'1 GW data center'!C6)</f>
+        <f>C19/C18</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
+          <t>Steel share including slab rebar (at-grade steel)</t>
+        </is>
+      </c>
+      <c r="B21" s="16">
+        <f>(B19+'1 GW data center'!B6)/(B18+'1 GW data center'!B6)</f>
+        <v/>
+      </c>
+      <c r="C21" s="16">
+        <f>(C19+'1 GW data center'!C6)/(C18+'1 GW data center'!C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
           <t>Structure and envelope only (first five rows)</t>
         </is>
       </c>
-      <c r="B21" s="16">
-        <f>SUM(F2:F6)/SUM(B2:B6)</f>
-        <v/>
-      </c>
-      <c r="C21" s="16">
-        <f>SUM(G2:G6)/SUM(C2:C6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Excludes slab on grade, paving, foundations and all concrete. Steel fractions per component are estimates [conf: L] (yellow cells). Printed band on the deck: 50–80% (Alex, 2026-09-04). Precast/tilt-up walls would add above-ground concrete and lower the share sharply.</t>
+      <c r="B22" s="16">
+        <f>SUM(F2:F7)/SUM(B2:B7)</f>
+        <v/>
+      </c>
+      <c r="C22" s="16">
+        <f>SUM(G2:G7)/SUM(C2:C7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>WALL SYSTEM CASES (independent of the Inputs toggle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tilt-up / precast wall mass if chosen (tons)</t>
+        </is>
+      </c>
+      <c r="B25" s="17">
+        <f>Derived!B4*Inputs!$B$14*Inputs!$B$12</f>
+        <v/>
+      </c>
+      <c r="C25" s="17">
+        <f>Derived!C4*Inputs!$C$14*Inputs!$C$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Metal-panel skin mass if chosen (tons)</t>
+        </is>
+      </c>
+      <c r="B26" s="17">
+        <f>Derived!B4*Inputs!$B$19/1000</f>
+        <v/>
+      </c>
+      <c r="C26" s="17">
+        <f>Derived!C4*Inputs!$C$19/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Steel share — metal-panel walls</t>
+        </is>
+      </c>
+      <c r="B27" s="16">
+        <f>(B19-F2-F5+B26*D5)/(B18-B2-B5+B26)</f>
+        <v/>
+      </c>
+      <c r="C27" s="16">
+        <f>(C19-F2-F5+C26*E5)/(C18-C2-C5+C26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Steel share — tilt-up / precast concrete walls</t>
+        </is>
+      </c>
+      <c r="B28" s="16">
+        <f>(B19-F2-F5+B25*D2)/(B18-B2-B5+B25)</f>
+        <v/>
+      </c>
+      <c r="C28" s="16">
+        <f>(C19-G2-G5+C25*E2)/(C18-C2-C5+C25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Excludes slab on grade, paving and foundations. The wall system matters: the main block follows Inputs walls_precast (0 = metal panel, 1 = tilt-up/precast); the two case rows above force each wall system regardless of the toggle. Steel fractions per component are estimates [conf: L] (yellow cells). Printed band on the deck: 50–80% (Alex, 2026-09-04), covering both wall systems.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DC investor deck: server boxes out of the long term; board-and-batten acoustic tile
Alex 2026-09-05: remove discussion of server boxes from the long term.
IT is now never replaced in the model; long-term SUPERWOOD falls to
56,000-346,000 tons (1.8-11 years of SuperMill Two). Workbook, markdown,
charts, web bars, Worth table, structural card, register, PRODUCT and
outline updated. Soon slide: acoustic barrier tile regenerated as a
vertical board-and-batten screen.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1451,14 +1451,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Share of IT mass that is server and equipment enclosures (boxes), replaceable long term</t>
+          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1467,26 +1467,26 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>estimated [L]; Alex 2026-09-04</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Server boxes eventually; the electronics never</t>
+          <t>Remainder is slab on grade, paving and yard</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
+          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>0.4</v>
+        <v>0.75</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1495,26 +1495,26 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Remainder is slab on grade, paving and yard</t>
+          <t>Technical potential, not a plan; no design or code pathway yet</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
+          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>0.75</v>
+        <v>0.9</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.75</v>
+        <v>0.9</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1528,53 +1528,53 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan; no design or code pathway yet</t>
+          <t>Technical potential, not a plan</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
+          <t>kg SUPERWOOD per kg of concrete replaced</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>0.9</v>
+        <v>0.05</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.9</v>
+        <v>0.15</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan</t>
+          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>kg SUPERWOOD per kg of concrete replaced</t>
+          <t>Ducting, plenums and air-distribution sheet metal</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>0.05</v>
+        <v>3</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.15</v>
+        <v>8</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>t/MW</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1584,86 +1584,82 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
+          <t>Separate from the mechanical-equipment row</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ducting, plenums and air-distribution sheet metal</t>
+          <t>Concrete emissions</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>3</v>
+        <v>0.12</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>8</v>
+        <v>0.12</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>t/MW</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>industry range [M]</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Separate from the mechanical-equipment row</t>
+          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Concrete emissions</t>
+          <t>SUPERWOOD average board thickness</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>0.12</v>
+        <v>7.2</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.12</v>
+        <v>7.2</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
-        </is>
-      </c>
+          <t>internal TEM basis [H]</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SUPERWOOD average board thickness</t>
+          <t>SUPERWOOD density</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>7.2</v>
+        <v>1300</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>7.2</v>
+        <v>1300</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>kg/m³</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>internal TEM basis [H]</t>
+          <t>internal TEM [H]</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -1671,23 +1667,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SUPERWOOD density</t>
+          <t>SuperMill One output</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>1300</v>
+        <v>1000000</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1300</v>
+        <v>1000000</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>kg/m³</t>
+          <t>sf/yr</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>internal TEM [H]</t>
+          <t>internal [H]</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -1695,14 +1691,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SuperMill One output</t>
+          <t>SuperMill Two output</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>1000000</v>
+        <v>36000000</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>1000000</v>
+        <v>36000000</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1719,42 +1715,46 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SuperMill Two output</t>
+          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>36000000</v>
+        <v>0.3</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>36000000</v>
+        <v>0.6</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>sf/yr</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>internal [H]</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
+          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>0.3</v>
+        <v>20</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.6</v>
+        <v>40</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>kg/m²</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1764,25 +1764,25 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
+          <t>Panel design unsettled</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
+          <t>Addressable share of other tray / containment / doors (medium term)</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>20</v>
+        <v>0.5</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>40</v>
+        <v>0.5</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>kg/m²</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1790,75 +1790,71 @@
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Panel design unsettled</t>
-        </is>
-      </c>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Addressable share of other tray / containment / doors (medium term)</t>
+          <t>Count rebar as addressable in the long term? (0/1)</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Rebar is a frontier market with no pathway; off by default</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Count rebar as addressable in the long term? (0/1)</t>
+          <t>Steel emissions, global average (BF-BOF)</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Rebar is a frontier market with no pathway; off by default</t>
-        </is>
-      </c>
+          <t>published-class [M]</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Steel emissions, global average (BF-BOF)</t>
+          <t>Steel emissions, recycled (EAF)</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>1.8</v>
+        <v>0.4</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>1.8</v>
+        <v>0.7</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1867,7 +1863,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>published-class [M]</t>
+          <t>industry range [M]</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -1875,14 +1871,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Steel emissions, recycled (EAF)</t>
+          <t>SUPERWOOD manufacturing emissions</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1891,22 +1887,26 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
+          <t>internal, pre-LCA [L]</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SUPERWOOD manufacturing emissions</t>
+          <t>SUPERWOOD biogenic carbon stored</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1920,21 +1920,21 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
+          <t>Report separately; module C release under EN 15804</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SUPERWOOD biogenic carbon stored</t>
+          <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1943,38 +1943,10 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
-        <is>
-          <t>Report separately; module C release under EN 15804</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>kg CO₂e/kg</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
         <is>
           <t>Used only for the interior finishes row</t>
         </is>
@@ -2197,11 +2169,11 @@
         </is>
       </c>
       <c r="B3" s="5">
-        <f>Inputs!$B$11*(1-Inputs!$B$30)*Inputs!$B$12*Inputs!$B$2-B5</f>
+        <f>Inputs!$B$11*(1-Inputs!$B$29)*Inputs!$B$12*Inputs!$B$2-B5</f>
         <v/>
       </c>
       <c r="C3" s="5">
-        <f>Inputs!$C$11*(1-Inputs!$C$30)*Inputs!$C$12*Inputs!$C$2-C5</f>
+        <f>Inputs!$C$11*(1-Inputs!$C$29)*Inputs!$C$12*Inputs!$C$2-C5</f>
         <v/>
       </c>
       <c r="D3" s="5">
@@ -2222,7 +2194,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="6">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$30</f>
         <v/>
       </c>
       <c r="J3" s="5">
@@ -2234,11 +2206,11 @@
         <v/>
       </c>
       <c r="L3" s="5">
-        <f>J3*Inputs!$B$33</f>
+        <f>J3*Inputs!$B$32</f>
         <v/>
       </c>
       <c r="M3" s="5">
-        <f>K3*Inputs!$C$33</f>
+        <f>K3*Inputs!$C$32</f>
         <v/>
       </c>
       <c r="N3" t="inlineStr">
@@ -2283,7 +2255,7 @@
         <v/>
       </c>
       <c r="X3" s="7">
-        <f>Inputs!$B$35</f>
+        <f>Inputs!$B$34</f>
         <v/>
       </c>
       <c r="Y3" s="5">
@@ -2295,7 +2267,7 @@
         <v/>
       </c>
       <c r="AA3" s="7">
-        <f>Inputs!$B$35</f>
+        <f>Inputs!$B$34</f>
         <v/>
       </c>
       <c r="AB3" t="inlineStr">
@@ -2311,11 +2283,11 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>Inputs!$B$11*Inputs!$B$30*Inputs!$B$12*Inputs!$B$2</f>
+        <f>Inputs!$B$11*Inputs!$B$29*Inputs!$B$12*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C4" s="5">
-        <f>Inputs!$C$11*Inputs!$C$30*Inputs!$C$12*Inputs!$C$2</f>
+        <f>Inputs!$C$11*Inputs!$C$29*Inputs!$C$12*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D4" s="5">
@@ -2336,7 +2308,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="6">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$31</f>
         <v/>
       </c>
       <c r="J4" s="5">
@@ -2348,11 +2320,11 @@
         <v/>
       </c>
       <c r="L4" s="5">
-        <f>J4*Inputs!$B$33</f>
+        <f>J4*Inputs!$B$32</f>
         <v/>
       </c>
       <c r="M4" s="5">
-        <f>K4*Inputs!$C$33</f>
+        <f>K4*Inputs!$C$32</f>
         <v/>
       </c>
       <c r="N4" t="inlineStr">
@@ -2397,7 +2369,7 @@
         <v/>
       </c>
       <c r="X4" s="7">
-        <f>Inputs!$B$35</f>
+        <f>Inputs!$B$34</f>
         <v/>
       </c>
       <c r="Y4" s="5">
@@ -2409,7 +2381,7 @@
         <v/>
       </c>
       <c r="AA4" s="7">
-        <f>Inputs!$B$35</f>
+        <f>Inputs!$B$34</f>
         <v/>
       </c>
       <c r="AB4" t="inlineStr">
@@ -2461,11 +2433,11 @@
         <v/>
       </c>
       <c r="L5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$41/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$40/1000</f>
         <v/>
       </c>
       <c r="M5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$41/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$40/1000</f>
         <v/>
       </c>
       <c r="N5" t="inlineStr">
@@ -2510,7 +2482,7 @@
         <v/>
       </c>
       <c r="X5" s="7">
-        <f>Inputs!$B$35</f>
+        <f>Inputs!$B$34</f>
         <v/>
       </c>
       <c r="Y5" s="5">
@@ -2522,7 +2494,7 @@
         <v/>
       </c>
       <c r="AA5" s="7">
-        <f>Inputs!$B$35</f>
+        <f>Inputs!$B$34</f>
         <v/>
       </c>
       <c r="AB5" t="inlineStr">
@@ -2563,7 +2535,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="6">
-        <f>Inputs!$B$30*Inputs!$B$32+(1-Inputs!$B$30)*Inputs!$B$31</f>
+        <f>Inputs!$B$29*Inputs!$B$31+(1-Inputs!$B$29)*Inputs!$B$30</f>
         <v/>
       </c>
       <c r="J6" s="5">
@@ -2575,11 +2547,11 @@
         <v/>
       </c>
       <c r="L6" s="5">
-        <f>J6*Inputs!$B$40</f>
+        <f>J6*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="M6" s="5">
-        <f>K6*Inputs!$C$40</f>
+        <f>K6*Inputs!$C$39</f>
         <v/>
       </c>
       <c r="N6" t="inlineStr">
@@ -2624,7 +2596,7 @@
         <v/>
       </c>
       <c r="X6" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y6" s="5">
@@ -2636,7 +2608,7 @@
         <v/>
       </c>
       <c r="AA6" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB6" t="inlineStr">
@@ -2688,11 +2660,11 @@
         <v/>
       </c>
       <c r="L7" s="5">
-        <f>J7*Inputs!$B$40</f>
+        <f>J7*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="M7" s="5">
-        <f>K7*Inputs!$C$40</f>
+        <f>K7*Inputs!$C$39</f>
         <v/>
       </c>
       <c r="N7" t="inlineStr">
@@ -2737,7 +2709,7 @@
         <v/>
       </c>
       <c r="X7" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y7" s="5">
@@ -2749,7 +2721,7 @@
         <v/>
       </c>
       <c r="AA7" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB7" t="inlineStr">
@@ -2801,11 +2773,11 @@
         <v/>
       </c>
       <c r="L8" s="5">
-        <f>J8*Inputs!$B$40</f>
+        <f>J8*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="M8" s="5">
-        <f>K8*Inputs!$C$40</f>
+        <f>K8*Inputs!$C$39</f>
         <v/>
       </c>
       <c r="N8" t="inlineStr">
@@ -2850,7 +2822,7 @@
         <v/>
       </c>
       <c r="X8" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y8" s="5">
@@ -2862,7 +2834,7 @@
         <v/>
       </c>
       <c r="AA8" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB8" t="inlineStr">
@@ -2963,7 +2935,7 @@
         <v/>
       </c>
       <c r="X9" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y9" s="5">
@@ -2975,7 +2947,7 @@
         <v/>
       </c>
       <c r="AA9" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB9" t="inlineStr">
@@ -3076,7 +3048,7 @@
         <v/>
       </c>
       <c r="X10" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y10" s="5">
@@ -3088,7 +3060,7 @@
         <v/>
       </c>
       <c r="AA10" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB10" t="inlineStr">
@@ -3189,7 +3161,7 @@
         <v/>
       </c>
       <c r="X11" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y11" s="5">
@@ -3201,7 +3173,7 @@
         <v/>
       </c>
       <c r="AA11" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB11" t="inlineStr">
@@ -3281,11 +3253,11 @@
         <v/>
       </c>
       <c r="L13" s="5">
-        <f>J13*Inputs!$B$40</f>
+        <f>J13*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="M13" s="5">
-        <f>K13*Inputs!$C$40</f>
+        <f>K13*Inputs!$C$39</f>
         <v/>
       </c>
       <c r="N13" t="inlineStr">
@@ -3330,7 +3302,7 @@
         <v/>
       </c>
       <c r="X13" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y13" s="5">
@@ -3342,7 +3314,7 @@
         <v/>
       </c>
       <c r="AA13" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB13" t="inlineStr">
@@ -3394,11 +3366,11 @@
         <v/>
       </c>
       <c r="L14" s="5">
-        <f>J14*Inputs!$B$40</f>
+        <f>J14*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="M14" s="5">
-        <f>K14*Inputs!$C$40</f>
+        <f>K14*Inputs!$C$39</f>
         <v/>
       </c>
       <c r="N14" t="inlineStr">
@@ -3443,7 +3415,7 @@
         <v/>
       </c>
       <c r="X14" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y14" s="5">
@@ -3455,7 +3427,7 @@
         <v/>
       </c>
       <c r="AA14" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB14" t="inlineStr">
@@ -3507,11 +3479,11 @@
         <v/>
       </c>
       <c r="L15" s="5">
-        <f>J15*Inputs!$B$40</f>
+        <f>J15*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="M15" s="5">
-        <f>K15*Inputs!$C$40</f>
+        <f>K15*Inputs!$C$39</f>
         <v/>
       </c>
       <c r="N15" t="inlineStr">
@@ -3556,7 +3528,7 @@
         <v/>
       </c>
       <c r="X15" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y15" s="5">
@@ -3568,7 +3540,7 @@
         <v/>
       </c>
       <c r="AA15" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB15" t="inlineStr">
@@ -3603,7 +3575,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="6">
-        <f>Inputs!$B$42</f>
+        <f>Inputs!$B$41</f>
         <v/>
       </c>
       <c r="H16" s="6" t="n">
@@ -3621,11 +3593,11 @@
         <v/>
       </c>
       <c r="L16" s="5">
-        <f>J16*Inputs!$B$40</f>
+        <f>J16*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="M16" s="5">
-        <f>K16*Inputs!$C$40</f>
+        <f>K16*Inputs!$C$39</f>
         <v/>
       </c>
       <c r="N16" t="inlineStr">
@@ -3670,7 +3642,7 @@
         <v/>
       </c>
       <c r="X16" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y16" s="5">
@@ -3682,7 +3654,7 @@
         <v/>
       </c>
       <c r="AA16" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB16" t="inlineStr">
@@ -3698,11 +3670,11 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>Inputs!$B$34*Inputs!$B$2</f>
+        <f>Inputs!$B$33*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>Inputs!$C$34*Inputs!$C$2</f>
+        <f>Inputs!$C$33*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D17" s="5">
@@ -3734,11 +3706,11 @@
         <v/>
       </c>
       <c r="L17" s="5">
-        <f>J17*Inputs!$B$40</f>
+        <f>J17*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="M17" s="5">
-        <f>K17*Inputs!$C$40</f>
+        <f>K17*Inputs!$C$39</f>
         <v/>
       </c>
       <c r="N17" t="inlineStr">
@@ -3783,7 +3755,7 @@
         <v/>
       </c>
       <c r="X17" s="7">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="Y17" s="5">
@@ -3795,7 +3767,7 @@
         <v/>
       </c>
       <c r="AA17" s="7">
-        <f>Inputs!$C$45</f>
+        <f>Inputs!$C$44</f>
         <v/>
       </c>
       <c r="AB17" t="inlineStr">
@@ -3896,7 +3868,7 @@
         <v/>
       </c>
       <c r="X18" s="7">
-        <f>Inputs!$B$48</f>
+        <f>Inputs!$B$47</f>
         <v/>
       </c>
       <c r="Y18" s="5">
@@ -3908,7 +3880,7 @@
         <v/>
       </c>
       <c r="AA18" s="7">
-        <f>Inputs!$B$48</f>
+        <f>Inputs!$B$47</f>
         <v/>
       </c>
       <c r="AB18" t="inlineStr">
@@ -4170,9 +4142,8 @@
       <c r="H21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="6">
-        <f>Inputs!$B$29</f>
-        <v/>
+      <c r="I21" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="J21" s="5">
         <f>B21*SUM($F21:$I21)</f>
@@ -4183,16 +4154,16 @@
         <v/>
       </c>
       <c r="L21" s="5">
-        <f>J21*Inputs!$B$40</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="M21" s="5">
-        <f>K21*Inputs!$C$40</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Server and equipment enclosures only (40% of IT mass, estimate); electronics never. Rack masses [H]; aggregate [L]</t>
+          <t>Servers, racks as shipped, and their enclosures are not replaced (Alex 2026-09-05; server boxes removed from the long-term horizon). Rack masses [H]; aggregate per MW [L]</t>
         </is>
       </c>
       <c r="O21" s="5">
@@ -4837,11 +4808,11 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>Inputs!$B$36/1000*Inputs!$B$37*0.092903</f>
+        <f>Inputs!$B$35/1000*Inputs!$B$36*0.092903</f>
         <v/>
       </c>
       <c r="C6" s="15">
-        <f>Inputs!$C$36/1000*Inputs!$C$37*0.092903</f>
+        <f>Inputs!$C$35/1000*Inputs!$C$36*0.092903</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -4857,11 +4828,11 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>Inputs!$B$38*B6/1000</f>
+        <f>Inputs!$B$37*B6/1000</f>
         <v/>
       </c>
       <c r="C7" s="15">
-        <f>Inputs!$C$38*C6/1000</f>
+        <f>Inputs!$C$37*C6/1000</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -4877,11 +4848,11 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>Inputs!$B$39*B6/1000</f>
+        <f>Inputs!$B$38*B6/1000</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>Inputs!$C$39*C6/1000</f>
+        <f>Inputs!$C$38*C6/1000</f>
         <v/>
       </c>
       <c r="D8" t="inlineStr">
@@ -4989,11 +4960,11 @@
         <v/>
       </c>
       <c r="D2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$46</f>
+        <f>'1 GW data center'!B29*Inputs!$B$45</f>
         <v/>
       </c>
       <c r="E2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$46</f>
+        <f>'1 GW data center'!C29*Inputs!$C$45</f>
         <v/>
       </c>
       <c r="F2" s="4">
@@ -5013,11 +4984,11 @@
         <v/>
       </c>
       <c r="J2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$47</f>
+        <f>'1 GW data center'!B29*Inputs!$B$46</f>
         <v/>
       </c>
       <c r="K2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$47</f>
+        <f>'1 GW data center'!C29*Inputs!$C$46</f>
         <v/>
       </c>
     </row>
@@ -5036,11 +5007,11 @@
         <v/>
       </c>
       <c r="D3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$46</f>
+        <f>'1 GW data center'!B34*Inputs!$B$45</f>
         <v/>
       </c>
       <c r="E3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$46</f>
+        <f>'1 GW data center'!C34*Inputs!$C$45</f>
         <v/>
       </c>
       <c r="F3" s="4">
@@ -5060,11 +5031,11 @@
         <v/>
       </c>
       <c r="J3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$47</f>
+        <f>'1 GW data center'!B34*Inputs!$B$46</f>
         <v/>
       </c>
       <c r="K3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$47</f>
+        <f>'1 GW data center'!C34*Inputs!$C$46</f>
         <v/>
       </c>
     </row>
@@ -5083,11 +5054,11 @@
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$46</f>
+        <f>'1 GW data center'!B38*Inputs!$B$45</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$46</f>
+        <f>'1 GW data center'!C38*Inputs!$C$45</f>
         <v/>
       </c>
       <c r="F4" s="4">
@@ -5107,18 +5078,18 @@
         <v/>
       </c>
       <c r="J4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$47</f>
+        <f>'1 GW data center'!B38*Inputs!$B$46</f>
         <v/>
       </c>
       <c r="K4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$47</f>
+        <f>'1 GW data center'!C38*Inputs!$C$46</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Long term (concrete, rebar, server enclosures)</t>
+          <t>Long term (concrete, rebar)</t>
         </is>
       </c>
       <c r="B5" s="4">
@@ -5130,11 +5101,11 @@
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$46</f>
+        <f>'1 GW data center'!B42*Inputs!$B$45</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$46</f>
+        <f>'1 GW data center'!C42*Inputs!$C$45</f>
         <v/>
       </c>
       <c r="F5" s="4">
@@ -5154,11 +5125,11 @@
         <v/>
       </c>
       <c r="J5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$47</f>
+        <f>'1 GW data center'!B42*Inputs!$B$46</f>
         <v/>
       </c>
       <c r="K5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$47</f>
+        <f>'1 GW data center'!C42*Inputs!$C$46</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
DC investor deck: server enclosures back in the long-term numbers, out of the labels
Alex: include server enclosures in the figures but do not list them in
the horizon descriptions because the number is small. Model, workbook,
charts, Worth table and slide 6 bars restored to the 40%-of-IT-mass
basis; labels read "slab, foundations"; footnotes still disclose the
inclusion.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1451,14 +1451,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
+          <t>Share of IT mass that is server and equipment enclosures (boxes), replaceable long term</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1467,26 +1467,26 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>estimated [L]; Alex 2026-09-04</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Remainder is slab on grade, paving and yard</t>
+          <t>Server boxes eventually; the electronics never</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
+          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1495,26 +1495,26 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan; no design or code pathway yet</t>
+          <t>Remainder is slab on grade, paving and yard</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
+          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1528,53 +1528,53 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan</t>
+          <t>Technical potential, not a plan; no design or code pathway yet</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>kg SUPERWOOD per kg of concrete replaced</t>
+          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>0.05</v>
+        <v>0.9</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.15</v>
+        <v>0.9</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
+          <t>Technical potential, not a plan</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ducting, plenums and air-distribution sheet metal</t>
+          <t>kg SUPERWOOD per kg of concrete replaced</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>3</v>
+        <v>0.05</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>8</v>
+        <v>0.15</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>t/MW</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1584,82 +1584,86 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Separate from the mechanical-equipment row</t>
+          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Concrete emissions</t>
+          <t>Ducting, plenums and air-distribution sheet metal</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>0.12</v>
+        <v>3</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.12</v>
+        <v>8</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>t/MW</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
+          <t>Separate from the mechanical-equipment row</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SUPERWOOD average board thickness</t>
+          <t>Concrete emissions</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>7.2</v>
+        <v>0.12</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>7.2</v>
+        <v>0.12</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>internal TEM basis [H]</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SUPERWOOD density</t>
+          <t>SUPERWOOD average board thickness</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>1300</v>
+        <v>7.2</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1300</v>
+        <v>7.2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>kg/m³</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>internal TEM [H]</t>
+          <t>internal TEM basis [H]</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -1667,23 +1671,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SuperMill One output</t>
+          <t>SUPERWOOD density</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>1000000</v>
+        <v>1300</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1000000</v>
+        <v>1300</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>sf/yr</t>
+          <t>kg/m³</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>internal [H]</t>
+          <t>internal TEM [H]</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -1691,14 +1695,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SuperMill Two output</t>
+          <t>SuperMill One output</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>36000000</v>
+        <v>1000000</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>36000000</v>
+        <v>1000000</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1715,46 +1719,42 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
+          <t>SuperMill Two output</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>0.3</v>
+        <v>36000000</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.6</v>
+        <v>36000000</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>sf/yr</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
-        </is>
-      </c>
+          <t>internal [H]</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
+          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>20</v>
+        <v>0.3</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>40</v>
+        <v>0.6</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>kg/m²</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1764,25 +1764,25 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Panel design unsettled</t>
+          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Addressable share of other tray / containment / doors (medium term)</t>
+          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>0.5</v>
+        <v>20</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0.5</v>
+        <v>40</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>kg/m²</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1790,71 +1790,75 @@
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Panel design unsettled</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Count rebar as addressable in the long term? (0/1)</t>
+          <t>Addressable share of other tray / containment / doors (medium term)</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Rebar is a frontier market with no pathway; off by default</t>
-        </is>
-      </c>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Steel emissions, global average (BF-BOF)</t>
+          <t>Count rebar as addressable in the long term? (0/1)</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>published-class [M]</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Rebar is a frontier market with no pathway; off by default</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Steel emissions, recycled (EAF)</t>
+          <t>Steel emissions, global average (BF-BOF)</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0.7</v>
+        <v>1.8</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1863,7 +1867,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
+          <t>published-class [M]</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -1871,14 +1875,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SUPERWOOD manufacturing emissions</t>
+          <t>Steel emissions, recycled (EAF)</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1887,26 +1891,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
-        </is>
-      </c>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SUPERWOOD biogenic carbon stored</t>
+          <t>SUPERWOOD manufacturing emissions</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1920,33 +1920,61 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Report separately; module C release under EN 15804</t>
+          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>SUPERWOOD biogenic carbon stored</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>internal, pre-LCA [L]</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Report separately; module C release under EN 15804</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
         </is>
       </c>
-      <c r="B47" s="2" t="n">
+      <c r="B48" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C47" s="2" t="n">
+      <c r="C48" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>kg CO₂e/kg</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Used only for the interior finishes row</t>
         </is>
@@ -2169,11 +2197,11 @@
         </is>
       </c>
       <c r="B3" s="5">
-        <f>Inputs!$B$11*(1-Inputs!$B$29)*Inputs!$B$12*Inputs!$B$2-B5</f>
+        <f>Inputs!$B$11*(1-Inputs!$B$30)*Inputs!$B$12*Inputs!$B$2-B5</f>
         <v/>
       </c>
       <c r="C3" s="5">
-        <f>Inputs!$C$11*(1-Inputs!$C$29)*Inputs!$C$12*Inputs!$C$2-C5</f>
+        <f>Inputs!$C$11*(1-Inputs!$C$30)*Inputs!$C$12*Inputs!$C$2-C5</f>
         <v/>
       </c>
       <c r="D3" s="5">
@@ -2194,7 +2222,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="6">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$31</f>
         <v/>
       </c>
       <c r="J3" s="5">
@@ -2206,11 +2234,11 @@
         <v/>
       </c>
       <c r="L3" s="5">
-        <f>J3*Inputs!$B$32</f>
+        <f>J3*Inputs!$B$33</f>
         <v/>
       </c>
       <c r="M3" s="5">
-        <f>K3*Inputs!$C$32</f>
+        <f>K3*Inputs!$C$33</f>
         <v/>
       </c>
       <c r="N3" t="inlineStr">
@@ -2255,7 +2283,7 @@
         <v/>
       </c>
       <c r="X3" s="7">
-        <f>Inputs!$B$34</f>
+        <f>Inputs!$B$35</f>
         <v/>
       </c>
       <c r="Y3" s="5">
@@ -2267,7 +2295,7 @@
         <v/>
       </c>
       <c r="AA3" s="7">
-        <f>Inputs!$B$34</f>
+        <f>Inputs!$B$35</f>
         <v/>
       </c>
       <c r="AB3" t="inlineStr">
@@ -2283,11 +2311,11 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>Inputs!$B$11*Inputs!$B$29*Inputs!$B$12*Inputs!$B$2</f>
+        <f>Inputs!$B$11*Inputs!$B$30*Inputs!$B$12*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C4" s="5">
-        <f>Inputs!$C$11*Inputs!$C$29*Inputs!$C$12*Inputs!$C$2</f>
+        <f>Inputs!$C$11*Inputs!$C$30*Inputs!$C$12*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D4" s="5">
@@ -2308,7 +2336,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="6">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$32</f>
         <v/>
       </c>
       <c r="J4" s="5">
@@ -2320,11 +2348,11 @@
         <v/>
       </c>
       <c r="L4" s="5">
-        <f>J4*Inputs!$B$32</f>
+        <f>J4*Inputs!$B$33</f>
         <v/>
       </c>
       <c r="M4" s="5">
-        <f>K4*Inputs!$C$32</f>
+        <f>K4*Inputs!$C$33</f>
         <v/>
       </c>
       <c r="N4" t="inlineStr">
@@ -2369,7 +2397,7 @@
         <v/>
       </c>
       <c r="X4" s="7">
-        <f>Inputs!$B$34</f>
+        <f>Inputs!$B$35</f>
         <v/>
       </c>
       <c r="Y4" s="5">
@@ -2381,7 +2409,7 @@
         <v/>
       </c>
       <c r="AA4" s="7">
-        <f>Inputs!$B$34</f>
+        <f>Inputs!$B$35</f>
         <v/>
       </c>
       <c r="AB4" t="inlineStr">
@@ -2433,11 +2461,11 @@
         <v/>
       </c>
       <c r="L5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$40/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$41/1000</f>
         <v/>
       </c>
       <c r="M5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$40/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$41/1000</f>
         <v/>
       </c>
       <c r="N5" t="inlineStr">
@@ -2482,7 +2510,7 @@
         <v/>
       </c>
       <c r="X5" s="7">
-        <f>Inputs!$B$34</f>
+        <f>Inputs!$B$35</f>
         <v/>
       </c>
       <c r="Y5" s="5">
@@ -2494,7 +2522,7 @@
         <v/>
       </c>
       <c r="AA5" s="7">
-        <f>Inputs!$B$34</f>
+        <f>Inputs!$B$35</f>
         <v/>
       </c>
       <c r="AB5" t="inlineStr">
@@ -2535,7 +2563,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="6">
-        <f>Inputs!$B$29*Inputs!$B$31+(1-Inputs!$B$29)*Inputs!$B$30</f>
+        <f>Inputs!$B$30*Inputs!$B$32+(1-Inputs!$B$30)*Inputs!$B$31</f>
         <v/>
       </c>
       <c r="J6" s="5">
@@ -2547,11 +2575,11 @@
         <v/>
       </c>
       <c r="L6" s="5">
-        <f>J6*Inputs!$B$39</f>
+        <f>J6*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M6" s="5">
-        <f>K6*Inputs!$C$39</f>
+        <f>K6*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N6" t="inlineStr">
@@ -2596,7 +2624,7 @@
         <v/>
       </c>
       <c r="X6" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y6" s="5">
@@ -2608,7 +2636,7 @@
         <v/>
       </c>
       <c r="AA6" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB6" t="inlineStr">
@@ -2660,11 +2688,11 @@
         <v/>
       </c>
       <c r="L7" s="5">
-        <f>J7*Inputs!$B$39</f>
+        <f>J7*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M7" s="5">
-        <f>K7*Inputs!$C$39</f>
+        <f>K7*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N7" t="inlineStr">
@@ -2709,7 +2737,7 @@
         <v/>
       </c>
       <c r="X7" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y7" s="5">
@@ -2721,7 +2749,7 @@
         <v/>
       </c>
       <c r="AA7" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB7" t="inlineStr">
@@ -2773,11 +2801,11 @@
         <v/>
       </c>
       <c r="L8" s="5">
-        <f>J8*Inputs!$B$39</f>
+        <f>J8*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M8" s="5">
-        <f>K8*Inputs!$C$39</f>
+        <f>K8*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N8" t="inlineStr">
@@ -2822,7 +2850,7 @@
         <v/>
       </c>
       <c r="X8" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y8" s="5">
@@ -2834,7 +2862,7 @@
         <v/>
       </c>
       <c r="AA8" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB8" t="inlineStr">
@@ -2935,7 +2963,7 @@
         <v/>
       </c>
       <c r="X9" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y9" s="5">
@@ -2947,7 +2975,7 @@
         <v/>
       </c>
       <c r="AA9" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB9" t="inlineStr">
@@ -3048,7 +3076,7 @@
         <v/>
       </c>
       <c r="X10" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y10" s="5">
@@ -3060,7 +3088,7 @@
         <v/>
       </c>
       <c r="AA10" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB10" t="inlineStr">
@@ -3161,7 +3189,7 @@
         <v/>
       </c>
       <c r="X11" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y11" s="5">
@@ -3173,7 +3201,7 @@
         <v/>
       </c>
       <c r="AA11" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB11" t="inlineStr">
@@ -3253,11 +3281,11 @@
         <v/>
       </c>
       <c r="L13" s="5">
-        <f>J13*Inputs!$B$39</f>
+        <f>J13*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M13" s="5">
-        <f>K13*Inputs!$C$39</f>
+        <f>K13*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N13" t="inlineStr">
@@ -3302,7 +3330,7 @@
         <v/>
       </c>
       <c r="X13" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y13" s="5">
@@ -3314,7 +3342,7 @@
         <v/>
       </c>
       <c r="AA13" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB13" t="inlineStr">
@@ -3366,11 +3394,11 @@
         <v/>
       </c>
       <c r="L14" s="5">
-        <f>J14*Inputs!$B$39</f>
+        <f>J14*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M14" s="5">
-        <f>K14*Inputs!$C$39</f>
+        <f>K14*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N14" t="inlineStr">
@@ -3415,7 +3443,7 @@
         <v/>
       </c>
       <c r="X14" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y14" s="5">
@@ -3427,7 +3455,7 @@
         <v/>
       </c>
       <c r="AA14" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB14" t="inlineStr">
@@ -3479,11 +3507,11 @@
         <v/>
       </c>
       <c r="L15" s="5">
-        <f>J15*Inputs!$B$39</f>
+        <f>J15*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M15" s="5">
-        <f>K15*Inputs!$C$39</f>
+        <f>K15*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N15" t="inlineStr">
@@ -3528,7 +3556,7 @@
         <v/>
       </c>
       <c r="X15" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y15" s="5">
@@ -3540,7 +3568,7 @@
         <v/>
       </c>
       <c r="AA15" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB15" t="inlineStr">
@@ -3575,7 +3603,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="6">
-        <f>Inputs!$B$41</f>
+        <f>Inputs!$B$42</f>
         <v/>
       </c>
       <c r="H16" s="6" t="n">
@@ -3593,11 +3621,11 @@
         <v/>
       </c>
       <c r="L16" s="5">
-        <f>J16*Inputs!$B$39</f>
+        <f>J16*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M16" s="5">
-        <f>K16*Inputs!$C$39</f>
+        <f>K16*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N16" t="inlineStr">
@@ -3642,7 +3670,7 @@
         <v/>
       </c>
       <c r="X16" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y16" s="5">
@@ -3654,7 +3682,7 @@
         <v/>
       </c>
       <c r="AA16" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB16" t="inlineStr">
@@ -3670,11 +3698,11 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>Inputs!$B$33*Inputs!$B$2</f>
+        <f>Inputs!$B$34*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>Inputs!$C$33*Inputs!$C$2</f>
+        <f>Inputs!$C$34*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D17" s="5">
@@ -3706,11 +3734,11 @@
         <v/>
       </c>
       <c r="L17" s="5">
-        <f>J17*Inputs!$B$39</f>
+        <f>J17*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M17" s="5">
-        <f>K17*Inputs!$C$39</f>
+        <f>K17*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N17" t="inlineStr">
@@ -3755,7 +3783,7 @@
         <v/>
       </c>
       <c r="X17" s="7">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="Y17" s="5">
@@ -3767,7 +3795,7 @@
         <v/>
       </c>
       <c r="AA17" s="7">
-        <f>Inputs!$C$44</f>
+        <f>Inputs!$C$45</f>
         <v/>
       </c>
       <c r="AB17" t="inlineStr">
@@ -3868,7 +3896,7 @@
         <v/>
       </c>
       <c r="X18" s="7">
-        <f>Inputs!$B$47</f>
+        <f>Inputs!$B$48</f>
         <v/>
       </c>
       <c r="Y18" s="5">
@@ -3880,7 +3908,7 @@
         <v/>
       </c>
       <c r="AA18" s="7">
-        <f>Inputs!$B$47</f>
+        <f>Inputs!$B$48</f>
         <v/>
       </c>
       <c r="AB18" t="inlineStr">
@@ -4142,8 +4170,9 @@
       <c r="H21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="6" t="n">
-        <v>0</v>
+      <c r="I21" s="6">
+        <f>Inputs!$B$29</f>
+        <v/>
       </c>
       <c r="J21" s="5">
         <f>B21*SUM($F21:$I21)</f>
@@ -4154,16 +4183,16 @@
         <v/>
       </c>
       <c r="L21" s="5">
-        <f>0</f>
+        <f>J21*Inputs!$B$40</f>
         <v/>
       </c>
       <c r="M21" s="5">
-        <f>0</f>
+        <f>K21*Inputs!$C$40</f>
         <v/>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Servers, racks as shipped, and their enclosures are not replaced (Alex 2026-09-05; server boxes removed from the long-term horizon). Rack masses [H]; aggregate per MW [L]</t>
+          <t>Server and equipment enclosures only (40% of IT mass, estimate); electronics never. Rack masses [H]; aggregate [L]</t>
         </is>
       </c>
       <c r="O21" s="5">
@@ -4808,11 +4837,11 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>Inputs!$B$35/1000*Inputs!$B$36*0.092903</f>
+        <f>Inputs!$B$36/1000*Inputs!$B$37*0.092903</f>
         <v/>
       </c>
       <c r="C6" s="15">
-        <f>Inputs!$C$35/1000*Inputs!$C$36*0.092903</f>
+        <f>Inputs!$C$36/1000*Inputs!$C$37*0.092903</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -4828,11 +4857,11 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>Inputs!$B$37*B6/1000</f>
+        <f>Inputs!$B$38*B6/1000</f>
         <v/>
       </c>
       <c r="C7" s="15">
-        <f>Inputs!$C$37*C6/1000</f>
+        <f>Inputs!$C$38*C6/1000</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -4848,11 +4877,11 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>Inputs!$B$38*B6/1000</f>
+        <f>Inputs!$B$39*B6/1000</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>Inputs!$C$38*C6/1000</f>
+        <f>Inputs!$C$39*C6/1000</f>
         <v/>
       </c>
       <c r="D8" t="inlineStr">
@@ -4960,11 +4989,11 @@
         <v/>
       </c>
       <c r="D2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$45</f>
+        <f>'1 GW data center'!B29*Inputs!$B$46</f>
         <v/>
       </c>
       <c r="E2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$45</f>
+        <f>'1 GW data center'!C29*Inputs!$C$46</f>
         <v/>
       </c>
       <c r="F2" s="4">
@@ -4984,11 +5013,11 @@
         <v/>
       </c>
       <c r="J2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$46</f>
+        <f>'1 GW data center'!B29*Inputs!$B$47</f>
         <v/>
       </c>
       <c r="K2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$46</f>
+        <f>'1 GW data center'!C29*Inputs!$C$47</f>
         <v/>
       </c>
     </row>
@@ -5007,11 +5036,11 @@
         <v/>
       </c>
       <c r="D3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$45</f>
+        <f>'1 GW data center'!B34*Inputs!$B$46</f>
         <v/>
       </c>
       <c r="E3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$45</f>
+        <f>'1 GW data center'!C34*Inputs!$C$46</f>
         <v/>
       </c>
       <c r="F3" s="4">
@@ -5031,11 +5060,11 @@
         <v/>
       </c>
       <c r="J3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$46</f>
+        <f>'1 GW data center'!B34*Inputs!$B$47</f>
         <v/>
       </c>
       <c r="K3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$46</f>
+        <f>'1 GW data center'!C34*Inputs!$C$47</f>
         <v/>
       </c>
     </row>
@@ -5054,11 +5083,11 @@
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$45</f>
+        <f>'1 GW data center'!B38*Inputs!$B$46</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$45</f>
+        <f>'1 GW data center'!C38*Inputs!$C$46</f>
         <v/>
       </c>
       <c r="F4" s="4">
@@ -5078,18 +5107,18 @@
         <v/>
       </c>
       <c r="J4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$46</f>
+        <f>'1 GW data center'!B38*Inputs!$B$47</f>
         <v/>
       </c>
       <c r="K4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$46</f>
+        <f>'1 GW data center'!C38*Inputs!$C$47</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Long term (concrete, rebar)</t>
+          <t>Long term (concrete, rebar, server enclosures)</t>
         </is>
       </c>
       <c r="B5" s="4">
@@ -5101,11 +5130,11 @@
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$45</f>
+        <f>'1 GW data center'!B42*Inputs!$B$46</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$45</f>
+        <f>'1 GW data center'!C42*Inputs!$C$46</f>
         <v/>
       </c>
       <c r="F5" s="4">
@@ -5125,11 +5154,11 @@
         <v/>
       </c>
       <c r="J5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$46</f>
+        <f>'1 GW data center'!B42*Inputs!$B$47</f>
         <v/>
       </c>
       <c r="K5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$46</f>
+        <f>'1 GW data center'!C42*Inputs!$C$47</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
DC investor deck: slide 6 estimates equipment steel carbon; groups reordered
Alex 2026-09-05: estimate the embodied carbon of the steel in electrical,
mechanical and IT equipment (60/50/40% of mass at the steel factor,
estimates), and order the stack contents first, then structure and
envelope, foundation at the bottom. Model v8, markdown, charts, both
web decks, PPTX and the register updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1977,6 +1977,90 @@
       <c r="F48" t="inlineStr">
         <is>
           <t>Used only for the interior finishes row</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Steel share of electrical equipment mass (gensets, transformers, switchgear, UPS cabinets)</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>estimated [L]; Alex asked for the estimate 2026-09-05</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Cast iron and steel in engines, transformer cores and tanks, switchgear and UPS enclosures; copper, aluminum, oil and cells excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Steel share of mechanical equipment mass (chillers, fan walls, coolers, piping)</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Shells, frames, casings and steel piping; copper tubes, aluminum coils and loop water excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Steel share of IT mass (rack frames, server chassis)</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Same 40% enclosure share used for the long-term replacement row</t>
         </is>
       </c>
     </row>
@@ -4008,19 +4092,21 @@
         <f>IF(SUM($F19:$I19)=0,0,M19*I19/SUM($F19:$I19))</f>
         <v/>
       </c>
-      <c r="X19" s="8" t="inlineStr">
-        <is>
-          <t>not estimated</t>
-        </is>
-      </c>
-      <c r="Y19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="8" t="n">
-        <v>0</v>
+      <c r="X19" s="7">
+        <f>Inputs!$B$49*Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y19" s="5">
+        <f>B19*X19</f>
+        <v/>
+      </c>
+      <c r="Z19" s="5">
+        <f>C19*X19</f>
+        <v/>
+      </c>
+      <c r="AA19" s="7">
+        <f>Inputs!$B$49*Inputs!$C$45</f>
+        <v/>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
@@ -4119,19 +4205,21 @@
         <f>IF(SUM($F20:$I20)=0,0,M20*I20/SUM($F20:$I20))</f>
         <v/>
       </c>
-      <c r="X20" s="8" t="inlineStr">
-        <is>
-          <t>not estimated</t>
-        </is>
-      </c>
-      <c r="Y20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="8" t="n">
-        <v>0</v>
+      <c r="X20" s="7">
+        <f>Inputs!$B$50*Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y20" s="5">
+        <f>B20*X20</f>
+        <v/>
+      </c>
+      <c r="Z20" s="5">
+        <f>C20*X20</f>
+        <v/>
+      </c>
+      <c r="AA20" s="7">
+        <f>Inputs!$B$50*Inputs!$C$45</f>
+        <v/>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
@@ -4231,19 +4319,21 @@
         <f>IF(SUM($F21:$I21)=0,0,M21*I21/SUM($F21:$I21))</f>
         <v/>
       </c>
-      <c r="X21" s="8" t="inlineStr">
-        <is>
-          <t>not estimated</t>
-        </is>
-      </c>
-      <c r="Y21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="8" t="n">
-        <v>0</v>
+      <c r="X21" s="7">
+        <f>Inputs!$B$51*Inputs!$B$44</f>
+        <v/>
+      </c>
+      <c r="Y21" s="5">
+        <f>B21*X21</f>
+        <v/>
+      </c>
+      <c r="Z21" s="5">
+        <f>C21*X21</f>
+        <v/>
+      </c>
+      <c r="AA21" s="7">
+        <f>Inputs!$B$51*Inputs!$C$45</f>
+        <v/>
       </c>
       <c r="AB21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
DC investor deck: material split and polymer factor actually applied
The previous two commits described this change but a guarded edit had
skipped the workbook and the polymer step failed before writing. Now
applied: per-row material split in the workbook (v9), plastics valued
at an average 3.0 kg CO2e/kg, legend and footnote say so, both decks,
charts, PPTX and register updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1647,47 +1647,51 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SUPERWOOD average board thickness</t>
+          <t>Polymers in paints, foam cores and plastic trim (average)</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>7.2</v>
+        <v>3</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>7.2</v>
+        <v>3</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>internal TEM basis [H]</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>industry range [M]; Alex 2026-09-05</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Cradle to gate; polyolefins and PVC about 2–2.5, polyurethane foam 3–4, coatings higher</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SUPERWOOD density</t>
+          <t>SUPERWOOD average board thickness</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>1300</v>
+        <v>7.2</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1300</v>
+        <v>7.2</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>kg/m³</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>internal TEM [H]</t>
+          <t>internal TEM basis [H]</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -1695,23 +1699,23 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SuperMill One output</t>
+          <t>SUPERWOOD density</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>1000000</v>
+        <v>1300</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>1000000</v>
+        <v>1300</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>sf/yr</t>
+          <t>kg/m³</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>internal [H]</t>
+          <t>internal TEM [H]</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -1719,14 +1723,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SuperMill Two output</t>
+          <t>SuperMill One output</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>36000000</v>
+        <v>1000000</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>36000000</v>
+        <v>1000000</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1743,46 +1747,42 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
+          <t>SuperMill Two output</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>0.3</v>
+        <v>36000000</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.6</v>
+        <v>36000000</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>sf/yr</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
-        </is>
-      </c>
+          <t>internal [H]</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
+          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>20</v>
+        <v>0.3</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>40</v>
+        <v>0.6</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>kg/m²</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1792,25 +1792,25 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Panel design unsettled</t>
+          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Addressable share of other tray / containment / doors (medium term)</t>
+          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0.5</v>
+        <v>20</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0.5</v>
+        <v>40</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>kg/m²</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1818,71 +1818,75 @@
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Panel design unsettled</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Count rebar as addressable in the long term? (0/1)</t>
+          <t>Addressable share of other tray / containment / doors (medium term)</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Rebar is a frontier market with no pathway; off by default</t>
-        </is>
-      </c>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Steel emissions, global average (BF-BOF)</t>
+          <t>Count rebar as addressable in the long term? (0/1)</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>published-class [M]</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Rebar is a frontier market with no pathway; off by default</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Steel emissions, recycled (EAF)</t>
+          <t>Steel emissions, global average (BF-BOF)</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0.7</v>
+        <v>1.8</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1891,7 +1895,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
+          <t>published-class [M]</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -1899,14 +1903,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SUPERWOOD manufacturing emissions</t>
+          <t>Steel emissions, recycled (EAF)</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1915,26 +1919,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
-        </is>
-      </c>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SUPERWOOD biogenic carbon stored</t>
+          <t>SUPERWOOD manufacturing emissions</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Report separately; module C release under EN 15804</t>
+          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
+          <t>SUPERWOOD biogenic carbon stored</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1971,96 +1971,40 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>internal, pre-LCA [L]</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Used only for the interior finishes row</t>
+          <t>Report separately; module C release under EN 15804</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Steel share of electrical equipment mass (gensets, transformers, switchgear, UPS cabinets)</t>
+          <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>estimated [L]; Alex asked for the estimate 2026-09-05</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Cast iron and steel in engines, transformer cores and tanks, switchgear and UPS enclosures; copper, aluminum, oil and cells excluded</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Steel share of mechanical equipment mass (chillers, fan walls, coolers, piping)</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C50" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>share</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Shells, frames, casings and steel piping; copper tubes, aluminum coils and loop water excluded</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Steel share of IT mass (rack frames, server chassis)</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C51" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>share</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Same 40% enclosure share used for the long-term replacement row</t>
+          <t>Used only for the interior finishes row</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB60"/>
+  <dimension ref="A1:AF60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -2106,6 +2050,10 @@
     <col width="18" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="10" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2247,6 +2195,26 @@
       <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Material class</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Steel share</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Concrete share</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Plastic share</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Other share</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2335,7 @@
         <v/>
       </c>
       <c r="X3" s="7">
-        <f>Inputs!$B$35</f>
+        <f>AC3*Inputs!$B$45+AD3*Inputs!$B$35+AE3*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y3" s="5">
@@ -2379,13 +2347,25 @@
         <v/>
       </c>
       <c r="AA3" s="7">
-        <f>Inputs!$B$35</f>
+        <f>AC3*Inputs!$C$46+AD3*Inputs!$B$35+AE3*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
           <t>concrete</t>
         </is>
+      </c>
+      <c r="AC3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2481,7 +2461,7 @@
         <v/>
       </c>
       <c r="X4" s="7">
-        <f>Inputs!$B$35</f>
+        <f>AC4*Inputs!$B$45+AD4*Inputs!$B$35+AE4*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y4" s="5">
@@ -2493,13 +2473,25 @@
         <v/>
       </c>
       <c r="AA4" s="7">
-        <f>Inputs!$B$35</f>
+        <f>AC4*Inputs!$C$46+AD4*Inputs!$B$35+AE4*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
           <t>concrete</t>
         </is>
+      </c>
+      <c r="AC4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2545,11 +2537,11 @@
         <v/>
       </c>
       <c r="L5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$41/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$42/1000</f>
         <v/>
       </c>
       <c r="M5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$41/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$42/1000</f>
         <v/>
       </c>
       <c r="N5" t="inlineStr">
@@ -2594,7 +2586,7 @@
         <v/>
       </c>
       <c r="X5" s="7">
-        <f>Inputs!$B$35</f>
+        <f>AC5*Inputs!$B$45+AD5*Inputs!$B$35+AE5*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y5" s="5">
@@ -2606,13 +2598,25 @@
         <v/>
       </c>
       <c r="AA5" s="7">
-        <f>Inputs!$B$35</f>
+        <f>AC5*Inputs!$C$46+AD5*Inputs!$B$35+AE5*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
           <t>concrete</t>
         </is>
+      </c>
+      <c r="AC5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2659,11 +2663,11 @@
         <v/>
       </c>
       <c r="L6" s="5">
-        <f>J6*Inputs!$B$40</f>
+        <f>J6*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M6" s="5">
-        <f>K6*Inputs!$C$40</f>
+        <f>K6*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N6" t="inlineStr">
@@ -2708,7 +2712,7 @@
         <v/>
       </c>
       <c r="X6" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC6*Inputs!$B$45+AD6*Inputs!$B$35+AE6*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y6" s="5">
@@ -2720,13 +2724,25 @@
         <v/>
       </c>
       <c r="AA6" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC6*Inputs!$C$46+AD6*Inputs!$B$35+AE6*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2772,11 +2788,11 @@
         <v/>
       </c>
       <c r="L7" s="5">
-        <f>J7*Inputs!$B$40</f>
+        <f>J7*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M7" s="5">
-        <f>K7*Inputs!$C$40</f>
+        <f>K7*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N7" t="inlineStr">
@@ -2821,7 +2837,7 @@
         <v/>
       </c>
       <c r="X7" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC7*Inputs!$B$45+AD7*Inputs!$B$35+AE7*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y7" s="5">
@@ -2833,13 +2849,25 @@
         <v/>
       </c>
       <c r="AA7" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC7*Inputs!$C$46+AD7*Inputs!$B$35+AE7*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -2885,11 +2913,11 @@
         <v/>
       </c>
       <c r="L8" s="5">
-        <f>J8*Inputs!$B$40</f>
+        <f>J8*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M8" s="5">
-        <f>K8*Inputs!$C$40</f>
+        <f>K8*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N8" t="inlineStr">
@@ -2934,7 +2962,7 @@
         <v/>
       </c>
       <c r="X8" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC8*Inputs!$B$45+AD8*Inputs!$B$35+AE8*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y8" s="5">
@@ -2946,13 +2974,25 @@
         <v/>
       </c>
       <c r="AA8" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC8*Inputs!$C$46+AD8*Inputs!$B$35+AE8*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -3047,7 +3087,7 @@
         <v/>
       </c>
       <c r="X9" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC9*Inputs!$B$45+AD9*Inputs!$B$35+AE9*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y9" s="5">
@@ -3059,13 +3099,25 @@
         <v/>
       </c>
       <c r="AA9" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC9*Inputs!$C$46+AD9*Inputs!$B$35+AE9*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC9" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AD9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AF9" s="2" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="10">
@@ -3160,7 +3212,7 @@
         <v/>
       </c>
       <c r="X10" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC10*Inputs!$B$45+AD10*Inputs!$B$35+AE10*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y10" s="5">
@@ -3172,13 +3224,25 @@
         <v/>
       </c>
       <c r="AA10" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC10*Inputs!$C$46+AD10*Inputs!$B$35+AE10*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -3273,7 +3337,7 @@
         <v/>
       </c>
       <c r="X11" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC11*Inputs!$B$45+AD11*Inputs!$B$35+AE11*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y11" s="5">
@@ -3285,13 +3349,25 @@
         <v/>
       </c>
       <c r="AA11" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC11*Inputs!$C$46+AD11*Inputs!$B$35+AE11*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -3365,11 +3441,11 @@
         <v/>
       </c>
       <c r="L13" s="5">
-        <f>J13*Inputs!$B$40</f>
+        <f>J13*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M13" s="5">
-        <f>K13*Inputs!$C$40</f>
+        <f>K13*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N13" t="inlineStr">
@@ -3414,7 +3490,7 @@
         <v/>
       </c>
       <c r="X13" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC13*Inputs!$B$45+AD13*Inputs!$B$35+AE13*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y13" s="5">
@@ -3426,13 +3502,25 @@
         <v/>
       </c>
       <c r="AA13" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC13*Inputs!$C$46+AD13*Inputs!$B$35+AE13*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -3478,11 +3566,11 @@
         <v/>
       </c>
       <c r="L14" s="5">
-        <f>J14*Inputs!$B$40</f>
+        <f>J14*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M14" s="5">
-        <f>K14*Inputs!$C$40</f>
+        <f>K14*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N14" t="inlineStr">
@@ -3527,7 +3615,7 @@
         <v/>
       </c>
       <c r="X14" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC14*Inputs!$B$45+AD14*Inputs!$B$35+AE14*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y14" s="5">
@@ -3539,13 +3627,25 @@
         <v/>
       </c>
       <c r="AA14" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC14*Inputs!$C$46+AD14*Inputs!$B$35+AE14*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC14" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AD14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AF14" s="2" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="15">
@@ -3591,11 +3691,11 @@
         <v/>
       </c>
       <c r="L15" s="5">
-        <f>J15*Inputs!$B$40</f>
+        <f>J15*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M15" s="5">
-        <f>K15*Inputs!$C$40</f>
+        <f>K15*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N15" t="inlineStr">
@@ -3640,7 +3740,7 @@
         <v/>
       </c>
       <c r="X15" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC15*Inputs!$B$45+AD15*Inputs!$B$35+AE15*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y15" s="5">
@@ -3652,13 +3752,25 @@
         <v/>
       </c>
       <c r="AA15" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC15*Inputs!$C$46+AD15*Inputs!$B$35+AE15*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3687,7 +3799,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="6">
-        <f>Inputs!$B$42</f>
+        <f>Inputs!$B$43</f>
         <v/>
       </c>
       <c r="H16" s="6" t="n">
@@ -3705,11 +3817,11 @@
         <v/>
       </c>
       <c r="L16" s="5">
-        <f>J16*Inputs!$B$40</f>
+        <f>J16*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M16" s="5">
-        <f>K16*Inputs!$C$40</f>
+        <f>K16*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N16" t="inlineStr">
@@ -3754,7 +3866,7 @@
         <v/>
       </c>
       <c r="X16" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC16*Inputs!$B$45+AD16*Inputs!$B$35+AE16*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y16" s="5">
@@ -3766,13 +3878,25 @@
         <v/>
       </c>
       <c r="AA16" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC16*Inputs!$C$46+AD16*Inputs!$B$35+AE16*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3818,11 +3942,11 @@
         <v/>
       </c>
       <c r="L17" s="5">
-        <f>J17*Inputs!$B$40</f>
+        <f>J17*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M17" s="5">
-        <f>K17*Inputs!$C$40</f>
+        <f>K17*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N17" t="inlineStr">
@@ -3867,7 +3991,7 @@
         <v/>
       </c>
       <c r="X17" s="7">
-        <f>Inputs!$B$44</f>
+        <f>AC17*Inputs!$B$45+AD17*Inputs!$B$35+AE17*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y17" s="5">
@@ -3879,13 +4003,25 @@
         <v/>
       </c>
       <c r="AA17" s="7">
-        <f>Inputs!$C$45</f>
+        <f>AC17*Inputs!$C$46+AD17*Inputs!$B$35+AE17*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
+      </c>
+      <c r="AC17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3980,7 +4116,7 @@
         <v/>
       </c>
       <c r="X18" s="7">
-        <f>Inputs!$B$48</f>
+        <f>AC18*Inputs!$B$45+AD18*Inputs!$B$35+AE18*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y18" s="5">
@@ -3992,13 +4128,25 @@
         <v/>
       </c>
       <c r="AA18" s="7">
-        <f>Inputs!$B$48</f>
+        <f>AC18*Inputs!$C$46+AD18*Inputs!$B$35+AE18*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
+      </c>
+      <c r="AC18" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AD18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF18" s="2" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="19">
@@ -4093,7 +4241,7 @@
         <v/>
       </c>
       <c r="X19" s="7">
-        <f>Inputs!$B$49*Inputs!$B$44</f>
+        <f>AC19*Inputs!$B$45+AD19*Inputs!$B$35+AE19*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y19" s="5">
@@ -4105,13 +4253,25 @@
         <v/>
       </c>
       <c r="AA19" s="7">
-        <f>Inputs!$B$49*Inputs!$C$45</f>
+        <f>AC19*Inputs!$C$46+AD19*Inputs!$B$35+AE19*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
           <t>equipment</t>
         </is>
+      </c>
+      <c r="AC19" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AD19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AF19" s="2" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="20">
@@ -4206,7 +4366,7 @@
         <v/>
       </c>
       <c r="X20" s="7">
-        <f>Inputs!$B$50*Inputs!$B$44</f>
+        <f>AC20*Inputs!$B$45+AD20*Inputs!$B$35+AE20*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y20" s="5">
@@ -4218,13 +4378,25 @@
         <v/>
       </c>
       <c r="AA20" s="7">
-        <f>Inputs!$B$50*Inputs!$C$45</f>
+        <f>AC20*Inputs!$C$46+AD20*Inputs!$B$35+AE20*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
           <t>equipment</t>
         </is>
+      </c>
+      <c r="AC20" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AD20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AF20" s="2" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="21">
@@ -4271,11 +4443,11 @@
         <v/>
       </c>
       <c r="L21" s="5">
-        <f>J21*Inputs!$B$40</f>
+        <f>J21*Inputs!$B$41</f>
         <v/>
       </c>
       <c r="M21" s="5">
-        <f>K21*Inputs!$C$40</f>
+        <f>K21*Inputs!$C$41</f>
         <v/>
       </c>
       <c r="N21" t="inlineStr">
@@ -4320,7 +4492,7 @@
         <v/>
       </c>
       <c r="X21" s="7">
-        <f>Inputs!$B$51*Inputs!$B$44</f>
+        <f>AC21*Inputs!$B$45+AD21*Inputs!$B$35+AE21*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="Y21" s="5">
@@ -4332,13 +4504,25 @@
         <v/>
       </c>
       <c r="AA21" s="7">
-        <f>Inputs!$B$51*Inputs!$C$45</f>
+        <f>AC21*Inputs!$C$46+AD21*Inputs!$B$35+AE21*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
           <t>equipment</t>
         </is>
+      </c>
+      <c r="AC21" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AD21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF21" s="2" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="23">
@@ -4927,11 +5111,11 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>Inputs!$B$36/1000*Inputs!$B$37*0.092903</f>
+        <f>Inputs!$B$37/1000*Inputs!$B$38*0.092903</f>
         <v/>
       </c>
       <c r="C6" s="15">
-        <f>Inputs!$C$36/1000*Inputs!$C$37*0.092903</f>
+        <f>Inputs!$C$37/1000*Inputs!$C$38*0.092903</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -4947,11 +5131,11 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>Inputs!$B$38*B6/1000</f>
+        <f>Inputs!$B$39*B6/1000</f>
         <v/>
       </c>
       <c r="C7" s="15">
-        <f>Inputs!$C$38*C6/1000</f>
+        <f>Inputs!$C$39*C6/1000</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -4967,11 +5151,11 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>Inputs!$B$39*B6/1000</f>
+        <f>Inputs!$B$40*B6/1000</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>Inputs!$C$39*C6/1000</f>
+        <f>Inputs!$C$40*C6/1000</f>
         <v/>
       </c>
       <c r="D8" t="inlineStr">
@@ -5079,11 +5263,11 @@
         <v/>
       </c>
       <c r="D2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$46</f>
+        <f>'1 GW data center'!B29*Inputs!$B$47</f>
         <v/>
       </c>
       <c r="E2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$46</f>
+        <f>'1 GW data center'!C29*Inputs!$C$47</f>
         <v/>
       </c>
       <c r="F2" s="4">
@@ -5103,11 +5287,11 @@
         <v/>
       </c>
       <c r="J2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$47</f>
+        <f>'1 GW data center'!B29*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="K2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$47</f>
+        <f>'1 GW data center'!C29*Inputs!$C$48</f>
         <v/>
       </c>
     </row>
@@ -5126,11 +5310,11 @@
         <v/>
       </c>
       <c r="D3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$46</f>
+        <f>'1 GW data center'!B34*Inputs!$B$47</f>
         <v/>
       </c>
       <c r="E3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$46</f>
+        <f>'1 GW data center'!C34*Inputs!$C$47</f>
         <v/>
       </c>
       <c r="F3" s="4">
@@ -5150,11 +5334,11 @@
         <v/>
       </c>
       <c r="J3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$47</f>
+        <f>'1 GW data center'!B34*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="K3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$47</f>
+        <f>'1 GW data center'!C34*Inputs!$C$48</f>
         <v/>
       </c>
     </row>
@@ -5173,11 +5357,11 @@
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$46</f>
+        <f>'1 GW data center'!B38*Inputs!$B$47</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$46</f>
+        <f>'1 GW data center'!C38*Inputs!$C$47</f>
         <v/>
       </c>
       <c r="F4" s="4">
@@ -5197,11 +5381,11 @@
         <v/>
       </c>
       <c r="J4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$47</f>
+        <f>'1 GW data center'!B38*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="K4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$47</f>
+        <f>'1 GW data center'!C38*Inputs!$C$48</f>
         <v/>
       </c>
     </row>
@@ -5220,11 +5404,11 @@
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$46</f>
+        <f>'1 GW data center'!B42*Inputs!$B$47</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$46</f>
+        <f>'1 GW data center'!C42*Inputs!$C$47</f>
         <v/>
       </c>
       <c r="F5" s="4">
@@ -5244,11 +5428,11 @@
         <v/>
       </c>
       <c r="J5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$47</f>
+        <f>'1 GW data center'!B42*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="K5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$47</f>
+        <f>'1 GW data center'!C42*Inputs!$C$48</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
DC investor deck: server rack cabinets soon, server enclosures long term
Alex 2026-09-06. The IT row now spans two horizons in the workbook
(rack cabinets 18% of IT mass soon, server enclosures 22% long term);
slide 6 bubbles, slide 7 Soon and Long rows, PPTX charts and the
register follow.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1451,14 +1451,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Share of IT mass that is server and equipment enclosures (boxes), replaceable long term</t>
+          <t>Share of IT mass that is server rack cabinets (frames, panels, doors) — substitutable soon</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>0.4</v>
+        <v>0.18</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.4</v>
+        <v>0.18</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1467,26 +1467,26 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>estimated [L]; Alex 2026-09-04</t>
+          <t>estimated [L]; Alex 2026-09-06</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Server boxes eventually; the electronics never</t>
+          <t>A loaded rack of 1–1.4 t carries a 150–250 kg steel cabinet</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
+          <t>Share of IT mass that is server enclosures (chassis) — long term</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>0.4</v>
+        <v>0.22</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.5</v>
+        <v>0.22</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1495,26 +1495,26 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>estimated [L]; Alex 2026-09-04/06</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Remainder is slab on grade, paving and yard</t>
+          <t>Server boxes eventually; the electronics never</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
+          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1523,26 +1523,26 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan; no design or code pathway yet</t>
+          <t>Remainder is slab on grade, paving and yard</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
+          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1556,53 +1556,53 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan</t>
+          <t>Technical potential, not a plan; no design or code pathway yet</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>kg SUPERWOOD per kg of concrete replaced</t>
+          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>0.05</v>
+        <v>0.9</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.15</v>
+        <v>0.9</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
+          <t>Technical potential, not a plan</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ducting, plenums and air-distribution sheet metal</t>
+          <t>kg SUPERWOOD per kg of concrete replaced</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>3</v>
+        <v>0.05</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>8</v>
+        <v>0.15</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>t/MW</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1612,49 +1612,49 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Separate from the mechanical-equipment row</t>
+          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Concrete emissions</t>
+          <t>Ducting, plenums and air-distribution sheet metal</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>0.12</v>
+        <v>3</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.12</v>
+        <v>8</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>t/MW</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
+          <t>Separate from the mechanical-equipment row</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Polymers in paints, foam cores and plastic trim (average)</t>
+          <t>Concrete emissions</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>3</v>
+        <v>0.12</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>3</v>
+        <v>0.12</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1663,59 +1663,63 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>industry range [M]; Alex 2026-09-05</t>
+          <t>industry range [M]</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Cradle to gate; polyolefins and PVC about 2–2.5, polyurethane foam 3–4, coatings higher</t>
+          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SUPERWOOD average board thickness</t>
+          <t>Polymers in paints, foam cores and plastic trim (average)</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>7.2</v>
+        <v>3</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>7.2</v>
+        <v>3</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>internal TEM basis [H]</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+          <t>industry range [M]; Alex 2026-09-05</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Cradle to gate; polyolefins and PVC about 2–2.5, polyurethane foam 3–4, coatings higher</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SUPERWOOD density</t>
+          <t>SUPERWOOD average board thickness</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>1300</v>
+        <v>7.2</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>1300</v>
+        <v>7.2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>kg/m³</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>internal TEM [H]</t>
+          <t>internal TEM basis [H]</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -1723,23 +1727,23 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SuperMill One output</t>
+          <t>SUPERWOOD density</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>1000000</v>
+        <v>1300</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>1000000</v>
+        <v>1300</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>sf/yr</t>
+          <t>kg/m³</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>internal [H]</t>
+          <t>internal TEM [H]</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -1747,14 +1751,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SuperMill Two output</t>
+          <t>SuperMill One output</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>36000000</v>
+        <v>1000000</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>36000000</v>
+        <v>1000000</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1771,46 +1775,42 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
+          <t>SuperMill Two output</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>0.3</v>
+        <v>36000000</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0.6</v>
+        <v>36000000</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>sf/yr</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
-        </is>
-      </c>
+          <t>internal [H]</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
+          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>20</v>
+        <v>0.3</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>40</v>
+        <v>0.6</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>kg/m²</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1820,25 +1820,25 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Panel design unsettled</t>
+          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Addressable share of other tray / containment / doors (medium term)</t>
+          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>0.5</v>
+        <v>20</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>0.5</v>
+        <v>40</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>kg/m²</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1846,71 +1846,75 @@
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Panel design unsettled</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Count rebar as addressable in the long term? (0/1)</t>
+          <t>Addressable share of other tray / containment / doors (medium term)</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Rebar is a frontier market with no pathway; off by default</t>
-        </is>
-      </c>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Steel emissions, global average (BF-BOF)</t>
+          <t>Count rebar as addressable in the long term? (0/1)</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>published-class [M]</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Rebar is a frontier market with no pathway; off by default</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Steel emissions, recycled (EAF)</t>
+          <t>Steel emissions, global average (BF-BOF)</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>0.7</v>
+        <v>1.8</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1919,7 +1923,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
+          <t>published-class [M]</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -1927,14 +1931,14 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SUPERWOOD manufacturing emissions</t>
+          <t>Steel emissions, recycled (EAF)</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1943,26 +1947,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
-        </is>
-      </c>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SUPERWOOD biogenic carbon stored</t>
+          <t>SUPERWOOD manufacturing emissions</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1976,33 +1976,61 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Report separately; module C release under EN 15804</t>
+          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>SUPERWOOD biogenic carbon stored</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>internal, pre-LCA [L]</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Report separately; module C release under EN 15804</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
         </is>
       </c>
-      <c r="B49" s="2" t="n">
+      <c r="B50" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C49" s="2" t="n">
+      <c r="C50" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>kg CO₂e/kg</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>Used only for the interior finishes row</t>
         </is>
@@ -2249,11 +2277,11 @@
         </is>
       </c>
       <c r="B3" s="5">
-        <f>Inputs!$B$11*(1-Inputs!$B$30)*Inputs!$B$12*Inputs!$B$2-B5</f>
+        <f>Inputs!$B$11*(1-Inputs!$B$31)*Inputs!$B$12*Inputs!$B$2-B5</f>
         <v/>
       </c>
       <c r="C3" s="5">
-        <f>Inputs!$C$11*(1-Inputs!$C$30)*Inputs!$C$12*Inputs!$C$2-C5</f>
+        <f>Inputs!$C$11*(1-Inputs!$C$31)*Inputs!$C$12*Inputs!$C$2-C5</f>
         <v/>
       </c>
       <c r="D3" s="5">
@@ -2274,7 +2302,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="6">
-        <f>Inputs!$B$31</f>
+        <f>Inputs!$B$32</f>
         <v/>
       </c>
       <c r="J3" s="5">
@@ -2286,11 +2314,11 @@
         <v/>
       </c>
       <c r="L3" s="5">
-        <f>J3*Inputs!$B$33</f>
+        <f>J3*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="M3" s="5">
-        <f>K3*Inputs!$C$33</f>
+        <f>K3*Inputs!$C$34</f>
         <v/>
       </c>
       <c r="N3" t="inlineStr">
@@ -2335,7 +2363,7 @@
         <v/>
       </c>
       <c r="X3" s="7">
-        <f>AC3*Inputs!$B$45+AD3*Inputs!$B$35+AE3*Inputs!$B$36</f>
+        <f>AC3*Inputs!$B$46+AD3*Inputs!$B$36+AE3*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y3" s="5">
@@ -2347,7 +2375,7 @@
         <v/>
       </c>
       <c r="AA3" s="7">
-        <f>AC3*Inputs!$C$46+AD3*Inputs!$B$35+AE3*Inputs!$B$36</f>
+        <f>AC3*Inputs!$C$47+AD3*Inputs!$B$36+AE3*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB3" t="inlineStr">
@@ -2375,11 +2403,11 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>Inputs!$B$11*Inputs!$B$30*Inputs!$B$12*Inputs!$B$2</f>
+        <f>Inputs!$B$11*Inputs!$B$31*Inputs!$B$12*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C4" s="5">
-        <f>Inputs!$C$11*Inputs!$C$30*Inputs!$C$12*Inputs!$C$2</f>
+        <f>Inputs!$C$11*Inputs!$C$31*Inputs!$C$12*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D4" s="5">
@@ -2400,7 +2428,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="6">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$33</f>
         <v/>
       </c>
       <c r="J4" s="5">
@@ -2412,11 +2440,11 @@
         <v/>
       </c>
       <c r="L4" s="5">
-        <f>J4*Inputs!$B$33</f>
+        <f>J4*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="M4" s="5">
-        <f>K4*Inputs!$C$33</f>
+        <f>K4*Inputs!$C$34</f>
         <v/>
       </c>
       <c r="N4" t="inlineStr">
@@ -2461,7 +2489,7 @@
         <v/>
       </c>
       <c r="X4" s="7">
-        <f>AC4*Inputs!$B$45+AD4*Inputs!$B$35+AE4*Inputs!$B$36</f>
+        <f>AC4*Inputs!$B$46+AD4*Inputs!$B$36+AE4*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y4" s="5">
@@ -2473,7 +2501,7 @@
         <v/>
       </c>
       <c r="AA4" s="7">
-        <f>AC4*Inputs!$C$46+AD4*Inputs!$B$35+AE4*Inputs!$B$36</f>
+        <f>AC4*Inputs!$C$47+AD4*Inputs!$B$36+AE4*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB4" t="inlineStr">
@@ -2537,11 +2565,11 @@
         <v/>
       </c>
       <c r="L5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$42/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$43/1000</f>
         <v/>
       </c>
       <c r="M5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$42/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$43/1000</f>
         <v/>
       </c>
       <c r="N5" t="inlineStr">
@@ -2586,7 +2614,7 @@
         <v/>
       </c>
       <c r="X5" s="7">
-        <f>AC5*Inputs!$B$45+AD5*Inputs!$B$35+AE5*Inputs!$B$36</f>
+        <f>AC5*Inputs!$B$46+AD5*Inputs!$B$36+AE5*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y5" s="5">
@@ -2598,7 +2626,7 @@
         <v/>
       </c>
       <c r="AA5" s="7">
-        <f>AC5*Inputs!$C$46+AD5*Inputs!$B$35+AE5*Inputs!$B$36</f>
+        <f>AC5*Inputs!$C$47+AD5*Inputs!$B$36+AE5*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB5" t="inlineStr">
@@ -2651,7 +2679,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="6">
-        <f>Inputs!$B$30*Inputs!$B$32+(1-Inputs!$B$30)*Inputs!$B$31</f>
+        <f>Inputs!$B$31*Inputs!$B$33+(1-Inputs!$B$31)*Inputs!$B$32</f>
         <v/>
       </c>
       <c r="J6" s="5">
@@ -2663,11 +2691,11 @@
         <v/>
       </c>
       <c r="L6" s="5">
-        <f>J6*Inputs!$B$41</f>
+        <f>J6*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M6" s="5">
-        <f>K6*Inputs!$C$41</f>
+        <f>K6*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N6" t="inlineStr">
@@ -2712,7 +2740,7 @@
         <v/>
       </c>
       <c r="X6" s="7">
-        <f>AC6*Inputs!$B$45+AD6*Inputs!$B$35+AE6*Inputs!$B$36</f>
+        <f>AC6*Inputs!$B$46+AD6*Inputs!$B$36+AE6*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y6" s="5">
@@ -2724,7 +2752,7 @@
         <v/>
       </c>
       <c r="AA6" s="7">
-        <f>AC6*Inputs!$C$46+AD6*Inputs!$B$35+AE6*Inputs!$B$36</f>
+        <f>AC6*Inputs!$C$47+AD6*Inputs!$B$36+AE6*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB6" t="inlineStr">
@@ -2788,11 +2816,11 @@
         <v/>
       </c>
       <c r="L7" s="5">
-        <f>J7*Inputs!$B$41</f>
+        <f>J7*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M7" s="5">
-        <f>K7*Inputs!$C$41</f>
+        <f>K7*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N7" t="inlineStr">
@@ -2837,7 +2865,7 @@
         <v/>
       </c>
       <c r="X7" s="7">
-        <f>AC7*Inputs!$B$45+AD7*Inputs!$B$35+AE7*Inputs!$B$36</f>
+        <f>AC7*Inputs!$B$46+AD7*Inputs!$B$36+AE7*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y7" s="5">
@@ -2849,7 +2877,7 @@
         <v/>
       </c>
       <c r="AA7" s="7">
-        <f>AC7*Inputs!$C$46+AD7*Inputs!$B$35+AE7*Inputs!$B$36</f>
+        <f>AC7*Inputs!$C$47+AD7*Inputs!$B$36+AE7*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB7" t="inlineStr">
@@ -2913,11 +2941,11 @@
         <v/>
       </c>
       <c r="L8" s="5">
-        <f>J8*Inputs!$B$41</f>
+        <f>J8*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M8" s="5">
-        <f>K8*Inputs!$C$41</f>
+        <f>K8*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N8" t="inlineStr">
@@ -2962,7 +2990,7 @@
         <v/>
       </c>
       <c r="X8" s="7">
-        <f>AC8*Inputs!$B$45+AD8*Inputs!$B$35+AE8*Inputs!$B$36</f>
+        <f>AC8*Inputs!$B$46+AD8*Inputs!$B$36+AE8*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y8" s="5">
@@ -2974,7 +3002,7 @@
         <v/>
       </c>
       <c r="AA8" s="7">
-        <f>AC8*Inputs!$C$46+AD8*Inputs!$B$35+AE8*Inputs!$B$36</f>
+        <f>AC8*Inputs!$C$47+AD8*Inputs!$B$36+AE8*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB8" t="inlineStr">
@@ -3087,7 +3115,7 @@
         <v/>
       </c>
       <c r="X9" s="7">
-        <f>AC9*Inputs!$B$45+AD9*Inputs!$B$35+AE9*Inputs!$B$36</f>
+        <f>AC9*Inputs!$B$46+AD9*Inputs!$B$36+AE9*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y9" s="5">
@@ -3099,7 +3127,7 @@
         <v/>
       </c>
       <c r="AA9" s="7">
-        <f>AC9*Inputs!$C$46+AD9*Inputs!$B$35+AE9*Inputs!$B$36</f>
+        <f>AC9*Inputs!$C$47+AD9*Inputs!$B$36+AE9*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB9" t="inlineStr">
@@ -3212,7 +3240,7 @@
         <v/>
       </c>
       <c r="X10" s="7">
-        <f>AC10*Inputs!$B$45+AD10*Inputs!$B$35+AE10*Inputs!$B$36</f>
+        <f>AC10*Inputs!$B$46+AD10*Inputs!$B$36+AE10*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y10" s="5">
@@ -3224,7 +3252,7 @@
         <v/>
       </c>
       <c r="AA10" s="7">
-        <f>AC10*Inputs!$C$46+AD10*Inputs!$B$35+AE10*Inputs!$B$36</f>
+        <f>AC10*Inputs!$C$47+AD10*Inputs!$B$36+AE10*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB10" t="inlineStr">
@@ -3337,7 +3365,7 @@
         <v/>
       </c>
       <c r="X11" s="7">
-        <f>AC11*Inputs!$B$45+AD11*Inputs!$B$35+AE11*Inputs!$B$36</f>
+        <f>AC11*Inputs!$B$46+AD11*Inputs!$B$36+AE11*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y11" s="5">
@@ -3349,7 +3377,7 @@
         <v/>
       </c>
       <c r="AA11" s="7">
-        <f>AC11*Inputs!$C$46+AD11*Inputs!$B$35+AE11*Inputs!$B$36</f>
+        <f>AC11*Inputs!$C$47+AD11*Inputs!$B$36+AE11*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB11" t="inlineStr">
@@ -3441,11 +3469,11 @@
         <v/>
       </c>
       <c r="L13" s="5">
-        <f>J13*Inputs!$B$41</f>
+        <f>J13*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M13" s="5">
-        <f>K13*Inputs!$C$41</f>
+        <f>K13*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N13" t="inlineStr">
@@ -3490,7 +3518,7 @@
         <v/>
       </c>
       <c r="X13" s="7">
-        <f>AC13*Inputs!$B$45+AD13*Inputs!$B$35+AE13*Inputs!$B$36</f>
+        <f>AC13*Inputs!$B$46+AD13*Inputs!$B$36+AE13*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y13" s="5">
@@ -3502,7 +3530,7 @@
         <v/>
       </c>
       <c r="AA13" s="7">
-        <f>AC13*Inputs!$C$46+AD13*Inputs!$B$35+AE13*Inputs!$B$36</f>
+        <f>AC13*Inputs!$C$47+AD13*Inputs!$B$36+AE13*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB13" t="inlineStr">
@@ -3566,11 +3594,11 @@
         <v/>
       </c>
       <c r="L14" s="5">
-        <f>J14*Inputs!$B$41</f>
+        <f>J14*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M14" s="5">
-        <f>K14*Inputs!$C$41</f>
+        <f>K14*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N14" t="inlineStr">
@@ -3615,7 +3643,7 @@
         <v/>
       </c>
       <c r="X14" s="7">
-        <f>AC14*Inputs!$B$45+AD14*Inputs!$B$35+AE14*Inputs!$B$36</f>
+        <f>AC14*Inputs!$B$46+AD14*Inputs!$B$36+AE14*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y14" s="5">
@@ -3627,7 +3655,7 @@
         <v/>
       </c>
       <c r="AA14" s="7">
-        <f>AC14*Inputs!$C$46+AD14*Inputs!$B$35+AE14*Inputs!$B$36</f>
+        <f>AC14*Inputs!$C$47+AD14*Inputs!$B$36+AE14*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB14" t="inlineStr">
@@ -3691,11 +3719,11 @@
         <v/>
       </c>
       <c r="L15" s="5">
-        <f>J15*Inputs!$B$41</f>
+        <f>J15*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M15" s="5">
-        <f>K15*Inputs!$C$41</f>
+        <f>K15*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N15" t="inlineStr">
@@ -3740,7 +3768,7 @@
         <v/>
       </c>
       <c r="X15" s="7">
-        <f>AC15*Inputs!$B$45+AD15*Inputs!$B$35+AE15*Inputs!$B$36</f>
+        <f>AC15*Inputs!$B$46+AD15*Inputs!$B$36+AE15*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y15" s="5">
@@ -3752,7 +3780,7 @@
         <v/>
       </c>
       <c r="AA15" s="7">
-        <f>AC15*Inputs!$C$46+AD15*Inputs!$B$35+AE15*Inputs!$B$36</f>
+        <f>AC15*Inputs!$C$47+AD15*Inputs!$B$36+AE15*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB15" t="inlineStr">
@@ -3799,7 +3827,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="6">
-        <f>Inputs!$B$43</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="H16" s="6" t="n">
@@ -3817,11 +3845,11 @@
         <v/>
       </c>
       <c r="L16" s="5">
-        <f>J16*Inputs!$B$41</f>
+        <f>J16*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M16" s="5">
-        <f>K16*Inputs!$C$41</f>
+        <f>K16*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N16" t="inlineStr">
@@ -3866,7 +3894,7 @@
         <v/>
       </c>
       <c r="X16" s="7">
-        <f>AC16*Inputs!$B$45+AD16*Inputs!$B$35+AE16*Inputs!$B$36</f>
+        <f>AC16*Inputs!$B$46+AD16*Inputs!$B$36+AE16*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y16" s="5">
@@ -3878,7 +3906,7 @@
         <v/>
       </c>
       <c r="AA16" s="7">
-        <f>AC16*Inputs!$C$46+AD16*Inputs!$B$35+AE16*Inputs!$B$36</f>
+        <f>AC16*Inputs!$C$47+AD16*Inputs!$B$36+AE16*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB16" t="inlineStr">
@@ -3906,11 +3934,11 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>Inputs!$B$34*Inputs!$B$2</f>
+        <f>Inputs!$B$35*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>Inputs!$C$34*Inputs!$C$2</f>
+        <f>Inputs!$C$35*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D17" s="5">
@@ -3942,11 +3970,11 @@
         <v/>
       </c>
       <c r="L17" s="5">
-        <f>J17*Inputs!$B$41</f>
+        <f>J17*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M17" s="5">
-        <f>K17*Inputs!$C$41</f>
+        <f>K17*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N17" t="inlineStr">
@@ -3991,7 +4019,7 @@
         <v/>
       </c>
       <c r="X17" s="7">
-        <f>AC17*Inputs!$B$45+AD17*Inputs!$B$35+AE17*Inputs!$B$36</f>
+        <f>AC17*Inputs!$B$46+AD17*Inputs!$B$36+AE17*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y17" s="5">
@@ -4003,7 +4031,7 @@
         <v/>
       </c>
       <c r="AA17" s="7">
-        <f>AC17*Inputs!$C$46+AD17*Inputs!$B$35+AE17*Inputs!$B$36</f>
+        <f>AC17*Inputs!$C$47+AD17*Inputs!$B$36+AE17*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB17" t="inlineStr">
@@ -4116,7 +4144,7 @@
         <v/>
       </c>
       <c r="X18" s="7">
-        <f>AC18*Inputs!$B$45+AD18*Inputs!$B$35+AE18*Inputs!$B$36</f>
+        <f>AC18*Inputs!$B$46+AD18*Inputs!$B$36+AE18*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y18" s="5">
@@ -4128,7 +4156,7 @@
         <v/>
       </c>
       <c r="AA18" s="7">
-        <f>AC18*Inputs!$C$46+AD18*Inputs!$B$35+AE18*Inputs!$B$36</f>
+        <f>AC18*Inputs!$C$47+AD18*Inputs!$B$36+AE18*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB18" t="inlineStr">
@@ -4241,7 +4269,7 @@
         <v/>
       </c>
       <c r="X19" s="7">
-        <f>AC19*Inputs!$B$45+AD19*Inputs!$B$35+AE19*Inputs!$B$36</f>
+        <f>AC19*Inputs!$B$46+AD19*Inputs!$B$36+AE19*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y19" s="5">
@@ -4253,7 +4281,7 @@
         <v/>
       </c>
       <c r="AA19" s="7">
-        <f>AC19*Inputs!$C$46+AD19*Inputs!$B$35+AE19*Inputs!$B$36</f>
+        <f>AC19*Inputs!$C$47+AD19*Inputs!$B$36+AE19*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB19" t="inlineStr">
@@ -4366,7 +4394,7 @@
         <v/>
       </c>
       <c r="X20" s="7">
-        <f>AC20*Inputs!$B$45+AD20*Inputs!$B$35+AE20*Inputs!$B$36</f>
+        <f>AC20*Inputs!$B$46+AD20*Inputs!$B$36+AE20*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y20" s="5">
@@ -4378,7 +4406,7 @@
         <v/>
       </c>
       <c r="AA20" s="7">
-        <f>AC20*Inputs!$C$46+AD20*Inputs!$B$35+AE20*Inputs!$B$36</f>
+        <f>AC20*Inputs!$C$47+AD20*Inputs!$B$36+AE20*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB20" t="inlineStr">
@@ -4424,14 +4452,15 @@
       <c r="F21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="6" t="n">
-        <v>0</v>
+      <c r="G21" s="6">
+        <f>Inputs!$B$29</f>
+        <v/>
       </c>
       <c r="H21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="6">
-        <f>Inputs!$B$29</f>
+        <f>Inputs!$B$30</f>
         <v/>
       </c>
       <c r="J21" s="5">
@@ -4443,16 +4472,16 @@
         <v/>
       </c>
       <c r="L21" s="5">
-        <f>J21*Inputs!$B$41</f>
+        <f>J21*Inputs!$B$42</f>
         <v/>
       </c>
       <c r="M21" s="5">
-        <f>K21*Inputs!$C$41</f>
+        <f>K21*Inputs!$C$42</f>
         <v/>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Server and equipment enclosures only (40% of IT mass, estimate); electronics never. Rack masses [H]; aggregate [L]</t>
+          <t>Rack cabinets soon (18% of IT mass), server enclosures long term (22%), estimates; electronics never. Rack masses [H]; aggregate [L]</t>
         </is>
       </c>
       <c r="O21" s="5">
@@ -4492,7 +4521,7 @@
         <v/>
       </c>
       <c r="X21" s="7">
-        <f>AC21*Inputs!$B$45+AD21*Inputs!$B$35+AE21*Inputs!$B$36</f>
+        <f>AC21*Inputs!$B$46+AD21*Inputs!$B$36+AE21*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="Y21" s="5">
@@ -4504,7 +4533,7 @@
         <v/>
       </c>
       <c r="AA21" s="7">
-        <f>AC21*Inputs!$C$46+AD21*Inputs!$B$35+AE21*Inputs!$B$36</f>
+        <f>AC21*Inputs!$C$47+AD21*Inputs!$B$36+AE21*Inputs!$B$37</f>
         <v/>
       </c>
       <c r="AB21" t="inlineStr">
@@ -5111,11 +5140,11 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>Inputs!$B$37/1000*Inputs!$B$38*0.092903</f>
+        <f>Inputs!$B$38/1000*Inputs!$B$39*0.092903</f>
         <v/>
       </c>
       <c r="C6" s="15">
-        <f>Inputs!$C$37/1000*Inputs!$C$38*0.092903</f>
+        <f>Inputs!$C$38/1000*Inputs!$C$39*0.092903</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -5131,11 +5160,11 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>Inputs!$B$39*B6/1000</f>
+        <f>Inputs!$B$40*B6/1000</f>
         <v/>
       </c>
       <c r="C7" s="15">
-        <f>Inputs!$C$39*C6/1000</f>
+        <f>Inputs!$C$40*C6/1000</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -5151,11 +5180,11 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>Inputs!$B$40*B6/1000</f>
+        <f>Inputs!$B$41*B6/1000</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>Inputs!$C$40*C6/1000</f>
+        <f>Inputs!$C$41*C6/1000</f>
         <v/>
       </c>
       <c r="D8" t="inlineStr">
@@ -5263,11 +5292,11 @@
         <v/>
       </c>
       <c r="D2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$47</f>
+        <f>'1 GW data center'!B29*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="E2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$47</f>
+        <f>'1 GW data center'!C29*Inputs!$C$48</f>
         <v/>
       </c>
       <c r="F2" s="4">
@@ -5287,11 +5316,11 @@
         <v/>
       </c>
       <c r="J2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$48</f>
+        <f>'1 GW data center'!B29*Inputs!$B$49</f>
         <v/>
       </c>
       <c r="K2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$48</f>
+        <f>'1 GW data center'!C29*Inputs!$C$49</f>
         <v/>
       </c>
     </row>
@@ -5310,11 +5339,11 @@
         <v/>
       </c>
       <c r="D3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$47</f>
+        <f>'1 GW data center'!B34*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="E3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$47</f>
+        <f>'1 GW data center'!C34*Inputs!$C$48</f>
         <v/>
       </c>
       <c r="F3" s="4">
@@ -5334,11 +5363,11 @@
         <v/>
       </c>
       <c r="J3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$48</f>
+        <f>'1 GW data center'!B34*Inputs!$B$49</f>
         <v/>
       </c>
       <c r="K3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$48</f>
+        <f>'1 GW data center'!C34*Inputs!$C$49</f>
         <v/>
       </c>
     </row>
@@ -5357,11 +5386,11 @@
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$47</f>
+        <f>'1 GW data center'!B38*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$47</f>
+        <f>'1 GW data center'!C38*Inputs!$C$48</f>
         <v/>
       </c>
       <c r="F4" s="4">
@@ -5381,11 +5410,11 @@
         <v/>
       </c>
       <c r="J4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$48</f>
+        <f>'1 GW data center'!B38*Inputs!$B$49</f>
         <v/>
       </c>
       <c r="K4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$48</f>
+        <f>'1 GW data center'!C38*Inputs!$C$49</f>
         <v/>
       </c>
     </row>
@@ -5404,11 +5433,11 @@
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$47</f>
+        <f>'1 GW data center'!B42*Inputs!$B$48</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$47</f>
+        <f>'1 GW data center'!C42*Inputs!$C$48</f>
         <v/>
       </c>
       <c r="F5" s="4">
@@ -5428,11 +5457,11 @@
         <v/>
       </c>
       <c r="J5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$48</f>
+        <f>'1 GW data center'!B42*Inputs!$B$49</f>
         <v/>
       </c>
       <c r="K5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$48</f>
+        <f>'1 GW data center'!C42*Inputs!$C$49</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
DC investor deck: loaded-rack analysis applied; mechanical shells medium term, fan blades long term
Alex 2026-09-06. IT row 50% steel / 8% plastic / 42% other; rack
cabinets 18% soon, server enclosures 30% long. Mechanical shells,
casings and fan-wall frames 25% medium term; fan blades 2% long term,
needs investigation. Workbook v11, split file, both decks, slide 7
figures, PPTX charts and register updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1423,42 +1423,42 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IT: servers and racks</t>
+          <t>Share of mechanical mass that is equipment shells, casings and fan-wall frames — SUPERWOOD in the medium term</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>15</v>
+        <v>0.25</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>70</v>
+        <v>0.25</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>t/MW</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>estimated [L]; Alex 2026-09-06</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Loaded rack ~1 t; GB200 NVL72 ~1.36 t [H]</t>
+          <t>About half of the steel in the row; compressor and pump bodies, tubes and steel piping excluded</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Share of IT mass that is server rack cabinets (frames, panels, doors) — substitutable soon</t>
+          <t>Share of mechanical mass that is fan blades — long term, needs investigation</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>0.18</v>
+        <v>0.02</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.18</v>
+        <v>0.02</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1472,49 +1472,49 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>A loaded rack of 1–1.4 t carries a 150–250 kg steel cabinet</t>
+          <t>Aluminum or composite blades today; SUPERWOOD blades are a research question</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Share of IT mass that is server enclosures (chassis) — long term</t>
+          <t>IT: servers and racks</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>0.22</v>
+        <v>15</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.22</v>
+        <v>70</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>t/MW</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>estimated [L]; Alex 2026-09-04/06</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Server boxes eventually; the electronics never</t>
+          <t>Loaded rack ~1 t; GB200 NVL72 ~1.36 t [H]</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
+          <t>Share of IT mass that is server rack cabinets (frames, panels, doors) — substitutable soon</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>0.4</v>
+        <v>0.18</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.5</v>
+        <v>0.18</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1523,26 +1523,26 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>estimated [L]; Alex 2026-09-06</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Remainder is slab on grade, paving and yard</t>
+          <t>A loaded rack of 1–1.4 t carries a 150–250 kg steel cabinet</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
+          <t>Share of IT mass that is server enclosures (sheet-steel chassis) — long term</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>0.75</v>
+        <v>0.3</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.75</v>
+        <v>0.3</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1551,26 +1551,26 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
+          <t>estimated [M]; analyses/it-rack-material-stack.md, applied 2026-09-06</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan; no design or code pathway yet</t>
+          <t>Server boxes eventually; the electronics never</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
+          <t>Share of all concrete that is foundations, footings, piers and equipment pads</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1579,195 +1579,203 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Technical potential, not a plan</t>
+          <t>Remainder is slab on grade, paving and yard</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>kg SUPERWOOD per kg of concrete replaced</t>
+          <t>Long-term technical potential: share of slab-on-grade and paving concrete replaceable</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.15</v>
+        <v>0.75</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
+          <t>Technical potential, not a plan; no design or code pathway yet</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ducting, plenums and air-distribution sheet metal</t>
+          <t>Long-term technical potential: share of foundations, footings, piers and pads replaceable</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>3</v>
+        <v>0.9</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>8</v>
+        <v>0.9</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>t/MW</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
+          <t>asserted-internal (Alex, 2026-09-01) [L]</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Separate from the mechanical-equipment row</t>
+          <t>Technical potential, not a plan</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Concrete emissions</t>
+          <t>kg SUPERWOOD per kg of concrete replaced</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>0.12</v>
+        <v>0.05</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
+          <t>Lightweight insulated wood-foundation concept; no design exists yet</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Polymers in paints, foam cores and plastic trim (average)</t>
+          <t>Ducting, plenums and air-distribution sheet metal</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>t/MW</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>industry range [M]; Alex 2026-09-05</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Cradle to gate; polyolefins and PVC about 2–2.5, polyurethane foam 3–4, coatings higher</t>
+          <t>Separate from the mechanical-equipment row</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SUPERWOOD average board thickness</t>
+          <t>Concrete emissions</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>7.2</v>
+        <v>0.12</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>7.2</v>
+        <v>0.12</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>internal TEM basis [H]</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Ready-mix, cradle to gate; typical 0.10–0.15</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SUPERWOOD density</t>
+          <t>Polymers in paints, foam cores and plastic trim (average)</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>1300</v>
+        <v>3</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>1300</v>
+        <v>3</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>kg/m³</t>
+          <t>kg CO₂e/kg</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>internal TEM [H]</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>industry range [M]; Alex 2026-09-05</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Cradle to gate; polyolefins and PVC about 2–2.5, polyurethane foam 3–4, coatings higher</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SuperMill One output</t>
+          <t>SUPERWOOD average board thickness</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>1000000</v>
+        <v>7.2</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>1000000</v>
+        <v>7.2</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>sf/yr</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>internal [H]</t>
+          <t>internal TEM basis [H]</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -1775,23 +1783,23 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SuperMill Two output</t>
+          <t>SUPERWOOD density</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>36000000</v>
+        <v>1300</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>36000000</v>
+        <v>1300</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>sf/yr</t>
+          <t>kg/m³</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>internal [H]</t>
+          <t>internal TEM [H]</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -1799,74 +1807,66 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
+          <t>SuperMill One output</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0.3</v>
+        <v>1000000</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0.6</v>
+        <v>1000000</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>kg/kg</t>
+          <t>sf/yr</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
-        </is>
-      </c>
+          <t>internal [H]</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
+          <t>SuperMill Two output</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>20</v>
+        <v>36000000</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>40</v>
+        <v>36000000</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>kg/m²</t>
+          <t>sf/yr</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>estimated [L]</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Panel design unsettled</t>
-        </is>
-      </c>
+          <t>internal [H]</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Addressable share of other tray / containment / doors (medium term)</t>
+          <t>Structural substitution: kg SUPERWOOD per kg steel replaced</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>kg/kg</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1874,56 +1874,60 @@
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Engineering-stamped per element (Fast + Epp) before external use</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Count rebar as addressable in the long term? (0/1)</t>
+          <t>SUPERWOOD in a hybrid wall panel replacing precast</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>kg/m²</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Rebar is a frontier market with no pathway; off by default</t>
+          <t>Panel design unsettled</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Steel emissions, global average (BF-BOF)</t>
+          <t>Addressable share of other tray / containment / doors (medium term)</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>1.8</v>
+        <v>0.5</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>1.8</v>
+        <v>0.5</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>published-class [M]</t>
+          <t>estimated [L]</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -1931,38 +1935,42 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Steel emissions, recycled (EAF)</t>
+          <t>Count rebar as addressable in the long term? (0/1)</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Rebar is a frontier market with no pathway; off by default</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SUPERWOOD manufacturing emissions</t>
+          <t>Steel emissions, global average (BF-BOF)</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>0.5</v>
+        <v>1.8</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0.5</v>
+        <v>1.8</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1971,26 +1979,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
-        </is>
-      </c>
+          <t>published-class [M]</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SUPERWOOD biogenic carbon stored</t>
+          <t>Steel emissions, recycled (EAF)</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>1.3</v>
+        <v>0.4</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1999,38 +2003,90 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Report separately; module C release under EN 15804</t>
-        </is>
-      </c>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>SUPERWOOD manufacturing emissions</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>internal, pre-LCA [L]</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SUPERWOOD biogenic carbon stored</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>internal, pre-LCA [L]</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Report separately; module C release under EN 15804</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
         </is>
       </c>
-      <c r="B50" s="2" t="n">
+      <c r="B52" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C50" s="2" t="n">
+      <c r="C52" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>kg CO₂e/kg</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Used only for the interior finishes row</t>
         </is>
@@ -2277,11 +2333,11 @@
         </is>
       </c>
       <c r="B3" s="5">
-        <f>Inputs!$B$11*(1-Inputs!$B$31)*Inputs!$B$12*Inputs!$B$2-B5</f>
+        <f>Inputs!$B$11*(1-Inputs!$B$33)*Inputs!$B$12*Inputs!$B$2-B5</f>
         <v/>
       </c>
       <c r="C3" s="5">
-        <f>Inputs!$C$11*(1-Inputs!$C$31)*Inputs!$C$12*Inputs!$C$2-C5</f>
+        <f>Inputs!$C$11*(1-Inputs!$C$33)*Inputs!$C$12*Inputs!$C$2-C5</f>
         <v/>
       </c>
       <c r="D3" s="5">
@@ -2302,7 +2358,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="6">
-        <f>Inputs!$B$32</f>
+        <f>Inputs!$B$34</f>
         <v/>
       </c>
       <c r="J3" s="5">
@@ -2314,11 +2370,11 @@
         <v/>
       </c>
       <c r="L3" s="5">
-        <f>J3*Inputs!$B$34</f>
+        <f>J3*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="M3" s="5">
-        <f>K3*Inputs!$C$34</f>
+        <f>K3*Inputs!$C$36</f>
         <v/>
       </c>
       <c r="N3" t="inlineStr">
@@ -2363,7 +2419,7 @@
         <v/>
       </c>
       <c r="X3" s="7">
-        <f>AC3*Inputs!$B$46+AD3*Inputs!$B$36+AE3*Inputs!$B$37</f>
+        <f>AC3*Inputs!$B$48+AD3*Inputs!$B$38+AE3*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y3" s="5">
@@ -2375,7 +2431,7 @@
         <v/>
       </c>
       <c r="AA3" s="7">
-        <f>AC3*Inputs!$C$47+AD3*Inputs!$B$36+AE3*Inputs!$B$37</f>
+        <f>AC3*Inputs!$C$49+AD3*Inputs!$B$38+AE3*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB3" t="inlineStr">
@@ -2403,11 +2459,11 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>Inputs!$B$11*Inputs!$B$31*Inputs!$B$12*Inputs!$B$2</f>
+        <f>Inputs!$B$11*Inputs!$B$33*Inputs!$B$12*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C4" s="5">
-        <f>Inputs!$C$11*Inputs!$C$31*Inputs!$C$12*Inputs!$C$2</f>
+        <f>Inputs!$C$11*Inputs!$C$33*Inputs!$C$12*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D4" s="5">
@@ -2428,7 +2484,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="6">
-        <f>Inputs!$B$33</f>
+        <f>Inputs!$B$35</f>
         <v/>
       </c>
       <c r="J4" s="5">
@@ -2440,11 +2496,11 @@
         <v/>
       </c>
       <c r="L4" s="5">
-        <f>J4*Inputs!$B$34</f>
+        <f>J4*Inputs!$B$36</f>
         <v/>
       </c>
       <c r="M4" s="5">
-        <f>K4*Inputs!$C$34</f>
+        <f>K4*Inputs!$C$36</f>
         <v/>
       </c>
       <c r="N4" t="inlineStr">
@@ -2489,7 +2545,7 @@
         <v/>
       </c>
       <c r="X4" s="7">
-        <f>AC4*Inputs!$B$46+AD4*Inputs!$B$36+AE4*Inputs!$B$37</f>
+        <f>AC4*Inputs!$B$48+AD4*Inputs!$B$38+AE4*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y4" s="5">
@@ -2501,7 +2557,7 @@
         <v/>
       </c>
       <c r="AA4" s="7">
-        <f>AC4*Inputs!$C$47+AD4*Inputs!$B$36+AE4*Inputs!$B$37</f>
+        <f>AC4*Inputs!$C$49+AD4*Inputs!$B$38+AE4*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB4" t="inlineStr">
@@ -2565,11 +2621,11 @@
         <v/>
       </c>
       <c r="L5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$43/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$B$13*Derived!B4*Inputs!$B$45/1000</f>
         <v/>
       </c>
       <c r="M5" s="5">
-        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$43/1000</f>
+        <f>SUM($F5:$I5)*Inputs!$C$13*Derived!C4*Inputs!$C$45/1000</f>
         <v/>
       </c>
       <c r="N5" t="inlineStr">
@@ -2614,7 +2670,7 @@
         <v/>
       </c>
       <c r="X5" s="7">
-        <f>AC5*Inputs!$B$46+AD5*Inputs!$B$36+AE5*Inputs!$B$37</f>
+        <f>AC5*Inputs!$B$48+AD5*Inputs!$B$38+AE5*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y5" s="5">
@@ -2626,7 +2682,7 @@
         <v/>
       </c>
       <c r="AA5" s="7">
-        <f>AC5*Inputs!$C$47+AD5*Inputs!$B$36+AE5*Inputs!$B$37</f>
+        <f>AC5*Inputs!$C$49+AD5*Inputs!$B$38+AE5*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB5" t="inlineStr">
@@ -2679,7 +2735,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="6">
-        <f>Inputs!$B$31*Inputs!$B$33+(1-Inputs!$B$31)*Inputs!$B$32</f>
+        <f>Inputs!$B$33*Inputs!$B$35+(1-Inputs!$B$33)*Inputs!$B$34</f>
         <v/>
       </c>
       <c r="J6" s="5">
@@ -2691,11 +2747,11 @@
         <v/>
       </c>
       <c r="L6" s="5">
-        <f>J6*Inputs!$B$42</f>
+        <f>J6*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M6" s="5">
-        <f>K6*Inputs!$C$42</f>
+        <f>K6*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N6" t="inlineStr">
@@ -2740,7 +2796,7 @@
         <v/>
       </c>
       <c r="X6" s="7">
-        <f>AC6*Inputs!$B$46+AD6*Inputs!$B$36+AE6*Inputs!$B$37</f>
+        <f>AC6*Inputs!$B$48+AD6*Inputs!$B$38+AE6*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y6" s="5">
@@ -2752,7 +2808,7 @@
         <v/>
       </c>
       <c r="AA6" s="7">
-        <f>AC6*Inputs!$C$47+AD6*Inputs!$B$36+AE6*Inputs!$B$37</f>
+        <f>AC6*Inputs!$C$49+AD6*Inputs!$B$38+AE6*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB6" t="inlineStr">
@@ -2816,11 +2872,11 @@
         <v/>
       </c>
       <c r="L7" s="5">
-        <f>J7*Inputs!$B$42</f>
+        <f>J7*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M7" s="5">
-        <f>K7*Inputs!$C$42</f>
+        <f>K7*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N7" t="inlineStr">
@@ -2865,7 +2921,7 @@
         <v/>
       </c>
       <c r="X7" s="7">
-        <f>AC7*Inputs!$B$46+AD7*Inputs!$B$36+AE7*Inputs!$B$37</f>
+        <f>AC7*Inputs!$B$48+AD7*Inputs!$B$38+AE7*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y7" s="5">
@@ -2877,7 +2933,7 @@
         <v/>
       </c>
       <c r="AA7" s="7">
-        <f>AC7*Inputs!$C$47+AD7*Inputs!$B$36+AE7*Inputs!$B$37</f>
+        <f>AC7*Inputs!$C$49+AD7*Inputs!$B$38+AE7*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB7" t="inlineStr">
@@ -2941,11 +2997,11 @@
         <v/>
       </c>
       <c r="L8" s="5">
-        <f>J8*Inputs!$B$42</f>
+        <f>J8*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M8" s="5">
-        <f>K8*Inputs!$C$42</f>
+        <f>K8*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N8" t="inlineStr">
@@ -2990,7 +3046,7 @@
         <v/>
       </c>
       <c r="X8" s="7">
-        <f>AC8*Inputs!$B$46+AD8*Inputs!$B$36+AE8*Inputs!$B$37</f>
+        <f>AC8*Inputs!$B$48+AD8*Inputs!$B$38+AE8*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y8" s="5">
@@ -3002,7 +3058,7 @@
         <v/>
       </c>
       <c r="AA8" s="7">
-        <f>AC8*Inputs!$C$47+AD8*Inputs!$B$36+AE8*Inputs!$B$37</f>
+        <f>AC8*Inputs!$C$49+AD8*Inputs!$B$38+AE8*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB8" t="inlineStr">
@@ -3115,7 +3171,7 @@
         <v/>
       </c>
       <c r="X9" s="7">
-        <f>AC9*Inputs!$B$46+AD9*Inputs!$B$36+AE9*Inputs!$B$37</f>
+        <f>AC9*Inputs!$B$48+AD9*Inputs!$B$38+AE9*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y9" s="5">
@@ -3127,7 +3183,7 @@
         <v/>
       </c>
       <c r="AA9" s="7">
-        <f>AC9*Inputs!$C$47+AD9*Inputs!$B$36+AE9*Inputs!$B$37</f>
+        <f>AC9*Inputs!$C$49+AD9*Inputs!$B$38+AE9*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB9" t="inlineStr">
@@ -3240,7 +3296,7 @@
         <v/>
       </c>
       <c r="X10" s="7">
-        <f>AC10*Inputs!$B$46+AD10*Inputs!$B$36+AE10*Inputs!$B$37</f>
+        <f>AC10*Inputs!$B$48+AD10*Inputs!$B$38+AE10*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y10" s="5">
@@ -3252,7 +3308,7 @@
         <v/>
       </c>
       <c r="AA10" s="7">
-        <f>AC10*Inputs!$C$47+AD10*Inputs!$B$36+AE10*Inputs!$B$37</f>
+        <f>AC10*Inputs!$C$49+AD10*Inputs!$B$38+AE10*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB10" t="inlineStr">
@@ -3365,7 +3421,7 @@
         <v/>
       </c>
       <c r="X11" s="7">
-        <f>AC11*Inputs!$B$46+AD11*Inputs!$B$36+AE11*Inputs!$B$37</f>
+        <f>AC11*Inputs!$B$48+AD11*Inputs!$B$38+AE11*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y11" s="5">
@@ -3377,7 +3433,7 @@
         <v/>
       </c>
       <c r="AA11" s="7">
-        <f>AC11*Inputs!$C$47+AD11*Inputs!$B$36+AE11*Inputs!$B$37</f>
+        <f>AC11*Inputs!$C$49+AD11*Inputs!$B$38+AE11*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB11" t="inlineStr">
@@ -3469,11 +3525,11 @@
         <v/>
       </c>
       <c r="L13" s="5">
-        <f>J13*Inputs!$B$42</f>
+        <f>J13*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M13" s="5">
-        <f>K13*Inputs!$C$42</f>
+        <f>K13*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N13" t="inlineStr">
@@ -3518,7 +3574,7 @@
         <v/>
       </c>
       <c r="X13" s="7">
-        <f>AC13*Inputs!$B$46+AD13*Inputs!$B$36+AE13*Inputs!$B$37</f>
+        <f>AC13*Inputs!$B$48+AD13*Inputs!$B$38+AE13*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y13" s="5">
@@ -3530,7 +3586,7 @@
         <v/>
       </c>
       <c r="AA13" s="7">
-        <f>AC13*Inputs!$C$47+AD13*Inputs!$B$36+AE13*Inputs!$B$37</f>
+        <f>AC13*Inputs!$C$49+AD13*Inputs!$B$38+AE13*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB13" t="inlineStr">
@@ -3594,11 +3650,11 @@
         <v/>
       </c>
       <c r="L14" s="5">
-        <f>J14*Inputs!$B$42</f>
+        <f>J14*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M14" s="5">
-        <f>K14*Inputs!$C$42</f>
+        <f>K14*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N14" t="inlineStr">
@@ -3643,7 +3699,7 @@
         <v/>
       </c>
       <c r="X14" s="7">
-        <f>AC14*Inputs!$B$46+AD14*Inputs!$B$36+AE14*Inputs!$B$37</f>
+        <f>AC14*Inputs!$B$48+AD14*Inputs!$B$38+AE14*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y14" s="5">
@@ -3655,7 +3711,7 @@
         <v/>
       </c>
       <c r="AA14" s="7">
-        <f>AC14*Inputs!$C$47+AD14*Inputs!$B$36+AE14*Inputs!$B$37</f>
+        <f>AC14*Inputs!$C$49+AD14*Inputs!$B$38+AE14*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB14" t="inlineStr">
@@ -3719,11 +3775,11 @@
         <v/>
       </c>
       <c r="L15" s="5">
-        <f>J15*Inputs!$B$42</f>
+        <f>J15*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M15" s="5">
-        <f>K15*Inputs!$C$42</f>
+        <f>K15*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N15" t="inlineStr">
@@ -3768,7 +3824,7 @@
         <v/>
       </c>
       <c r="X15" s="7">
-        <f>AC15*Inputs!$B$46+AD15*Inputs!$B$36+AE15*Inputs!$B$37</f>
+        <f>AC15*Inputs!$B$48+AD15*Inputs!$B$38+AE15*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y15" s="5">
@@ -3780,7 +3836,7 @@
         <v/>
       </c>
       <c r="AA15" s="7">
-        <f>AC15*Inputs!$C$47+AD15*Inputs!$B$36+AE15*Inputs!$B$37</f>
+        <f>AC15*Inputs!$C$49+AD15*Inputs!$B$38+AE15*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB15" t="inlineStr">
@@ -3827,7 +3883,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="6">
-        <f>Inputs!$B$44</f>
+        <f>Inputs!$B$46</f>
         <v/>
       </c>
       <c r="H16" s="6" t="n">
@@ -3845,11 +3901,11 @@
         <v/>
       </c>
       <c r="L16" s="5">
-        <f>J16*Inputs!$B$42</f>
+        <f>J16*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M16" s="5">
-        <f>K16*Inputs!$C$42</f>
+        <f>K16*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N16" t="inlineStr">
@@ -3894,7 +3950,7 @@
         <v/>
       </c>
       <c r="X16" s="7">
-        <f>AC16*Inputs!$B$46+AD16*Inputs!$B$36+AE16*Inputs!$B$37</f>
+        <f>AC16*Inputs!$B$48+AD16*Inputs!$B$38+AE16*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y16" s="5">
@@ -3906,7 +3962,7 @@
         <v/>
       </c>
       <c r="AA16" s="7">
-        <f>AC16*Inputs!$C$47+AD16*Inputs!$B$36+AE16*Inputs!$B$37</f>
+        <f>AC16*Inputs!$C$49+AD16*Inputs!$B$38+AE16*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB16" t="inlineStr">
@@ -3934,11 +3990,11 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>Inputs!$B$35*Inputs!$B$2</f>
+        <f>Inputs!$B$37*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>Inputs!$C$35*Inputs!$C$2</f>
+        <f>Inputs!$C$37*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D17" s="5">
@@ -3970,11 +4026,11 @@
         <v/>
       </c>
       <c r="L17" s="5">
-        <f>J17*Inputs!$B$42</f>
+        <f>J17*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M17" s="5">
-        <f>K17*Inputs!$C$42</f>
+        <f>K17*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N17" t="inlineStr">
@@ -4019,7 +4075,7 @@
         <v/>
       </c>
       <c r="X17" s="7">
-        <f>AC17*Inputs!$B$46+AD17*Inputs!$B$36+AE17*Inputs!$B$37</f>
+        <f>AC17*Inputs!$B$48+AD17*Inputs!$B$38+AE17*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y17" s="5">
@@ -4031,7 +4087,7 @@
         <v/>
       </c>
       <c r="AA17" s="7">
-        <f>AC17*Inputs!$C$47+AD17*Inputs!$B$36+AE17*Inputs!$B$37</f>
+        <f>AC17*Inputs!$C$49+AD17*Inputs!$B$38+AE17*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB17" t="inlineStr">
@@ -4144,7 +4200,7 @@
         <v/>
       </c>
       <c r="X18" s="7">
-        <f>AC18*Inputs!$B$46+AD18*Inputs!$B$36+AE18*Inputs!$B$37</f>
+        <f>AC18*Inputs!$B$48+AD18*Inputs!$B$38+AE18*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y18" s="5">
@@ -4156,7 +4212,7 @@
         <v/>
       </c>
       <c r="AA18" s="7">
-        <f>AC18*Inputs!$C$47+AD18*Inputs!$B$36+AE18*Inputs!$B$37</f>
+        <f>AC18*Inputs!$C$49+AD18*Inputs!$B$38+AE18*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB18" t="inlineStr">
@@ -4269,7 +4325,7 @@
         <v/>
       </c>
       <c r="X19" s="7">
-        <f>AC19*Inputs!$B$46+AD19*Inputs!$B$36+AE19*Inputs!$B$37</f>
+        <f>AC19*Inputs!$B$48+AD19*Inputs!$B$38+AE19*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y19" s="5">
@@ -4281,7 +4337,7 @@
         <v/>
       </c>
       <c r="AA19" s="7">
-        <f>AC19*Inputs!$C$47+AD19*Inputs!$B$36+AE19*Inputs!$B$37</f>
+        <f>AC19*Inputs!$C$49+AD19*Inputs!$B$38+AE19*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB19" t="inlineStr">
@@ -4330,11 +4386,13 @@
       <c r="G20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="6" t="n">
-        <v>0</v>
+      <c r="H20" s="6">
+        <f>Inputs!$B$28</f>
+        <v/>
+      </c>
+      <c r="I20" s="6">
+        <f>Inputs!$B$29</f>
+        <v/>
       </c>
       <c r="J20" s="5">
         <f>B20*SUM($F20:$I20)</f>
@@ -4345,16 +4403,16 @@
         <v/>
       </c>
       <c r="L20" s="5">
-        <f>0</f>
+        <f>J20*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M20" s="5">
-        <f>0</f>
+        <f>K20*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Chillers, fan walls, coolers, piping (ductwork is its own row)</t>
+          <t>Shells, casings and fan-wall frames medium term (Alex 2026-09-06); fan blades long term, needs investigation; compressors, pumps, tubes, piping and water stay</t>
         </is>
       </c>
       <c r="O20" s="5">
@@ -4394,7 +4452,7 @@
         <v/>
       </c>
       <c r="X20" s="7">
-        <f>AC20*Inputs!$B$46+AD20*Inputs!$B$36+AE20*Inputs!$B$37</f>
+        <f>AC20*Inputs!$B$48+AD20*Inputs!$B$38+AE20*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y20" s="5">
@@ -4406,7 +4464,7 @@
         <v/>
       </c>
       <c r="AA20" s="7">
-        <f>AC20*Inputs!$C$47+AD20*Inputs!$B$36+AE20*Inputs!$B$37</f>
+        <f>AC20*Inputs!$C$49+AD20*Inputs!$B$38+AE20*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB20" t="inlineStr">
@@ -4434,11 +4492,11 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>Inputs!$B$28*Inputs!$B$2</f>
+        <f>Inputs!$B$30*Inputs!$B$2</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>Inputs!$C$28*Inputs!$C$2</f>
+        <f>Inputs!$C$30*Inputs!$C$2</f>
         <v/>
       </c>
       <c r="D21" s="5">
@@ -4453,14 +4511,14 @@
         <v>0</v>
       </c>
       <c r="G21" s="6">
-        <f>Inputs!$B$29</f>
+        <f>Inputs!$B$31</f>
         <v/>
       </c>
       <c r="H21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="6">
-        <f>Inputs!$B$30</f>
+        <f>Inputs!$B$32</f>
         <v/>
       </c>
       <c r="J21" s="5">
@@ -4472,16 +4530,16 @@
         <v/>
       </c>
       <c r="L21" s="5">
-        <f>J21*Inputs!$B$42</f>
+        <f>J21*Inputs!$B$44</f>
         <v/>
       </c>
       <c r="M21" s="5">
-        <f>K21*Inputs!$C$42</f>
+        <f>K21*Inputs!$C$44</f>
         <v/>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Rack cabinets soon (18% of IT mass), server enclosures long term (22%), estimates; electronics never. Rack masses [H]; aggregate [L]</t>
+          <t>Rack cabinets soon (18% of IT mass), server enclosures long term (30%), per analyses/it-rack-material-stack.md; electronics never. Rack masses [H]; aggregate [L]</t>
         </is>
       </c>
       <c r="O21" s="5">
@@ -4521,7 +4579,7 @@
         <v/>
       </c>
       <c r="X21" s="7">
-        <f>AC21*Inputs!$B$46+AD21*Inputs!$B$36+AE21*Inputs!$B$37</f>
+        <f>AC21*Inputs!$B$48+AD21*Inputs!$B$38+AE21*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y21" s="5">
@@ -4533,7 +4591,7 @@
         <v/>
       </c>
       <c r="AA21" s="7">
-        <f>AC21*Inputs!$C$47+AD21*Inputs!$B$36+AE21*Inputs!$B$37</f>
+        <f>AC21*Inputs!$C$49+AD21*Inputs!$B$38+AE21*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB21" t="inlineStr">
@@ -4542,16 +4600,16 @@
         </is>
       </c>
       <c r="AC21" s="2" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AD21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AE21" s="2" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="AF21" s="2" t="n">
-        <v>0.5</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="23">
@@ -5140,11 +5198,11 @@
         </is>
       </c>
       <c r="B6" s="15">
-        <f>Inputs!$B$38/1000*Inputs!$B$39*0.092903</f>
+        <f>Inputs!$B$40/1000*Inputs!$B$41*0.092903</f>
         <v/>
       </c>
       <c r="C6" s="15">
-        <f>Inputs!$C$38/1000*Inputs!$C$39*0.092903</f>
+        <f>Inputs!$C$40/1000*Inputs!$C$41*0.092903</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -5160,11 +5218,11 @@
         </is>
       </c>
       <c r="B7" s="15">
-        <f>Inputs!$B$40*B6/1000</f>
+        <f>Inputs!$B$42*B6/1000</f>
         <v/>
       </c>
       <c r="C7" s="15">
-        <f>Inputs!$C$40*C6/1000</f>
+        <f>Inputs!$C$42*C6/1000</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -5180,11 +5238,11 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>Inputs!$B$41*B6/1000</f>
+        <f>Inputs!$B$43*B6/1000</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>Inputs!$C$41*C6/1000</f>
+        <f>Inputs!$C$43*C6/1000</f>
         <v/>
       </c>
       <c r="D8" t="inlineStr">
@@ -5292,11 +5350,11 @@
         <v/>
       </c>
       <c r="D2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$48</f>
+        <f>'1 GW data center'!B29*Inputs!$B$50</f>
         <v/>
       </c>
       <c r="E2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$48</f>
+        <f>'1 GW data center'!C29*Inputs!$C$50</f>
         <v/>
       </c>
       <c r="F2" s="4">
@@ -5316,11 +5374,11 @@
         <v/>
       </c>
       <c r="J2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$49</f>
+        <f>'1 GW data center'!B29*Inputs!$B$51</f>
         <v/>
       </c>
       <c r="K2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$49</f>
+        <f>'1 GW data center'!C29*Inputs!$C$51</f>
         <v/>
       </c>
     </row>
@@ -5339,11 +5397,11 @@
         <v/>
       </c>
       <c r="D3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$48</f>
+        <f>'1 GW data center'!B34*Inputs!$B$50</f>
         <v/>
       </c>
       <c r="E3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$48</f>
+        <f>'1 GW data center'!C34*Inputs!$C$50</f>
         <v/>
       </c>
       <c r="F3" s="4">
@@ -5363,11 +5421,11 @@
         <v/>
       </c>
       <c r="J3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$49</f>
+        <f>'1 GW data center'!B34*Inputs!$B$51</f>
         <v/>
       </c>
       <c r="K3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$49</f>
+        <f>'1 GW data center'!C34*Inputs!$C$51</f>
         <v/>
       </c>
     </row>
@@ -5386,11 +5444,11 @@
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$48</f>
+        <f>'1 GW data center'!B38*Inputs!$B$50</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$48</f>
+        <f>'1 GW data center'!C38*Inputs!$C$50</f>
         <v/>
       </c>
       <c r="F4" s="4">
@@ -5410,11 +5468,11 @@
         <v/>
       </c>
       <c r="J4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$49</f>
+        <f>'1 GW data center'!B38*Inputs!$B$51</f>
         <v/>
       </c>
       <c r="K4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$49</f>
+        <f>'1 GW data center'!C38*Inputs!$C$51</f>
         <v/>
       </c>
     </row>
@@ -5433,11 +5491,11 @@
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$48</f>
+        <f>'1 GW data center'!B42*Inputs!$B$50</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$48</f>
+        <f>'1 GW data center'!C42*Inputs!$C$50</f>
         <v/>
       </c>
       <c r="F5" s="4">
@@ -5457,11 +5515,11 @@
         <v/>
       </c>
       <c r="J5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$49</f>
+        <f>'1 GW data center'!B42*Inputs!$B$51</f>
         <v/>
       </c>
       <c r="K5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$49</f>
+        <f>'1 GW data center'!C42*Inputs!$C$51</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Analyses: Foundations scenario sheet with soil cases and a concrete-basis switch
Footprint-based concrete (slab, thickened zones, footings, grade beams,
generator, transformer and mechanical pads, site paving, yard mats) with
good / moderate / poor soil allowances and a switch between the
published per-MW intensity and the footprint bottom-up. Wall system
stays on walls_precast. Deck figures unchanged (per-MW basis) pending
Alex's choice of scenario.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 GW data center" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carbon" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steel share" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foundations" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carbon" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steel share" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -701,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1963,130 +1964,890 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Steel emissions, global average (BF-BOF)</t>
+          <t>Concrete basis: 0 = published per-MW intensity, 1 = footprint bottom-up (Foundations sheet)</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>published-class [M]</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Scenario switch, added 2026-09-06; the deck prints the per-MW basis until Alex decides</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Steel emissions, recycled (EAF)</t>
+          <t>Soil case for the footprint basis: 1 good (spread footings), 2 moderate (lean concrete, larger footings), 3 poor (piles, pile caps, structural slab)</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>industry range [M]</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Geotechnical allowance, Foundations sheet</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SUPERWOOD manufacturing emissions</t>
+          <t>Hall slab on grade thickness</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>0.5</v>
+        <v>8</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>in</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
-        </is>
-      </c>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SUPERWOOD biogenic carbon stored</t>
+          <t>Share of hall floor thickened (electrical rooms, dense rack rows)</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>1.3</v>
+        <v>0.15</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>1.3</v>
+        <v>0.25</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>kg CO₂e/kg</t>
+          <t>share</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>internal, pre-LCA [L]</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Report separately; module C release under EN 15804</t>
-        </is>
-      </c>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Thickened slab thickness</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Column bay</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Square bays</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Spread footing plan dimension</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Square footings</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Spread footing depth</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Perimeter grade beam width</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Perimeter grade beam depth</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Generator unit size</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Smaller units in the high case mean more pads</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Generator redundancy factor</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>factor</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>N+1 to N+25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Generator pad volume</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>787.5</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>cf</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>40x12x1 ft to 45x14x1.25 ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Transformer / switchgear pads per generator</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Transformer / switchgear pad volume</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>562.5</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>cf</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>20x15x1 ft to 25x18x1.25 ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Mechanical equipment pads as a share of floor area</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Chillers, coolers, fan walls on grade or roof</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Mechanical pad thickness</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Site paving, roads, yards, parking as a multiple of building footprint</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Site paving thickness</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Case 2: share of footprint over-excavated and replaced with lean concrete / CLSM</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Case 2: lean concrete thickness</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Case 2: enlargement of footings, grade beams and pads</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>factor</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Case 3: piles or drilled piers per column</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Case 3: pile diameter</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Case 3: pile length</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Case 3: pile cap volume per column (replaces the spread footing)</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>cf</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>10x10x3 ft to 12x12x3.5 ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Case 3: pier spacing under grade beams</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Case 3: slab thickening to a structural slab</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Substation / transformer yard mats per GW</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>acres</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Yard mat thickness</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>estimated [L]</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Steel emissions, global average (BF-BOF)</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>published-class [M]</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Steel emissions, recycled (EAF)</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>industry range [M]</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SUPERWOOD manufacturing emissions</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>internal, pre-LCA [L]</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Canva DCII deck; LCA under way, Prof. Ming Hu, Notre Dame</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>SUPERWOOD biogenic carbon stored</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>kg CO₂e/kg</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>internal, pre-LCA [L]</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Report separately; module C release under EN 15804</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
           <t>Interior finishes emissions (gypsum, wood, steel studs — mixed)</t>
         </is>
       </c>
-      <c r="B52" s="2" t="n">
+      <c r="B82" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C52" s="2" t="n">
+      <c r="C82" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>kg CO₂e/kg</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>estimated [L]</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>Used only for the interior finishes row</t>
         </is>
@@ -2333,11 +3094,11 @@
         </is>
       </c>
       <c r="B3" s="5">
-        <f>Inputs!$B$11*(1-Inputs!$B$33)*Inputs!$B$12*Inputs!$B$2-B5</f>
+        <f>IF(Inputs!$B$48=1,Foundations!B28,Inputs!$B$11*(1-Inputs!$B$33)*Inputs!$B$12*Inputs!$B$2)-B5</f>
         <v/>
       </c>
       <c r="C3" s="5">
-        <f>Inputs!$C$11*(1-Inputs!$C$33)*Inputs!$C$12*Inputs!$C$2-C5</f>
+        <f>IF(Inputs!$C$48=1,Foundations!C28,Inputs!$C$11*(1-Inputs!$C$33)*Inputs!$C$12*Inputs!$C$2)-C5</f>
         <v/>
       </c>
       <c r="D3" s="5">
@@ -2419,7 +3180,7 @@
         <v/>
       </c>
       <c r="X3" s="7">
-        <f>AC3*Inputs!$B$48+AD3*Inputs!$B$38+AE3*Inputs!$B$39</f>
+        <f>AC3*Inputs!$B$78+AD3*Inputs!$B$38+AE3*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y3" s="5">
@@ -2431,7 +3192,7 @@
         <v/>
       </c>
       <c r="AA3" s="7">
-        <f>AC3*Inputs!$C$49+AD3*Inputs!$B$38+AE3*Inputs!$B$39</f>
+        <f>AC3*Inputs!$C$79+AD3*Inputs!$B$38+AE3*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB3" t="inlineStr">
@@ -2459,11 +3220,11 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>Inputs!$B$11*Inputs!$B$33*Inputs!$B$12*Inputs!$B$2</f>
+        <f>IF(Inputs!$B$48=1,Foundations!B29,Inputs!$B$11*Inputs!$B$33*Inputs!$B$12*Inputs!$B$2)</f>
         <v/>
       </c>
       <c r="C4" s="5">
-        <f>Inputs!$C$11*Inputs!$C$33*Inputs!$C$12*Inputs!$C$2</f>
+        <f>IF(Inputs!$C$48=1,Foundations!C29,Inputs!$C$11*Inputs!$C$33*Inputs!$C$12*Inputs!$C$2)</f>
         <v/>
       </c>
       <c r="D4" s="5">
@@ -2545,7 +3306,7 @@
         <v/>
       </c>
       <c r="X4" s="7">
-        <f>AC4*Inputs!$B$48+AD4*Inputs!$B$38+AE4*Inputs!$B$39</f>
+        <f>AC4*Inputs!$B$78+AD4*Inputs!$B$38+AE4*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y4" s="5">
@@ -2557,7 +3318,7 @@
         <v/>
       </c>
       <c r="AA4" s="7">
-        <f>AC4*Inputs!$C$49+AD4*Inputs!$B$38+AE4*Inputs!$B$39</f>
+        <f>AC4*Inputs!$C$79+AD4*Inputs!$B$38+AE4*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB4" t="inlineStr">
@@ -2670,7 +3431,7 @@
         <v/>
       </c>
       <c r="X5" s="7">
-        <f>AC5*Inputs!$B$48+AD5*Inputs!$B$38+AE5*Inputs!$B$39</f>
+        <f>AC5*Inputs!$B$78+AD5*Inputs!$B$38+AE5*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y5" s="5">
@@ -2682,7 +3443,7 @@
         <v/>
       </c>
       <c r="AA5" s="7">
-        <f>AC5*Inputs!$C$49+AD5*Inputs!$B$38+AE5*Inputs!$B$39</f>
+        <f>AC5*Inputs!$C$79+AD5*Inputs!$B$38+AE5*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB5" t="inlineStr">
@@ -2710,11 +3471,11 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>Inputs!$B$11*Inputs!$B$17/1000*Inputs!$B$2</f>
+        <f>IF(Inputs!$B$48=1,Foundations!B26+Foundations!B27,Inputs!$B$11*Inputs!$B$2)*Inputs!$B$17/1000</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>Inputs!$C$11*Inputs!$C$17/1000*Inputs!$C$2</f>
+        <f>IF(Inputs!$C$48=1,Foundations!C26+Foundations!C27,Inputs!$C$11*Inputs!$C$2)*Inputs!$C$17/1000</f>
         <v/>
       </c>
       <c r="D6" s="5">
@@ -2796,7 +3557,7 @@
         <v/>
       </c>
       <c r="X6" s="7">
-        <f>AC6*Inputs!$B$48+AD6*Inputs!$B$38+AE6*Inputs!$B$39</f>
+        <f>AC6*Inputs!$B$78+AD6*Inputs!$B$38+AE6*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y6" s="5">
@@ -2808,7 +3569,7 @@
         <v/>
       </c>
       <c r="AA6" s="7">
-        <f>AC6*Inputs!$C$49+AD6*Inputs!$B$38+AE6*Inputs!$B$39</f>
+        <f>AC6*Inputs!$C$79+AD6*Inputs!$B$38+AE6*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB6" t="inlineStr">
@@ -2921,7 +3682,7 @@
         <v/>
       </c>
       <c r="X7" s="7">
-        <f>AC7*Inputs!$B$48+AD7*Inputs!$B$38+AE7*Inputs!$B$39</f>
+        <f>AC7*Inputs!$B$78+AD7*Inputs!$B$38+AE7*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y7" s="5">
@@ -2933,7 +3694,7 @@
         <v/>
       </c>
       <c r="AA7" s="7">
-        <f>AC7*Inputs!$C$49+AD7*Inputs!$B$38+AE7*Inputs!$B$39</f>
+        <f>AC7*Inputs!$C$79+AD7*Inputs!$B$38+AE7*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB7" t="inlineStr">
@@ -3046,7 +3807,7 @@
         <v/>
       </c>
       <c r="X8" s="7">
-        <f>AC8*Inputs!$B$48+AD8*Inputs!$B$38+AE8*Inputs!$B$39</f>
+        <f>AC8*Inputs!$B$78+AD8*Inputs!$B$38+AE8*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y8" s="5">
@@ -3058,7 +3819,7 @@
         <v/>
       </c>
       <c r="AA8" s="7">
-        <f>AC8*Inputs!$C$49+AD8*Inputs!$B$38+AE8*Inputs!$B$39</f>
+        <f>AC8*Inputs!$C$79+AD8*Inputs!$B$38+AE8*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB8" t="inlineStr">
@@ -3171,7 +3932,7 @@
         <v/>
       </c>
       <c r="X9" s="7">
-        <f>AC9*Inputs!$B$48+AD9*Inputs!$B$38+AE9*Inputs!$B$39</f>
+        <f>AC9*Inputs!$B$78+AD9*Inputs!$B$38+AE9*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y9" s="5">
@@ -3183,7 +3944,7 @@
         <v/>
       </c>
       <c r="AA9" s="7">
-        <f>AC9*Inputs!$C$49+AD9*Inputs!$B$38+AE9*Inputs!$B$39</f>
+        <f>AC9*Inputs!$C$79+AD9*Inputs!$B$38+AE9*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB9" t="inlineStr">
@@ -3296,7 +4057,7 @@
         <v/>
       </c>
       <c r="X10" s="7">
-        <f>AC10*Inputs!$B$48+AD10*Inputs!$B$38+AE10*Inputs!$B$39</f>
+        <f>AC10*Inputs!$B$78+AD10*Inputs!$B$38+AE10*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y10" s="5">
@@ -3308,7 +4069,7 @@
         <v/>
       </c>
       <c r="AA10" s="7">
-        <f>AC10*Inputs!$C$49+AD10*Inputs!$B$38+AE10*Inputs!$B$39</f>
+        <f>AC10*Inputs!$C$79+AD10*Inputs!$B$38+AE10*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB10" t="inlineStr">
@@ -3421,7 +4182,7 @@
         <v/>
       </c>
       <c r="X11" s="7">
-        <f>AC11*Inputs!$B$48+AD11*Inputs!$B$38+AE11*Inputs!$B$39</f>
+        <f>AC11*Inputs!$B$78+AD11*Inputs!$B$38+AE11*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y11" s="5">
@@ -3433,7 +4194,7 @@
         <v/>
       </c>
       <c r="AA11" s="7">
-        <f>AC11*Inputs!$C$49+AD11*Inputs!$B$38+AE11*Inputs!$B$39</f>
+        <f>AC11*Inputs!$C$79+AD11*Inputs!$B$38+AE11*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB11" t="inlineStr">
@@ -3574,7 +4335,7 @@
         <v/>
       </c>
       <c r="X13" s="7">
-        <f>AC13*Inputs!$B$48+AD13*Inputs!$B$38+AE13*Inputs!$B$39</f>
+        <f>AC13*Inputs!$B$78+AD13*Inputs!$B$38+AE13*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y13" s="5">
@@ -3586,7 +4347,7 @@
         <v/>
       </c>
       <c r="AA13" s="7">
-        <f>AC13*Inputs!$C$49+AD13*Inputs!$B$38+AE13*Inputs!$B$39</f>
+        <f>AC13*Inputs!$C$79+AD13*Inputs!$B$38+AE13*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB13" t="inlineStr">
@@ -3699,7 +4460,7 @@
         <v/>
       </c>
       <c r="X14" s="7">
-        <f>AC14*Inputs!$B$48+AD14*Inputs!$B$38+AE14*Inputs!$B$39</f>
+        <f>AC14*Inputs!$B$78+AD14*Inputs!$B$38+AE14*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y14" s="5">
@@ -3711,7 +4472,7 @@
         <v/>
       </c>
       <c r="AA14" s="7">
-        <f>AC14*Inputs!$C$49+AD14*Inputs!$B$38+AE14*Inputs!$B$39</f>
+        <f>AC14*Inputs!$C$79+AD14*Inputs!$B$38+AE14*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB14" t="inlineStr">
@@ -3824,7 +4585,7 @@
         <v/>
       </c>
       <c r="X15" s="7">
-        <f>AC15*Inputs!$B$48+AD15*Inputs!$B$38+AE15*Inputs!$B$39</f>
+        <f>AC15*Inputs!$B$78+AD15*Inputs!$B$38+AE15*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y15" s="5">
@@ -3836,7 +4597,7 @@
         <v/>
       </c>
       <c r="AA15" s="7">
-        <f>AC15*Inputs!$C$49+AD15*Inputs!$B$38+AE15*Inputs!$B$39</f>
+        <f>AC15*Inputs!$C$79+AD15*Inputs!$B$38+AE15*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB15" t="inlineStr">
@@ -3950,7 +4711,7 @@
         <v/>
       </c>
       <c r="X16" s="7">
-        <f>AC16*Inputs!$B$48+AD16*Inputs!$B$38+AE16*Inputs!$B$39</f>
+        <f>AC16*Inputs!$B$78+AD16*Inputs!$B$38+AE16*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y16" s="5">
@@ -3962,7 +4723,7 @@
         <v/>
       </c>
       <c r="AA16" s="7">
-        <f>AC16*Inputs!$C$49+AD16*Inputs!$B$38+AE16*Inputs!$B$39</f>
+        <f>AC16*Inputs!$C$79+AD16*Inputs!$B$38+AE16*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB16" t="inlineStr">
@@ -4075,7 +4836,7 @@
         <v/>
       </c>
       <c r="X17" s="7">
-        <f>AC17*Inputs!$B$48+AD17*Inputs!$B$38+AE17*Inputs!$B$39</f>
+        <f>AC17*Inputs!$B$78+AD17*Inputs!$B$38+AE17*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y17" s="5">
@@ -4087,7 +4848,7 @@
         <v/>
       </c>
       <c r="AA17" s="7">
-        <f>AC17*Inputs!$C$49+AD17*Inputs!$B$38+AE17*Inputs!$B$39</f>
+        <f>AC17*Inputs!$C$79+AD17*Inputs!$B$38+AE17*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB17" t="inlineStr">
@@ -4200,7 +4961,7 @@
         <v/>
       </c>
       <c r="X18" s="7">
-        <f>AC18*Inputs!$B$48+AD18*Inputs!$B$38+AE18*Inputs!$B$39</f>
+        <f>AC18*Inputs!$B$78+AD18*Inputs!$B$38+AE18*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y18" s="5">
@@ -4212,7 +4973,7 @@
         <v/>
       </c>
       <c r="AA18" s="7">
-        <f>AC18*Inputs!$C$49+AD18*Inputs!$B$38+AE18*Inputs!$B$39</f>
+        <f>AC18*Inputs!$C$79+AD18*Inputs!$B$38+AE18*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB18" t="inlineStr">
@@ -4325,7 +5086,7 @@
         <v/>
       </c>
       <c r="X19" s="7">
-        <f>AC19*Inputs!$B$48+AD19*Inputs!$B$38+AE19*Inputs!$B$39</f>
+        <f>AC19*Inputs!$B$78+AD19*Inputs!$B$38+AE19*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y19" s="5">
@@ -4337,7 +5098,7 @@
         <v/>
       </c>
       <c r="AA19" s="7">
-        <f>AC19*Inputs!$C$49+AD19*Inputs!$B$38+AE19*Inputs!$B$39</f>
+        <f>AC19*Inputs!$C$79+AD19*Inputs!$B$38+AE19*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB19" t="inlineStr">
@@ -4452,7 +5213,7 @@
         <v/>
       </c>
       <c r="X20" s="7">
-        <f>AC20*Inputs!$B$48+AD20*Inputs!$B$38+AE20*Inputs!$B$39</f>
+        <f>AC20*Inputs!$B$78+AD20*Inputs!$B$38+AE20*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y20" s="5">
@@ -4464,7 +5225,7 @@
         <v/>
       </c>
       <c r="AA20" s="7">
-        <f>AC20*Inputs!$C$49+AD20*Inputs!$B$38+AE20*Inputs!$B$39</f>
+        <f>AC20*Inputs!$C$79+AD20*Inputs!$B$38+AE20*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB20" t="inlineStr">
@@ -4579,7 +5340,7 @@
         <v/>
       </c>
       <c r="X21" s="7">
-        <f>AC21*Inputs!$B$48+AD21*Inputs!$B$38+AE21*Inputs!$B$39</f>
+        <f>AC21*Inputs!$B$78+AD21*Inputs!$B$38+AE21*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="Y21" s="5">
@@ -4591,7 +5352,7 @@
         <v/>
       </c>
       <c r="AA21" s="7">
-        <f>AC21*Inputs!$C$49+AD21*Inputs!$B$38+AE21*Inputs!$B$39</f>
+        <f>AC21*Inputs!$C$79+AD21*Inputs!$B$38+AE21*Inputs!$B$39</f>
         <v/>
       </c>
       <c r="AB21" t="inlineStr">
@@ -5262,6 +6023,579 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Low  m³</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>High  m³</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Building floor area, sf</t>
+        </is>
+      </c>
+      <c r="B2" s="5">
+        <f>Inputs!$B$3*Inputs!$B$2</f>
+        <v/>
+      </c>
+      <c r="C2" s="5">
+        <f>Inputs!$C$3*Inputs!$C$2</f>
+        <v/>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>from Inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total hall perimeter, ft</t>
+        </is>
+      </c>
+      <c r="B3" s="5">
+        <f>Derived!B2*4*SQRT(Inputs!$B$4)</f>
+        <v/>
+      </c>
+      <c r="C3" s="5">
+        <f>Derived!C2*4*SQRT(Inputs!$C$4)</f>
+        <v/>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>buildings x 4 sides</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Columns</t>
+        </is>
+      </c>
+      <c r="B4" s="5">
+        <f>B2/(Inputs!$B$53^2)</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>C2/(Inputs!$C$53^2)</f>
+        <v/>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>one per bay</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hall slab on grade</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>B2*Inputs!$B$50/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>C2*Inputs!$C$50/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>6–8 in over the floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Thickened slab zones</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>B2*Inputs!$B$51*(Inputs!$B$52-Inputs!$B$50)/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>C2*Inputs!$C$51*(Inputs!$C$52-Inputs!$C$50)/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>extra depth over 15–25% of the floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Column footings</t>
+        </is>
+      </c>
+      <c r="B7" s="5">
+        <f>B4*Inputs!$B$54^2*Inputs!$B$55*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>C4*Inputs!$C$54^2*Inputs!$C$55*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>spread footings, good soils</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Perimeter grade beams</t>
+        </is>
+      </c>
+      <c r="B8" s="5">
+        <f>B3*Inputs!$B$56*Inputs!$B$57*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>C3*Inputs!$C$56*Inputs!$C$57*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Generators</t>
+        </is>
+      </c>
+      <c r="B9" s="5">
+        <f>Inputs!$B$2/Inputs!$B$58*Inputs!$B$59</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>Inputs!$C$2/Inputs!$C$58*Inputs!$C$59</f>
+        <v/>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>units incl. redundancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Generator pads</t>
+        </is>
+      </c>
+      <c r="B10" s="5">
+        <f>B9*Inputs!$B$60*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>C9*Inputs!$C$60*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Transformer and switchgear pads</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>B9*Inputs!$B$61*Inputs!$B$62*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>C9*Inputs!$C$61*Inputs!$C$62*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mechanical equipment pads</t>
+        </is>
+      </c>
+      <c r="B12" s="5">
+        <f>B2*Inputs!$B$63*Inputs!$B$64/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C12" s="5">
+        <f>C2*Inputs!$C$63*Inputs!$C$64/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Case 1 good soils — building and pads</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>B5+B6+B7+B8+B10+B11+B12</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>C5+C6+C7+C8+C10+C11+C12</f>
+        <v/>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Case 2 — lean concrete / CLSM under footprint</t>
+        </is>
+      </c>
+      <c r="B14" s="5">
+        <f>B2*Inputs!$B$67*Inputs!$B$68/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C14" s="5">
+        <f>C2*Inputs!$C$67*Inputs!$C$68/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Case 2 — larger footings, grade beams and pads</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>(B7+B8+B10+B11+B12)*Inputs!$B$69</f>
+        <v/>
+      </c>
+      <c r="C15" s="5">
+        <f>(C7+C8+C10+C11+C12)*Inputs!$C$69</f>
+        <v/>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Case 2 moderate soils — allowance</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>B14+B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="5">
+        <f>C14+C15</f>
+        <v/>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>added to case 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Case 3 — piles or drilled piers under columns</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>B4*Inputs!$B$70*PI()*(Inputs!$B$71/2)^2*Inputs!$B$72*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C17" s="5">
+        <f>C4*Inputs!$C$70*PI()*(Inputs!$C$71/2)^2*Inputs!$C$72*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Case 3 — pile caps net of spread footings</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>B4*Inputs!$B$73*0.0283168-B7</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f>C4*Inputs!$C$73*0.0283168-C7</f>
+        <v/>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Case 3 — piers under grade beams</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>B3/Inputs!$B$74*PI()*(Inputs!$B$71/2)^2*Inputs!$B$72*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C19" s="5">
+        <f>C3/Inputs!$C$74*PI()*(Inputs!$C$71/2)^2*Inputs!$C$72*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Case 3 — structural slab thickening</t>
+        </is>
+      </c>
+      <c r="B20" s="5">
+        <f>B2*Inputs!$B$75/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C20" s="5">
+        <f>C2*Inputs!$C$75/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Case 3 poor soils — allowance</t>
+        </is>
+      </c>
+      <c r="B21" s="5">
+        <f>B17+B18+B19+B20</f>
+        <v/>
+      </c>
+      <c r="C21" s="5">
+        <f>C17+C18+C19+C20</f>
+        <v/>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>added to case 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Selected soil allowance</t>
+        </is>
+      </c>
+      <c r="B22" s="5">
+        <f>CHOOSE(Inputs!$B$49,0,B16,B21)</f>
+        <v/>
+      </c>
+      <c r="C22" s="5">
+        <f>CHOOSE(Inputs!$C$49,0,C16,C21)</f>
+        <v/>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Inputs soil_case</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Site paving, roads, yards, parking</t>
+        </is>
+      </c>
+      <c r="B23" s="5">
+        <f>B2*Inputs!$B$65*Inputs!$B$66/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C23" s="5">
+        <f>C2*Inputs!$C$65*Inputs!$C$66/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Substation / transformer yard mats</t>
+        </is>
+      </c>
+      <c r="B24" s="5">
+        <f>Inputs!$B$76*Inputs!$B$2/1000*43560*Inputs!$B$77/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="C24" s="5">
+        <f>Inputs!$C$76*Inputs!$C$2/1000*43560*Inputs!$C$77/12*0.0283168</f>
+        <v/>
+      </c>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>All-in with site work, selected soil case</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>B13+B22+B23+B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="5">
+        <f>C13+C22+C23+C24</f>
+        <v/>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Slab and paving, footprint basis (m³)</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>B5+B6+B23+IF(Inputs!$B$49=3,B20,0)</f>
+        <v/>
+      </c>
+      <c r="C26" s="5">
+        <f>C5+C6+C23+IF(Inputs!$C$49=3,C20,0)</f>
+        <v/>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>feeds the main sheet when concrete_basis = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Foundations, footings and pads, footprint basis (m³)</t>
+        </is>
+      </c>
+      <c r="B27" s="5">
+        <f>B7+B8+B10+B11+B12+B24+IF(Inputs!$B$49=2,B16,IF(Inputs!$B$49=3,B17+B18+B19,0))</f>
+        <v/>
+      </c>
+      <c r="C27" s="5">
+        <f>C7+C8+C10+C11+C12+C24+IF(Inputs!$C$49=2,C16,IF(Inputs!$C$49=3,C17+C18+C19,0))</f>
+        <v/>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>feeds the main sheet when concrete_basis = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Slab and paving, footprint basis (t)</t>
+        </is>
+      </c>
+      <c r="B28" s="5">
+        <f>B26*Inputs!$B$12</f>
+        <v/>
+      </c>
+      <c r="C28" s="5">
+        <f>C26*Inputs!$C$12</f>
+        <v/>
+      </c>
+      <c r="D28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Foundations, footings and pads, footprint basis (t)</t>
+        </is>
+      </c>
+      <c r="B29" s="5">
+        <f>B27*Inputs!$B$12</f>
+        <v/>
+      </c>
+      <c r="C29" s="5">
+        <f>C27*Inputs!$C$12</f>
+        <v/>
+      </c>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Per-MW basis for comparison (m³)</t>
+        </is>
+      </c>
+      <c r="B30" s="5">
+        <f>Inputs!$B$11*Inputs!$B$2</f>
+        <v/>
+      </c>
+      <c r="C30" s="5">
+        <f>Inputs!$C$11*Inputs!$C$2</f>
+        <v/>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>published, secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Wall system: tilt-up versus insulated metal panel is the Inputs walls_precast switch (precast row on the main sheet, steel-share sheet reports both). Soil cases and the concrete basis switch are Inputs soil_case and concrete_basis. All element inputs are estimates [L]; see foundation-bottom-up.md.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5350,11 +6684,11 @@
         <v/>
       </c>
       <c r="D2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$50</f>
+        <f>'1 GW data center'!B29*Inputs!$B$80</f>
         <v/>
       </c>
       <c r="E2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$50</f>
+        <f>'1 GW data center'!C29*Inputs!$C$80</f>
         <v/>
       </c>
       <c r="F2" s="4">
@@ -5374,11 +6708,11 @@
         <v/>
       </c>
       <c r="J2" s="4">
-        <f>'1 GW data center'!B29*Inputs!$B$51</f>
+        <f>'1 GW data center'!B29*Inputs!$B$81</f>
         <v/>
       </c>
       <c r="K2" s="4">
-        <f>'1 GW data center'!C29*Inputs!$C$51</f>
+        <f>'1 GW data center'!C29*Inputs!$C$81</f>
         <v/>
       </c>
     </row>
@@ -5397,11 +6731,11 @@
         <v/>
       </c>
       <c r="D3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$50</f>
+        <f>'1 GW data center'!B34*Inputs!$B$80</f>
         <v/>
       </c>
       <c r="E3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$50</f>
+        <f>'1 GW data center'!C34*Inputs!$C$80</f>
         <v/>
       </c>
       <c r="F3" s="4">
@@ -5421,11 +6755,11 @@
         <v/>
       </c>
       <c r="J3" s="4">
-        <f>'1 GW data center'!B34*Inputs!$B$51</f>
+        <f>'1 GW data center'!B34*Inputs!$B$81</f>
         <v/>
       </c>
       <c r="K3" s="4">
-        <f>'1 GW data center'!C34*Inputs!$C$51</f>
+        <f>'1 GW data center'!C34*Inputs!$C$81</f>
         <v/>
       </c>
     </row>
@@ -5444,11 +6778,11 @@
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$50</f>
+        <f>'1 GW data center'!B38*Inputs!$B$80</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$50</f>
+        <f>'1 GW data center'!C38*Inputs!$C$80</f>
         <v/>
       </c>
       <c r="F4" s="4">
@@ -5468,11 +6802,11 @@
         <v/>
       </c>
       <c r="J4" s="4">
-        <f>'1 GW data center'!B38*Inputs!$B$51</f>
+        <f>'1 GW data center'!B38*Inputs!$B$81</f>
         <v/>
       </c>
       <c r="K4" s="4">
-        <f>'1 GW data center'!C38*Inputs!$C$51</f>
+        <f>'1 GW data center'!C38*Inputs!$C$81</f>
         <v/>
       </c>
     </row>
@@ -5491,11 +6825,11 @@
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$50</f>
+        <f>'1 GW data center'!B42*Inputs!$B$80</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$50</f>
+        <f>'1 GW data center'!C42*Inputs!$C$80</f>
         <v/>
       </c>
       <c r="F5" s="4">
@@ -5515,11 +6849,11 @@
         <v/>
       </c>
       <c r="J5" s="4">
-        <f>'1 GW data center'!B42*Inputs!$B$51</f>
+        <f>'1 GW data center'!B42*Inputs!$B$81</f>
         <v/>
       </c>
       <c r="K5" s="4">
-        <f>'1 GW data center'!C42*Inputs!$C$51</f>
+        <f>'1 GW data center'!C42*Inputs!$C$81</f>
         <v/>
       </c>
     </row>
@@ -5535,7 +6869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
DC investor deck: footprint concrete basis with moderate soils by default and a soils slider
Alex 2026-09-06. Workbook defaults to the footprint bottom-up with
moderate soils; analyses/export_scenarios.py evaluates good, moderate
and poor soils into scenarios.json. Slides 6 and 7 carry a soils slider
(keys G / O / P) that swaps the concrete rows, the foundation subtotal
and the long-term SUPERWOOD row; PPTX charts and Worth row print
moderate soils. Footer: wordmark at the right edge of the window.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -1968,10 +1968,10 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Scenario switch, added 2026-09-06; the deck prints the per-MW basis until Alex decides</t>
+          <t>Deck default since 2026-09-06 (Alex): footprint basis</t>
         </is>
       </c>
     </row>
@@ -1996,10 +1996,10 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Geotechnical allowance, Foundations sheet</t>
+          <t>Deck default since 2026-09-06 (Alex): moderate soils; the web deck has a soils slider</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DC investor deck: nested soil cases, compact soils row, short group labels with hover detail, Requirement nav label
Poor soils now include the moderate-soils measures so foundation
concrete rises monotonically. Slide 6 groups read Contents, Building,
Foundation in larger type with the full description on hover or focus.
Slide 7 dock label is "Requirement".

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
+++ b/superwood-datacenter-investor/analyses/materials-mass-and-replacement.xlsx
@@ -6397,20 +6397,20 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Case 3 poor soils — allowance</t>
+          <t>Case 3 poor soils — allowance (includes the case 2 measures)</t>
         </is>
       </c>
       <c r="B21" s="5">
-        <f>B17+B18+B19+B20</f>
+        <f>B16+B17+B18+B19+B20</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>C17+C18+C19+C20</f>
+        <f>C16+C17+C18+C19+C20</f>
         <v/>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>added to case 1</t>
+          <t>nested: ground replacement and larger elements plus piles, caps, piers and a structural slab</t>
         </is>
       </c>
     </row>
@@ -6513,16 +6513,16 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>B7+B8+B10+B11+B12+B24+IF(Inputs!$B$49=2,B16,IF(Inputs!$B$49=3,B17+B18+B19,0))</f>
+        <f>B7+B8+B10+B11+B12+B24+IF(Inputs!$B$49&gt;=2,B16,0)+IF(Inputs!$B$49=3,B17+B18+B19,0)</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>C7+C8+C10+C11+C12+C24+IF(Inputs!$C$49=2,C16,IF(Inputs!$C$49=3,C17+C18+C19,0))</f>
+        <f>C7+C8+C10+C11+C12+C24+IF(Inputs!$C$49&gt;=2,C16,0)+IF(Inputs!$C$49=3,C17+C18+C19,0)</f>
         <v/>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>feeds the main sheet when concrete_basis = 1</t>
+          <t>feeds the main sheet when concrete_basis = 1; soil cases nest</t>
         </is>
       </c>
     </row>

</xml_diff>